<commit_message>
Add Base scenario alongside Reach in three-school projection (Current/Base/Reach)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;–&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,14 +53,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
-    <font/>
     <font>
       <i val="1"/>
       <color rgb="00404040"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +74,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -115,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -132,25 +136,25 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,37 +520,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J98"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Making Cinderella — Season 1 MBB Revenue: Current vs. With MC   (figures in $000s; estimates)</t>
+          <t>Making Cinderella — Season 1 MBB Revenue: Current / Base / Reach   (figures in $000s; estimates)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ST. JOSEPH'S  (Hagan 4,200 · A-10 · Philly)</t>
+          <t>ST. JOSEPH'S  (Hagan 4,200 · A-10)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>DAVIDSON  (Belk 5,223 · A-10 · Curry alma mater)</t>
+          <t>DAVIDSON  (Belk 5,223 · Curry alma mater)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -568,12 +572,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>With MC</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Δ</t>
+          <t>Reach</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -583,12 +587,12 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>With MC</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Δ</t>
+          <t>Reach</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -598,12 +602,12 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>With MC</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Δ</t>
+          <t>Reach</t>
         </is>
       </c>
     </row>
@@ -632,32 +636,29 @@
       <c r="B5" s="7" t="n">
         <v>700</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="8" t="n">
+        <v>1380</v>
+      </c>
+      <c r="D5" s="7" t="n">
         <v>1800</v>
-      </c>
-      <c r="D5" s="7">
-        <f>C5-B5</f>
-        <v/>
       </c>
       <c r="E5" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="8" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G5" s="7" t="n">
         <v>2200</v>
-      </c>
-      <c r="G5" s="7">
-        <f>F5-E5</f>
-        <v/>
       </c>
       <c r="H5" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="I5" s="8" t="n">
+        <v>2430</v>
+      </c>
+      <c r="J5" s="7" t="n">
         <v>3000</v>
-      </c>
-      <c r="J5" s="7">
-        <f>I5-H5</f>
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -669,32 +670,29 @@
       <c r="B6" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
+        <v>2320</v>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>3500</v>
-      </c>
-      <c r="D6" s="7">
-        <f>C6-B6</f>
-        <v/>
       </c>
       <c r="E6" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="8" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G6" s="7" t="n">
         <v>3500</v>
-      </c>
-      <c r="G6" s="7">
-        <f>F6-E6</f>
-        <v/>
       </c>
       <c r="H6" s="7" t="n">
         <v>700</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I6" s="8" t="n">
+        <v>1820</v>
+      </c>
+      <c r="J6" s="7" t="n">
         <v>2500</v>
-      </c>
-      <c r="J6" s="7">
-        <f>I6-H6</f>
-        <v/>
       </c>
     </row>
     <row r="7">
@@ -706,32 +704,29 @@
       <c r="B7" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="8" t="n">
+        <v>550</v>
+      </c>
+      <c r="D7" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="D7" s="7">
-        <f>C7-B7</f>
-        <v/>
       </c>
       <c r="E7" s="7" t="n">
         <v>250</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="8" t="n">
+        <v>720</v>
+      </c>
+      <c r="G7" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="G7" s="7">
-        <f>F7-E7</f>
-        <v/>
       </c>
       <c r="H7" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="I7" s="8" t="n">
+        <v>670</v>
+      </c>
+      <c r="J7" s="7" t="n">
         <v>900</v>
-      </c>
-      <c r="J7" s="7">
-        <f>I7-H7</f>
-        <v/>
       </c>
     </row>
     <row r="8">
@@ -743,32 +738,29 @@
       <c r="B8" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="D8" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="D8" s="7">
-        <f>C8-B8</f>
-        <v/>
       </c>
       <c r="E8" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="8" t="n">
+        <v>330</v>
+      </c>
+      <c r="G8" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="G8" s="7">
-        <f>F8-E8</f>
-        <v/>
       </c>
       <c r="H8" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="I8" s="8" t="n">
+        <v>230</v>
+      </c>
+      <c r="J8" s="7" t="n">
         <v>350</v>
-      </c>
-      <c r="J8" s="7">
-        <f>I8-H8</f>
-        <v/>
       </c>
     </row>
     <row r="9">
@@ -780,32 +772,29 @@
       <c r="B9" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="8" t="n">
+        <v>360</v>
+      </c>
+      <c r="D9" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="D9" s="7">
-        <f>C9-B9</f>
-        <v/>
       </c>
       <c r="E9" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="G9" s="7" t="n">
         <v>550</v>
-      </c>
-      <c r="G9" s="7">
-        <f>F9-E9</f>
-        <v/>
       </c>
       <c r="H9" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="I9" s="8" t="n">
+        <v>550</v>
+      </c>
+      <c r="J9" s="7" t="n">
         <v>700</v>
-      </c>
-      <c r="J9" s="7">
-        <f>I9-H9</f>
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -817,32 +806,29 @@
       <c r="B10" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="8" t="n">
+        <v>210</v>
+      </c>
+      <c r="D10" s="7" t="n">
         <v>300</v>
-      </c>
-      <c r="D10" s="7">
-        <f>C10-B10</f>
-        <v/>
       </c>
       <c r="E10" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="G10" s="7" t="n">
         <v>350</v>
-      </c>
-      <c r="G10" s="7">
-        <f>F10-E10</f>
-        <v/>
       </c>
       <c r="H10" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="I10" s="8" t="n">
+        <v>270</v>
+      </c>
+      <c r="J10" s="7" t="n">
         <v>350</v>
-      </c>
-      <c r="J10" s="7">
-        <f>I10-H10</f>
-        <v/>
       </c>
     </row>
     <row r="11">
@@ -854,73 +840,70 @@
       <c r="B11" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="8" t="n">
+        <v>340</v>
+      </c>
+      <c r="D11" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="D11" s="7">
-        <f>C11-B11</f>
-        <v/>
       </c>
       <c r="E11" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F11" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="G11" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="G11" s="7">
-        <f>F11-E11</f>
-        <v/>
       </c>
       <c r="H11" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="I11" s="8" t="n">
+        <v>370</v>
+      </c>
+      <c r="J11" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="J11" s="7">
-        <f>I11-H11</f>
-        <v/>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Ticketing &amp; game-day</t>
         </is>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="10">
         <f>SUM(B5:B11)</f>
         <v/>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <f>SUM(C5:C11)</f>
         <v/>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="10">
         <f>SUM(D5:D11)</f>
         <v/>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="10">
         <f>SUM(E5:E11)</f>
         <v/>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="10">
         <f>SUM(F5:F11)</f>
         <v/>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="10">
         <f>SUM(G5:G11)</f>
         <v/>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="10">
         <f>SUM(H5:H11)</f>
         <v/>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="10">
         <f>SUM(I5:I11)</f>
         <v/>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="10">
         <f>SUM(J5:J11)</f>
         <v/>
       </c>
@@ -950,32 +933,29 @@
       <c r="B15" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="8" t="n">
+        <v>530</v>
+      </c>
+      <c r="D15" s="7" t="n">
         <v>550</v>
-      </c>
-      <c r="D15" s="7">
-        <f>C15-B15</f>
-        <v/>
       </c>
       <c r="E15" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F15" s="8" t="n">
+        <v>530</v>
+      </c>
+      <c r="G15" s="7" t="n">
         <v>550</v>
-      </c>
-      <c r="G15" s="7">
-        <f>F15-E15</f>
-        <v/>
       </c>
       <c r="H15" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="I15" s="7" t="n">
+      <c r="I15" s="8" t="n">
+        <v>330</v>
+      </c>
+      <c r="J15" s="7" t="n">
         <v>350</v>
-      </c>
-      <c r="J15" s="7">
-        <f>I15-H15</f>
-        <v/>
       </c>
     </row>
     <row r="16">
@@ -987,32 +967,29 @@
       <c r="B16" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="8" t="n">
+        <v>170</v>
+      </c>
+      <c r="D16" s="7" t="n">
         <v>250</v>
-      </c>
-      <c r="D16" s="7">
-        <f>C16-B16</f>
-        <v/>
       </c>
       <c r="E16" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="F16" s="7" t="n">
+      <c r="F16" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="G16" s="7" t="n">
         <v>300</v>
-      </c>
-      <c r="G16" s="7">
-        <f>F16-E16</f>
-        <v/>
       </c>
       <c r="H16" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="I16" s="7" t="n">
+      <c r="I16" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="J16" s="7" t="n">
         <v>200</v>
-      </c>
-      <c r="J16" s="7">
-        <f>I16-H16</f>
-        <v/>
       </c>
     </row>
     <row r="17">
@@ -1024,32 +1001,29 @@
       <c r="B17" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="D17" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="D17" s="7">
-        <f>C17-B17</f>
-        <v/>
       </c>
       <c r="E17" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F17" s="7" t="n">
+      <c r="F17" s="8" t="n">
+        <v>280</v>
+      </c>
+      <c r="G17" s="7" t="n">
         <v>450</v>
-      </c>
-      <c r="G17" s="7">
-        <f>F17-E17</f>
-        <v/>
       </c>
       <c r="H17" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="I17" s="7" t="n">
+      <c r="I17" s="8" t="n">
+        <v>230</v>
+      </c>
+      <c r="J17" s="7" t="n">
         <v>350</v>
-      </c>
-      <c r="J17" s="7">
-        <f>I17-H17</f>
-        <v/>
       </c>
     </row>
     <row r="18">
@@ -1061,73 +1035,70 @@
       <c r="B18" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="D18" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="D18" s="7">
-        <f>C18-B18</f>
-        <v/>
       </c>
       <c r="E18" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="F18" s="7" t="n">
+      <c r="F18" s="8" t="n">
+        <v>110</v>
+      </c>
+      <c r="G18" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="G18" s="7">
-        <f>F18-E18</f>
-        <v/>
       </c>
       <c r="H18" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="I18" s="7" t="n">
+      <c r="I18" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J18" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="J18" s="7">
-        <f>I18-H18</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Media &amp; broadcasting</t>
         </is>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <f>SUM(B15:B18)</f>
         <v/>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <f>SUM(C15:C18)</f>
         <v/>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <f>SUM(D15:D18)</f>
         <v/>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="10">
         <f>SUM(E15:E18)</f>
         <v/>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="10">
         <f>SUM(F15:F18)</f>
         <v/>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="10">
         <f>SUM(G15:G18)</f>
         <v/>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="10">
         <f>SUM(H15:H18)</f>
         <v/>
       </c>
-      <c r="I19" s="9">
+      <c r="I19" s="10">
         <f>SUM(I15:I18)</f>
         <v/>
       </c>
-      <c r="J19" s="9">
+      <c r="J19" s="10">
         <f>SUM(J15:J18)</f>
         <v/>
       </c>
@@ -1157,32 +1128,29 @@
       <c r="B22" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="8" t="n">
+        <v>440</v>
+      </c>
+      <c r="D22" s="7" t="n">
         <v>450</v>
-      </c>
-      <c r="D22" s="7">
-        <f>C22-B22</f>
-        <v/>
       </c>
       <c r="E22" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="F22" s="7" t="n">
+      <c r="F22" s="8" t="n">
+        <v>440</v>
+      </c>
+      <c r="G22" s="7" t="n">
         <v>450</v>
-      </c>
-      <c r="G22" s="7">
-        <f>F22-E22</f>
-        <v/>
       </c>
       <c r="H22" s="7" t="n">
         <v>250</v>
       </c>
-      <c r="I22" s="7" t="n">
+      <c r="I22" s="8" t="n">
+        <v>290</v>
+      </c>
+      <c r="J22" s="7" t="n">
         <v>300</v>
-      </c>
-      <c r="J22" s="7">
-        <f>I22-H22</f>
-        <v/>
       </c>
     </row>
     <row r="23">
@@ -1194,32 +1162,29 @@
       <c r="B23" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="D23" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="D23" s="7">
-        <f>C23-B23</f>
-        <v/>
       </c>
       <c r="E23" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="F23" s="7" t="n">
+      <c r="F23" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="G23" s="7" t="n">
         <v>180</v>
-      </c>
-      <c r="G23" s="7">
-        <f>F23-E23</f>
-        <v/>
       </c>
       <c r="H23" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="I23" s="7" t="n">
+      <c r="I23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="J23" s="7">
-        <f>I23-H23</f>
-        <v/>
       </c>
     </row>
     <row r="24">
@@ -1231,32 +1196,29 @@
       <c r="B24" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="8" t="n">
+        <v>590</v>
+      </c>
+      <c r="D24" s="7" t="n">
         <v>700</v>
-      </c>
-      <c r="D24" s="7">
-        <f>C24-B24</f>
-        <v/>
       </c>
       <c r="E24" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="F24" s="7" t="n">
+      <c r="F24" s="8" t="n">
+        <v>680</v>
+      </c>
+      <c r="G24" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="G24" s="7">
-        <f>F24-E24</f>
-        <v/>
       </c>
       <c r="H24" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="I24" s="7" t="n">
+      <c r="I24" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="J24" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="J24" s="7">
-        <f>I24-H24</f>
-        <v/>
       </c>
     </row>
     <row r="25">
@@ -1268,73 +1230,70 @@
       <c r="B25" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="8" t="n">
         <v>220</v>
       </c>
-      <c r="D25" s="7">
-        <f>C25-B25</f>
-        <v/>
+      <c r="D25" s="7" t="n">
+        <v>220</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="F25" s="7" t="n">
+      <c r="F25" s="8" t="n">
         <v>220</v>
       </c>
-      <c r="G25" s="7">
-        <f>F25-E25</f>
-        <v/>
+      <c r="G25" s="7" t="n">
+        <v>220</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>180</v>
       </c>
-      <c r="I25" s="7" t="n">
+      <c r="I25" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="J25" s="7">
-        <f>I25-H25</f>
-        <v/>
+      <c r="J25" s="7" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Conference &amp; NCAA distributions</t>
         </is>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <f>SUM(B22:B25)</f>
         <v/>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="10">
         <f>SUM(C22:C25)</f>
         <v/>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <f>SUM(D22:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="10">
         <f>SUM(E22:E25)</f>
         <v/>
       </c>
-      <c r="F26" s="9">
+      <c r="F26" s="10">
         <f>SUM(F22:F25)</f>
         <v/>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="10">
         <f>SUM(G22:G25)</f>
         <v/>
       </c>
-      <c r="H26" s="9">
+      <c r="H26" s="10">
         <f>SUM(H22:H25)</f>
         <v/>
       </c>
-      <c r="I26" s="9">
+      <c r="I26" s="10">
         <f>SUM(I22:I25)</f>
         <v/>
       </c>
-      <c r="J26" s="9">
+      <c r="J26" s="10">
         <f>SUM(J22:J25)</f>
         <v/>
       </c>
@@ -1364,32 +1323,29 @@
       <c r="B29" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C29" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="D29" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="D29" s="7">
-        <f>C29-B29</f>
-        <v/>
       </c>
       <c r="E29" s="7" t="n">
         <v>350</v>
       </c>
-      <c r="F29" s="7" t="n">
+      <c r="F29" s="8" t="n">
+        <v>680</v>
+      </c>
+      <c r="G29" s="7" t="n">
         <v>900</v>
-      </c>
-      <c r="G29" s="7">
-        <f>F29-E29</f>
-        <v/>
       </c>
       <c r="H29" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="I29" s="7" t="n">
+      <c r="I29" s="8" t="n">
+        <v>640</v>
+      </c>
+      <c r="J29" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="J29" s="7">
-        <f>I29-H29</f>
-        <v/>
       </c>
     </row>
     <row r="30">
@@ -1401,32 +1357,29 @@
       <c r="B30" s="7" t="n">
         <v>250</v>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C30" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="D30" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="D30" s="7">
-        <f>C30-B30</f>
-        <v/>
       </c>
       <c r="E30" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="F30" s="7" t="n">
+      <c r="F30" s="8" t="n">
+        <v>840</v>
+      </c>
+      <c r="G30" s="7" t="n">
         <v>1200</v>
-      </c>
-      <c r="G30" s="7">
-        <f>F30-E30</f>
-        <v/>
       </c>
       <c r="H30" s="7" t="n">
         <v>350</v>
       </c>
-      <c r="I30" s="7" t="n">
+      <c r="I30" s="8" t="n">
+        <v>740</v>
+      </c>
+      <c r="J30" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="J30" s="7">
-        <f>I30-H30</f>
-        <v/>
       </c>
     </row>
     <row r="31">
@@ -1438,32 +1391,29 @@
       <c r="B31" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C31" s="8" t="n">
+        <v>140</v>
+      </c>
+      <c r="D31" s="7" t="n">
         <v>200</v>
-      </c>
-      <c r="D31" s="7">
-        <f>C31-B31</f>
-        <v/>
       </c>
       <c r="E31" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="F31" s="7" t="n">
+      <c r="F31" s="8" t="n">
+        <v>210</v>
+      </c>
+      <c r="G31" s="7" t="n">
         <v>300</v>
-      </c>
-      <c r="G31" s="7">
-        <f>F31-E31</f>
-        <v/>
       </c>
       <c r="H31" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="I31" s="7" t="n">
+      <c r="I31" s="8" t="n">
+        <v>190</v>
+      </c>
+      <c r="J31" s="7" t="n">
         <v>250</v>
-      </c>
-      <c r="J31" s="7">
-        <f>I31-H31</f>
-        <v/>
       </c>
     </row>
     <row r="32">
@@ -1475,32 +1425,29 @@
       <c r="B32" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="C32" s="7" t="n">
+      <c r="C32" s="8" t="n">
+        <v>280</v>
+      </c>
+      <c r="D32" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="D32" s="7">
-        <f>C32-B32</f>
-        <v/>
       </c>
       <c r="E32" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="F32" s="7" t="n">
+      <c r="F32" s="8" t="n">
+        <v>320</v>
+      </c>
+      <c r="G32" s="7" t="n">
         <v>450</v>
-      </c>
-      <c r="G32" s="7">
-        <f>F32-E32</f>
-        <v/>
       </c>
       <c r="H32" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="I32" s="7" t="n">
+      <c r="I32" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="J32" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="J32" s="7">
-        <f>I32-H32</f>
-        <v/>
       </c>
     </row>
     <row r="33">
@@ -1512,32 +1459,29 @@
       <c r="B33" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C33" s="7" t="n">
+      <c r="C33" s="8" t="n">
+        <v>480</v>
+      </c>
+      <c r="D33" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="D33" s="7">
-        <f>C33-B33</f>
-        <v/>
       </c>
       <c r="E33" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="7" t="n">
+      <c r="F33" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="G33" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="G33" s="7">
-        <f>F33-E33</f>
-        <v/>
       </c>
       <c r="H33" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I33" s="7" t="n">
+      <c r="I33" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="J33" s="7" t="n">
         <v>700</v>
-      </c>
-      <c r="J33" s="7">
-        <f>I33-H33</f>
-        <v/>
       </c>
     </row>
     <row r="34">
@@ -1549,32 +1493,29 @@
       <c r="B34" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="C34" s="7" t="n">
+      <c r="C34" s="8" t="n">
+        <v>110</v>
+      </c>
+      <c r="D34" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="D34" s="7">
-        <f>C34-B34</f>
-        <v/>
       </c>
       <c r="E34" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="F34" s="7" t="n">
+      <c r="F34" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="G34" s="7" t="n">
         <v>180</v>
-      </c>
-      <c r="G34" s="7">
-        <f>F34-E34</f>
-        <v/>
       </c>
       <c r="H34" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="I34" s="7" t="n">
+      <c r="I34" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J34" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="J34" s="7">
-        <f>I34-H34</f>
-        <v/>
       </c>
     </row>
     <row r="35">
@@ -1586,73 +1527,70 @@
       <c r="B35" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="C35" s="7" t="n">
+      <c r="C35" s="8" t="n">
+        <v>310</v>
+      </c>
+      <c r="D35" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="D35" s="7">
-        <f>C35-B35</f>
-        <v/>
       </c>
       <c r="E35" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="F35" s="7" t="n">
+      <c r="F35" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="G35" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="G35" s="7">
-        <f>F35-E35</f>
-        <v/>
       </c>
       <c r="H35" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="I35" s="7" t="n">
+      <c r="I35" s="8" t="n">
+        <v>280</v>
+      </c>
+      <c r="J35" s="7" t="n">
         <v>450</v>
       </c>
-      <c r="J35" s="7">
-        <f>I35-H35</f>
-        <v/>
-      </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Corporate sponsorship &amp; multimedia rights</t>
         </is>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="10">
         <f>SUM(B29:B35)</f>
         <v/>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="10">
         <f>SUM(C29:C35)</f>
         <v/>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="10">
         <f>SUM(D29:D35)</f>
         <v/>
       </c>
-      <c r="E36" s="9">
+      <c r="E36" s="10">
         <f>SUM(E29:E35)</f>
         <v/>
       </c>
-      <c r="F36" s="9">
+      <c r="F36" s="10">
         <f>SUM(F29:F35)</f>
         <v/>
       </c>
-      <c r="G36" s="9">
+      <c r="G36" s="10">
         <f>SUM(G29:G35)</f>
         <v/>
       </c>
-      <c r="H36" s="9">
+      <c r="H36" s="10">
         <f>SUM(H29:H35)</f>
         <v/>
       </c>
-      <c r="I36" s="9">
+      <c r="I36" s="10">
         <f>SUM(I29:I35)</f>
         <v/>
       </c>
-      <c r="J36" s="9">
+      <c r="J36" s="10">
         <f>SUM(J29:J35)</f>
         <v/>
       </c>
@@ -1682,32 +1620,29 @@
       <c r="B39" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C39" s="7" t="n">
+      <c r="C39" s="8" t="n">
+        <v>930</v>
+      </c>
+      <c r="D39" s="7" t="n">
         <v>1200</v>
-      </c>
-      <c r="D39" s="7">
-        <f>C39-B39</f>
-        <v/>
       </c>
       <c r="E39" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="F39" s="7" t="n">
+      <c r="F39" s="8" t="n">
+        <v>1400</v>
+      </c>
+      <c r="G39" s="7" t="n">
         <v>1800</v>
-      </c>
-      <c r="G39" s="7">
-        <f>F39-E39</f>
-        <v/>
       </c>
       <c r="H39" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="I39" s="7" t="n">
+      <c r="I39" s="8" t="n">
+        <v>780</v>
+      </c>
+      <c r="J39" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="J39" s="7">
-        <f>I39-H39</f>
-        <v/>
       </c>
     </row>
     <row r="40">
@@ -1719,32 +1654,29 @@
       <c r="B40" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="C40" s="7" t="n">
+      <c r="C40" s="8" t="n">
+        <v>580</v>
+      </c>
+      <c r="D40" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="D40" s="7">
-        <f>C40-B40</f>
-        <v/>
       </c>
       <c r="E40" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="F40" s="7" t="n">
+      <c r="F40" s="8" t="n">
+        <v>880</v>
+      </c>
+      <c r="G40" s="7" t="n">
         <v>1200</v>
-      </c>
-      <c r="G40" s="7">
-        <f>F40-E40</f>
-        <v/>
       </c>
       <c r="H40" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="I40" s="7" t="n">
+      <c r="I40" s="8" t="n">
+        <v>480</v>
+      </c>
+      <c r="J40" s="7" t="n">
         <v>700</v>
-      </c>
-      <c r="J40" s="7">
-        <f>I40-H40</f>
-        <v/>
       </c>
     </row>
     <row r="41">
@@ -1756,32 +1688,29 @@
       <c r="B41" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="C41" s="7" t="n">
+      <c r="C41" s="8" t="n">
+        <v>640</v>
+      </c>
+      <c r="D41" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="D41" s="7">
-        <f>C41-B41</f>
-        <v/>
       </c>
       <c r="E41" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="F41" s="7" t="n">
+      <c r="F41" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G41" s="7" t="n">
         <v>1500</v>
-      </c>
-      <c r="G41" s="7">
-        <f>F41-E41</f>
-        <v/>
       </c>
       <c r="H41" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="I41" s="7" t="n">
+      <c r="I41" s="8" t="n">
+        <v>560</v>
+      </c>
+      <c r="J41" s="7" t="n">
         <v>900</v>
-      </c>
-      <c r="J41" s="7">
-        <f>I41-H41</f>
-        <v/>
       </c>
     </row>
     <row r="42">
@@ -1793,32 +1722,29 @@
       <c r="B42" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="C42" s="7" t="n">
+      <c r="C42" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="D42" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="D42" s="7">
-        <f>C42-B42</f>
-        <v/>
       </c>
       <c r="E42" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="F42" s="7" t="n">
+      <c r="F42" s="8" t="n">
+        <v>480</v>
+      </c>
+      <c r="G42" s="7" t="n">
         <v>700</v>
-      </c>
-      <c r="G42" s="7">
-        <f>F42-E42</f>
-        <v/>
       </c>
       <c r="H42" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="I42" s="7" t="n">
+      <c r="I42" s="8" t="n">
+        <v>320</v>
+      </c>
+      <c r="J42" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="J42" s="7">
-        <f>I42-H42</f>
-        <v/>
       </c>
     </row>
     <row r="43">
@@ -1830,73 +1756,70 @@
       <c r="B43" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="C43" s="7" t="n">
+      <c r="C43" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="D43" s="7" t="n">
         <v>1200</v>
-      </c>
-      <c r="D43" s="7">
-        <f>C43-B43</f>
-        <v/>
       </c>
       <c r="E43" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="F43" s="7" t="n">
+      <c r="F43" s="8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="G43" s="7" t="n">
         <v>1500</v>
-      </c>
-      <c r="G43" s="7">
-        <f>F43-E43</f>
-        <v/>
       </c>
       <c r="H43" s="7" t="n">
         <v>250</v>
       </c>
-      <c r="I43" s="7" t="n">
+      <c r="I43" s="8" t="n">
+        <v>660</v>
+      </c>
+      <c r="J43" s="7" t="n">
         <v>1000</v>
       </c>
-      <c r="J43" s="7">
-        <f>I43-H43</f>
-        <v/>
-      </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="A44" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Philanthropy &amp; donor</t>
         </is>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="10">
         <f>SUM(B39:B43)</f>
         <v/>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="10">
         <f>SUM(C39:C43)</f>
         <v/>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="10">
         <f>SUM(D39:D43)</f>
         <v/>
       </c>
-      <c r="E44" s="9">
+      <c r="E44" s="10">
         <f>SUM(E39:E43)</f>
         <v/>
       </c>
-      <c r="F44" s="9">
+      <c r="F44" s="10">
         <f>SUM(F39:F43)</f>
         <v/>
       </c>
-      <c r="G44" s="9">
+      <c r="G44" s="10">
         <f>SUM(G39:G43)</f>
         <v/>
       </c>
-      <c r="H44" s="9">
+      <c r="H44" s="10">
         <f>SUM(H39:H43)</f>
         <v/>
       </c>
-      <c r="I44" s="9">
+      <c r="I44" s="10">
         <f>SUM(I39:I43)</f>
         <v/>
       </c>
-      <c r="J44" s="9">
+      <c r="J44" s="10">
         <f>SUM(J39:J43)</f>
         <v/>
       </c>
@@ -1926,32 +1849,29 @@
       <c r="B47" s="7" t="n">
         <v>250</v>
       </c>
-      <c r="C47" s="7" t="n">
+      <c r="C47" s="8" t="n">
+        <v>520</v>
+      </c>
+      <c r="D47" s="7" t="n">
         <v>700</v>
-      </c>
-      <c r="D47" s="7">
-        <f>C47-B47</f>
-        <v/>
       </c>
       <c r="E47" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="F47" s="7" t="n">
+      <c r="F47" s="8" t="n">
+        <v>660</v>
+      </c>
+      <c r="G47" s="7" t="n">
         <v>900</v>
-      </c>
-      <c r="G47" s="7">
-        <f>F47-E47</f>
-        <v/>
       </c>
       <c r="H47" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="I47" s="7" t="n">
+      <c r="I47" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="J47" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="J47" s="7">
-        <f>I47-H47</f>
-        <v/>
       </c>
     </row>
     <row r="48">
@@ -1963,32 +1883,29 @@
       <c r="B48" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="C48" s="7" t="n">
+      <c r="C48" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="D48" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="D48" s="7">
-        <f>C48-B48</f>
-        <v/>
       </c>
       <c r="E48" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="F48" s="7" t="n">
+      <c r="F48" s="8" t="n">
+        <v>390</v>
+      </c>
+      <c r="G48" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="G48" s="7">
-        <f>F48-E48</f>
-        <v/>
       </c>
       <c r="H48" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="I48" s="7" t="n">
+      <c r="I48" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="J48" s="7" t="n">
         <v>300</v>
-      </c>
-      <c r="J48" s="7">
-        <f>I48-H48</f>
-        <v/>
       </c>
     </row>
     <row r="49">
@@ -2000,32 +1917,29 @@
       <c r="B49" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="C49" s="7" t="n">
+      <c r="C49" s="8" t="n">
+        <v>520</v>
+      </c>
+      <c r="D49" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="D49" s="7">
-        <f>C49-B49</f>
-        <v/>
       </c>
       <c r="E49" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="F49" s="7" t="n">
+      <c r="F49" s="8" t="n">
+        <v>660</v>
+      </c>
+      <c r="G49" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="G49" s="7">
-        <f>F49-E49</f>
-        <v/>
       </c>
       <c r="H49" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="I49" s="7" t="n">
+      <c r="I49" s="8" t="n">
+        <v>410</v>
+      </c>
+      <c r="J49" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="J49" s="7">
-        <f>I49-H49</f>
-        <v/>
       </c>
     </row>
     <row r="50">
@@ -2037,73 +1951,70 @@
       <c r="B50" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="C50" s="7" t="n">
+      <c r="C50" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="D50" s="7" t="n">
         <v>100</v>
-      </c>
-      <c r="D50" s="7">
-        <f>C50-B50</f>
-        <v/>
       </c>
       <c r="E50" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="F50" s="7" t="n">
+      <c r="F50" s="8" t="n">
+        <v>110</v>
+      </c>
+      <c r="G50" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="G50" s="7">
-        <f>F50-E50</f>
-        <v/>
       </c>
       <c r="H50" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="I50" s="7" t="n">
+      <c r="I50" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J50" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="J50" s="7">
-        <f>I50-H50</f>
-        <v/>
-      </c>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Apparel &amp; licensing</t>
         </is>
       </c>
-      <c r="B51" s="9">
+      <c r="B51" s="10">
         <f>SUM(B47:B50)</f>
         <v/>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="10">
         <f>SUM(C47:C50)</f>
         <v/>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="10">
         <f>SUM(D47:D50)</f>
         <v/>
       </c>
-      <c r="E51" s="9">
+      <c r="E51" s="10">
         <f>SUM(E47:E50)</f>
         <v/>
       </c>
-      <c r="F51" s="9">
+      <c r="F51" s="10">
         <f>SUM(F47:F50)</f>
         <v/>
       </c>
-      <c r="G51" s="9">
+      <c r="G51" s="10">
         <f>SUM(G47:G50)</f>
         <v/>
       </c>
-      <c r="H51" s="9">
+      <c r="H51" s="10">
         <f>SUM(H47:H50)</f>
         <v/>
       </c>
-      <c r="I51" s="9">
+      <c r="I51" s="10">
         <f>SUM(I47:I50)</f>
         <v/>
       </c>
-      <c r="J51" s="9">
+      <c r="J51" s="10">
         <f>SUM(J47:J50)</f>
         <v/>
       </c>
@@ -2133,32 +2044,29 @@
       <c r="B54" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="C54" s="7" t="n">
+      <c r="C54" s="8" t="n">
+        <v>490</v>
+      </c>
+      <c r="D54" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="D54" s="7">
-        <f>C54-B54</f>
-        <v/>
       </c>
       <c r="E54" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="F54" s="7" t="n">
+      <c r="F54" s="8" t="n">
+        <v>490</v>
+      </c>
+      <c r="G54" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="G54" s="7">
-        <f>F54-E54</f>
-        <v/>
       </c>
       <c r="H54" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="I54" s="7" t="n">
+      <c r="I54" s="8" t="n">
+        <v>460</v>
+      </c>
+      <c r="J54" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="J54" s="7">
-        <f>I54-H54</f>
-        <v/>
       </c>
     </row>
     <row r="55">
@@ -2170,32 +2078,29 @@
       <c r="B55" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="C55" s="7" t="n">
+      <c r="C55" s="8" t="n">
+        <v>530</v>
+      </c>
+      <c r="D55" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="D55" s="7">
-        <f>C55-B55</f>
-        <v/>
       </c>
       <c r="E55" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="F55" s="7" t="n">
+      <c r="F55" s="8" t="n">
+        <v>620</v>
+      </c>
+      <c r="G55" s="7" t="n">
         <v>900</v>
-      </c>
-      <c r="G55" s="7">
-        <f>F55-E55</f>
-        <v/>
       </c>
       <c r="H55" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="I55" s="7" t="n">
+      <c r="I55" s="8" t="n">
+        <v>550</v>
+      </c>
+      <c r="J55" s="7" t="n">
         <v>700</v>
-      </c>
-      <c r="J55" s="7">
-        <f>I55-H55</f>
-        <v/>
       </c>
     </row>
     <row r="56">
@@ -2207,32 +2112,29 @@
       <c r="B56" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="C56" s="7" t="n">
+      <c r="C56" s="8" t="n">
+        <v>280</v>
+      </c>
+      <c r="D56" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="D56" s="7">
-        <f>C56-B56</f>
-        <v/>
       </c>
       <c r="E56" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="F56" s="7" t="n">
+      <c r="F56" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="G56" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="G56" s="7">
-        <f>F56-E56</f>
-        <v/>
       </c>
       <c r="H56" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="I56" s="7" t="n">
+      <c r="I56" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="J56" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="J56" s="7">
-        <f>I56-H56</f>
-        <v/>
       </c>
     </row>
     <row r="57">
@@ -2244,73 +2146,70 @@
       <c r="B57" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C57" s="7" t="n">
+      <c r="C57" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="D57" s="7" t="n">
         <v>100</v>
-      </c>
-      <c r="D57" s="7">
-        <f>C57-B57</f>
-        <v/>
       </c>
       <c r="E57" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="F57" s="7" t="n">
+      <c r="F57" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G57" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="G57" s="7">
-        <f>F57-E57</f>
-        <v/>
       </c>
       <c r="H57" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="I57" s="7" t="n">
+      <c r="I57" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J57" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="J57" s="7">
-        <f>I57-H57</f>
-        <v/>
-      </c>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="A58" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Guarantees &amp; scheduling</t>
         </is>
       </c>
-      <c r="B58" s="9">
+      <c r="B58" s="10">
         <f>SUM(B54:B57)</f>
         <v/>
       </c>
-      <c r="C58" s="9">
+      <c r="C58" s="10">
         <f>SUM(C54:C57)</f>
         <v/>
       </c>
-      <c r="D58" s="9">
+      <c r="D58" s="10">
         <f>SUM(D54:D57)</f>
         <v/>
       </c>
-      <c r="E58" s="9">
+      <c r="E58" s="10">
         <f>SUM(E54:E57)</f>
         <v/>
       </c>
-      <c r="F58" s="9">
+      <c r="F58" s="10">
         <f>SUM(F54:F57)</f>
         <v/>
       </c>
-      <c r="G58" s="9">
+      <c r="G58" s="10">
         <f>SUM(G54:G57)</f>
         <v/>
       </c>
-      <c r="H58" s="9">
+      <c r="H58" s="10">
         <f>SUM(H54:H57)</f>
         <v/>
       </c>
-      <c r="I58" s="9">
+      <c r="I58" s="10">
         <f>SUM(I54:I57)</f>
         <v/>
       </c>
-      <c r="J58" s="9">
+      <c r="J58" s="10">
         <f>SUM(J54:J57)</f>
         <v/>
       </c>
@@ -2340,32 +2239,29 @@
       <c r="B61" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="C61" s="7" t="n">
+      <c r="C61" s="8" t="n">
+        <v>310</v>
+      </c>
+      <c r="D61" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="D61" s="7">
-        <f>C61-B61</f>
-        <v/>
       </c>
       <c r="E61" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="F61" s="7" t="n">
+      <c r="F61" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="G61" s="7" t="n">
         <v>500</v>
-      </c>
-      <c r="G61" s="7">
-        <f>F61-E61</f>
-        <v/>
       </c>
       <c r="H61" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="I61" s="7" t="n">
+      <c r="I61" s="8" t="n">
+        <v>280</v>
+      </c>
+      <c r="J61" s="7" t="n">
         <v>350</v>
-      </c>
-      <c r="J61" s="7">
-        <f>I61-H61</f>
-        <v/>
       </c>
     </row>
     <row r="62">
@@ -2377,32 +2273,29 @@
       <c r="B62" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="C62" s="7" t="n">
+      <c r="C62" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="D62" s="7" t="n">
         <v>200</v>
-      </c>
-      <c r="D62" s="7">
-        <f>C62-B62</f>
-        <v/>
       </c>
       <c r="E62" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="F62" s="7" t="n">
+      <c r="F62" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="G62" s="7" t="n">
         <v>250</v>
-      </c>
-      <c r="G62" s="7">
-        <f>F62-E62</f>
-        <v/>
       </c>
       <c r="H62" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="I62" s="7" t="n">
+      <c r="I62" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="J62" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="J62" s="7">
-        <f>I62-H62</f>
-        <v/>
       </c>
     </row>
     <row r="63">
@@ -2414,73 +2307,70 @@
       <c r="B63" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C63" s="7" t="n">
+      <c r="C63" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="D63" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="D63" s="7">
-        <f>C63-B63</f>
-        <v/>
       </c>
       <c r="E63" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="F63" s="7" t="n">
+      <c r="F63" s="8" t="n">
+        <v>140</v>
+      </c>
+      <c r="G63" s="7" t="n">
         <v>180</v>
-      </c>
-      <c r="G63" s="7">
-        <f>F63-E63</f>
-        <v/>
       </c>
       <c r="H63" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="I63" s="7" t="n">
+      <c r="I63" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="J63" s="7" t="n">
         <v>250</v>
       </c>
-      <c r="J63" s="7">
-        <f>I63-H63</f>
-        <v/>
-      </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="A64" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Camps, clinics &amp; operations</t>
         </is>
       </c>
-      <c r="B64" s="9">
+      <c r="B64" s="10">
         <f>SUM(B61:B63)</f>
         <v/>
       </c>
-      <c r="C64" s="9">
+      <c r="C64" s="10">
         <f>SUM(C61:C63)</f>
         <v/>
       </c>
-      <c r="D64" s="9">
+      <c r="D64" s="10">
         <f>SUM(D61:D63)</f>
         <v/>
       </c>
-      <c r="E64" s="9">
+      <c r="E64" s="10">
         <f>SUM(E61:E63)</f>
         <v/>
       </c>
-      <c r="F64" s="9">
+      <c r="F64" s="10">
         <f>SUM(F61:F63)</f>
         <v/>
       </c>
-      <c r="G64" s="9">
+      <c r="G64" s="10">
         <f>SUM(G61:G63)</f>
         <v/>
       </c>
-      <c r="H64" s="9">
+      <c r="H64" s="10">
         <f>SUM(H61:H63)</f>
         <v/>
       </c>
-      <c r="I64" s="9">
+      <c r="I64" s="10">
         <f>SUM(I61:I63)</f>
         <v/>
       </c>
-      <c r="J64" s="9">
+      <c r="J64" s="10">
         <f>SUM(J61:J63)</f>
         <v/>
       </c>
@@ -2510,32 +2400,29 @@
       <c r="B67" s="7" t="n">
         <v>800</v>
       </c>
-      <c r="C67" s="7" t="n">
+      <c r="C67" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="D67" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="D67" s="7">
-        <f>C67-B67</f>
-        <v/>
       </c>
       <c r="E67" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="F67" s="7" t="n">
+      <c r="F67" s="8" t="n">
+        <v>450</v>
+      </c>
+      <c r="G67" s="7" t="n">
         <v>300</v>
-      </c>
-      <c r="G67" s="7">
-        <f>F67-E67</f>
-        <v/>
       </c>
       <c r="H67" s="7" t="n">
         <v>1200</v>
       </c>
-      <c r="I67" s="7" t="n">
+      <c r="I67" s="8" t="n">
+        <v>950</v>
+      </c>
+      <c r="J67" s="7" t="n">
         <v>700</v>
-      </c>
-      <c r="J67" s="7">
-        <f>I67-H67</f>
-        <v/>
       </c>
     </row>
     <row r="68">
@@ -2547,32 +2434,29 @@
       <c r="B68" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="C68" s="7" t="n">
+      <c r="C68" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="D68" s="7" t="n">
         <v>100</v>
-      </c>
-      <c r="D68" s="7">
-        <f>C68-B68</f>
-        <v/>
       </c>
       <c r="E68" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="F68" s="7" t="n">
+      <c r="F68" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="G68" s="7" t="n">
         <v>50</v>
-      </c>
-      <c r="G68" s="7">
-        <f>F68-E68</f>
-        <v/>
       </c>
       <c r="H68" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="I68" s="7" t="n">
+      <c r="I68" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="J68" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="J68" s="7">
-        <f>I68-H68</f>
-        <v/>
       </c>
     </row>
     <row r="69">
@@ -2584,32 +2468,29 @@
       <c r="B69" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C69" s="7" t="n">
+      <c r="C69" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D69" s="7">
-        <f>C69-B69</f>
-        <v/>
+      <c r="D69" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="E69" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F69" s="7" t="n">
+      <c r="F69" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G69" s="7">
-        <f>F69-E69</f>
-        <v/>
+      <c r="G69" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
         <v>800</v>
       </c>
-      <c r="I69" s="7" t="n">
+      <c r="I69" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="J69" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="J69" s="7">
-        <f>I69-H69</f>
-        <v/>
       </c>
     </row>
     <row r="70">
@@ -2621,32 +2502,29 @@
       <c r="B70" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="C70" s="7" t="n">
+      <c r="C70" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="D70" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="D70" s="7">
-        <f>C70-B70</f>
-        <v/>
       </c>
       <c r="E70" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="F70" s="7" t="n">
+      <c r="F70" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="G70" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="G70" s="7">
-        <f>F70-E70</f>
-        <v/>
       </c>
       <c r="H70" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="I70" s="7" t="n">
+      <c r="I70" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J70" s="7" t="n">
         <v>80</v>
-      </c>
-      <c r="J70" s="7">
-        <f>I70-H70</f>
-        <v/>
       </c>
     </row>
     <row r="71">
@@ -2658,32 +2536,29 @@
       <c r="B71" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C71" s="7" t="n">
+      <c r="C71" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="D71" s="7" t="n">
         <v>100</v>
-      </c>
-      <c r="D71" s="7">
-        <f>C71-B71</f>
-        <v/>
       </c>
       <c r="E71" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="F71" s="7" t="n">
+      <c r="F71" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="G71" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="G71" s="7">
-        <f>F71-E71</f>
-        <v/>
       </c>
       <c r="H71" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="I71" s="7" t="n">
+      <c r="I71" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J71" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="J71" s="7">
-        <f>I71-H71</f>
-        <v/>
       </c>
     </row>
     <row r="72">
@@ -2695,73 +2570,70 @@
       <c r="B72" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C72" s="7" t="n">
+      <c r="C72" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="D72" s="7" t="n">
         <v>100</v>
-      </c>
-      <c r="D72" s="7">
-        <f>C72-B72</f>
-        <v/>
       </c>
       <c r="E72" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="F72" s="7" t="n">
+      <c r="F72" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G72" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="G72" s="7">
-        <f>F72-E72</f>
-        <v/>
       </c>
       <c r="H72" s="7" t="n">
         <v>70</v>
       </c>
-      <c r="I72" s="7" t="n">
+      <c r="I72" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J72" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="J72" s="7">
-        <f>I72-H72</f>
-        <v/>
-      </c>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="inlineStr">
+      <c r="A73" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Institutional &amp; other support</t>
         </is>
       </c>
-      <c r="B73" s="9">
+      <c r="B73" s="10">
         <f>SUM(B67:B72)</f>
         <v/>
       </c>
-      <c r="C73" s="9">
+      <c r="C73" s="10">
         <f>SUM(C67:C72)</f>
         <v/>
       </c>
-      <c r="D73" s="9">
+      <c r="D73" s="10">
         <f>SUM(D67:D72)</f>
         <v/>
       </c>
-      <c r="E73" s="9">
+      <c r="E73" s="10">
         <f>SUM(E67:E72)</f>
         <v/>
       </c>
-      <c r="F73" s="9">
+      <c r="F73" s="10">
         <f>SUM(F67:F72)</f>
         <v/>
       </c>
-      <c r="G73" s="9">
+      <c r="G73" s="10">
         <f>SUM(G67:G72)</f>
         <v/>
       </c>
-      <c r="H73" s="9">
+      <c r="H73" s="10">
         <f>SUM(H67:H72)</f>
         <v/>
       </c>
-      <c r="I73" s="9">
+      <c r="I73" s="10">
         <f>SUM(I67:I72)</f>
         <v/>
       </c>
-      <c r="J73" s="9">
+      <c r="J73" s="10">
         <f>SUM(J67:J72)</f>
         <v/>
       </c>
@@ -2791,32 +2663,29 @@
       <c r="B76" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="C76" s="7" t="n">
+      <c r="C76" s="8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D76" s="7" t="n">
         <v>3000</v>
-      </c>
-      <c r="D76" s="7">
-        <f>C76-B76</f>
-        <v/>
       </c>
       <c r="E76" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="F76" s="7" t="n">
+      <c r="F76" s="8" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G76" s="7" t="n">
         <v>3500</v>
-      </c>
-      <c r="G76" s="7">
-        <f>F76-E76</f>
-        <v/>
       </c>
       <c r="H76" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="I76" s="7" t="n">
+      <c r="I76" s="8" t="n">
+        <v>1680</v>
+      </c>
+      <c r="J76" s="7" t="n">
         <v>2500</v>
-      </c>
-      <c r="J76" s="7">
-        <f>I76-H76</f>
-        <v/>
       </c>
     </row>
     <row r="77">
@@ -2828,32 +2697,29 @@
       <c r="B77" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C77" s="7" t="n">
+      <c r="C77" s="8" t="n">
+        <v>540</v>
+      </c>
+      <c r="D77" s="7" t="n">
         <v>800</v>
-      </c>
-      <c r="D77" s="7">
-        <f>C77-B77</f>
-        <v/>
       </c>
       <c r="E77" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="F77" s="7" t="n">
+      <c r="F77" s="8" t="n">
+        <v>680</v>
+      </c>
+      <c r="G77" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="G77" s="7">
-        <f>F77-E77</f>
-        <v/>
       </c>
       <c r="H77" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="I77" s="7" t="n">
+      <c r="I77" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="J77" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="J77" s="7">
-        <f>I77-H77</f>
-        <v/>
       </c>
     </row>
     <row r="78">
@@ -2865,425 +2731,390 @@
       <c r="B78" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C78" s="7" t="n">
+      <c r="C78" s="8" t="n">
+        <v>1620</v>
+      </c>
+      <c r="D78" s="7" t="n">
         <v>2500</v>
-      </c>
-      <c r="D78" s="7">
-        <f>C78-B78</f>
-        <v/>
       </c>
       <c r="E78" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F78" s="7" t="n">
+      <c r="F78" s="8" t="n">
+        <v>1620</v>
+      </c>
+      <c r="G78" s="7" t="n">
         <v>2500</v>
-      </c>
-      <c r="G78" s="7">
-        <f>F78-E78</f>
-        <v/>
       </c>
       <c r="H78" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I78" s="7" t="n">
+      <c r="I78" s="8" t="n">
+        <v>1620</v>
+      </c>
+      <c r="J78" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="J78" s="7">
-        <f>I78-H78</f>
-        <v/>
-      </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="inlineStr">
+      <c r="A79" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — NIL / revenue-share era</t>
         </is>
       </c>
-      <c r="B79" s="9">
+      <c r="B79" s="10">
         <f>SUM(B76:B78)</f>
         <v/>
       </c>
-      <c r="C79" s="9">
+      <c r="C79" s="10">
         <f>SUM(C76:C78)</f>
         <v/>
       </c>
-      <c r="D79" s="9">
+      <c r="D79" s="10">
         <f>SUM(D76:D78)</f>
         <v/>
       </c>
-      <c r="E79" s="9">
+      <c r="E79" s="10">
         <f>SUM(E76:E78)</f>
         <v/>
       </c>
-      <c r="F79" s="9">
+      <c r="F79" s="10">
         <f>SUM(F76:F78)</f>
         <v/>
       </c>
-      <c r="G79" s="9">
+      <c r="G79" s="10">
         <f>SUM(G76:G78)</f>
         <v/>
       </c>
-      <c r="H79" s="9">
+      <c r="H79" s="10">
         <f>SUM(H76:H78)</f>
         <v/>
       </c>
-      <c r="I79" s="9">
+      <c r="I79" s="10">
         <f>SUM(I76:I78)</f>
         <v/>
       </c>
-      <c r="J79" s="9">
+      <c r="J79" s="10">
         <f>SUM(J76:J78)</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="10" t="inlineStr">
+      <c r="A81" s="11" t="inlineStr">
         <is>
           <t>PROGRAM REVENUE  (categories 1–9, excl. NIL)</t>
         </is>
       </c>
-      <c r="B81" s="11">
+      <c r="B81" s="12">
         <f>B12+B19+B26+B36+B44+B51+B58+B64+B73</f>
         <v/>
       </c>
-      <c r="C81" s="11">
+      <c r="C81" s="12">
         <f>C12+C19+C26+C36+C44+C51+C58+C64+C73</f>
         <v/>
       </c>
-      <c r="D81" s="11">
+      <c r="D81" s="12">
         <f>D12+D19+D26+D36+D44+D51+D58+D64+D73</f>
         <v/>
       </c>
-      <c r="E81" s="11">
+      <c r="E81" s="12">
         <f>E12+E19+E26+E36+E44+E51+E58+E64+E73</f>
         <v/>
       </c>
-      <c r="F81" s="11">
+      <c r="F81" s="12">
         <f>F12+F19+F26+F36+F44+F51+F58+F64+F73</f>
         <v/>
       </c>
-      <c r="G81" s="11">
+      <c r="G81" s="12">
         <f>G12+G19+G26+G36+G44+G51+G58+G64+G73</f>
         <v/>
       </c>
-      <c r="H81" s="11">
+      <c r="H81" s="12">
         <f>H12+H19+H26+H36+H44+H51+H58+H64+H73</f>
         <v/>
       </c>
-      <c r="I81" s="11">
+      <c r="I81" s="12">
         <f>I12+I19+I26+I36+I44+I51+I58+I64+I73</f>
         <v/>
       </c>
-      <c r="J81" s="11">
+      <c r="J81" s="12">
         <f>J12+J19+J26+J36+J44+J51+J58+J64+J73</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="12" t="inlineStr">
-        <is>
-          <t>NIL / rev-share funding  (memo — SPV-funded, cost-side)</t>
-        </is>
-      </c>
-      <c r="B82" s="13">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>NIL / rev-share funding  (memo — SPV-funded cost)</t>
+        </is>
+      </c>
+      <c r="B82" s="14">
         <f>B79</f>
         <v/>
       </c>
-      <c r="C82" s="13">
+      <c r="C82" s="14">
         <f>C79</f>
         <v/>
       </c>
-      <c r="D82" s="13">
+      <c r="D82" s="14">
         <f>D79</f>
         <v/>
       </c>
-      <c r="E82" s="13">
+      <c r="E82" s="14">
         <f>E79</f>
         <v/>
       </c>
-      <c r="F82" s="13">
+      <c r="F82" s="14">
         <f>F79</f>
         <v/>
       </c>
-      <c r="G82" s="13">
+      <c r="G82" s="14">
         <f>G79</f>
         <v/>
       </c>
-      <c r="H82" s="13">
+      <c r="H82" s="14">
         <f>H79</f>
         <v/>
       </c>
-      <c r="I82" s="13">
+      <c r="I82" s="14">
         <f>I79</f>
         <v/>
       </c>
-      <c r="J82" s="13">
+      <c r="J82" s="14">
         <f>J79</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="14" t="inlineStr">
-        <is>
-          <t>RECONCILIATION TO DEAL BUCKETS  (Season 1; SPV = Making Cinderella)</t>
-        </is>
-      </c>
-      <c r="B84" s="15" t="n"/>
-      <c r="C84" s="15" t="n"/>
-      <c r="D84" s="15" t="n"/>
-      <c r="E84" s="15" t="n"/>
-      <c r="F84" s="15" t="n"/>
-      <c r="G84" s="15" t="n"/>
-      <c r="H84" s="15" t="n"/>
-      <c r="I84" s="15" t="n"/>
-      <c r="J84" s="15" t="n"/>
+      <c r="A84" s="15" t="inlineStr">
+        <is>
+          <t>RECONCILIATION TO DEAL BUCKETS  (SPV = Making Cinderella)</t>
+        </is>
+      </c>
+      <c r="B84" s="16" t="n"/>
+      <c r="C84" s="16" t="n"/>
+      <c r="D84" s="16" t="n"/>
+      <c r="E84" s="16" t="n"/>
+      <c r="F84" s="16" t="n"/>
+      <c r="G84" s="16" t="n"/>
+      <c r="H84" s="16" t="n"/>
+      <c r="I84" s="16" t="n"/>
+      <c r="J84" s="16" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="16" t="inlineStr"/>
-      <c r="B85" s="16" t="inlineStr">
-        <is>
-          <t>Bkt1 Cur</t>
-        </is>
-      </c>
-      <c r="C85" s="16" t="inlineStr">
-        <is>
-          <t>Bkt1 w/MC</t>
-        </is>
-      </c>
-      <c r="D85" s="16" t="inlineStr">
-        <is>
-          <t>Bkt1 Δ</t>
-        </is>
-      </c>
-      <c r="E85" s="16" t="inlineStr">
-        <is>
-          <t>SPV 80%×Δ</t>
-        </is>
-      </c>
-      <c r="F85" s="16" t="inlineStr">
-        <is>
-          <t>Struct(100% sch)</t>
-        </is>
-      </c>
-      <c r="G85" s="16" t="inlineStr">
-        <is>
-          <t>Donor w/MC</t>
-        </is>
-      </c>
-      <c r="H85" s="16" t="inlineStr">
-        <is>
-          <t>Instit. w/MC</t>
-        </is>
-      </c>
-      <c r="I85" s="16" t="inlineStr">
-        <is>
-          <t>NIL (memo)</t>
-        </is>
-      </c>
-      <c r="J85" s="16" t="inlineStr"/>
+      <c r="A85" s="17" t="inlineStr"/>
+      <c r="B85" s="17" t="inlineStr">
+        <is>
+          <t>B1 Cur</t>
+        </is>
+      </c>
+      <c r="C85" s="17" t="inlineStr">
+        <is>
+          <t>B1 Base</t>
+        </is>
+      </c>
+      <c r="D85" s="17" t="inlineStr">
+        <is>
+          <t>B1 Reach</t>
+        </is>
+      </c>
+      <c r="E85" s="17" t="inlineStr">
+        <is>
+          <t>SPV80% Base</t>
+        </is>
+      </c>
+      <c r="F85" s="17" t="inlineStr">
+        <is>
+          <t>SPV80% Reach</t>
+        </is>
+      </c>
+      <c r="G85" s="17" t="inlineStr">
+        <is>
+          <t>Struct (100% sch)</t>
+        </is>
+      </c>
+      <c r="H85" s="17" t="inlineStr">
+        <is>
+          <t>Donor Reach</t>
+        </is>
+      </c>
+      <c r="I85" s="17" t="inlineStr"/>
+      <c r="J85" s="17" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="17" t="inlineStr">
+      <c r="A86" s="18" t="inlineStr">
         <is>
           <t>St. Joseph's</t>
         </is>
       </c>
-      <c r="B86" s="18">
+      <c r="B86" s="19">
         <f>B12+B19+B36+B51+B58+B64</f>
         <v/>
       </c>
-      <c r="C86" s="18">
+      <c r="C86" s="19">
         <f>C12+C19+C36+C51+C58+C64</f>
         <v/>
       </c>
-      <c r="D86" s="18">
-        <f>(C12+C19+C36+C51+C58+C64)-(B12+B19+B36+B51+B58+B64)</f>
-        <v/>
-      </c>
-      <c r="E86" s="19">
-        <f>0.8*D86</f>
-        <v/>
-      </c>
-      <c r="F86" s="18">
-        <f>C26</f>
-        <v/>
-      </c>
-      <c r="G86" s="18">
-        <f>C44</f>
-        <v/>
-      </c>
-      <c r="H86" s="18">
-        <f>C73</f>
-        <v/>
-      </c>
-      <c r="I86" s="18">
-        <f>C79</f>
+      <c r="D86" s="19">
+        <f>D12+D19+D36+D51+D58+D64</f>
+        <v/>
+      </c>
+      <c r="E86" s="20">
+        <f>0.8*(C86-B86)</f>
+        <v/>
+      </c>
+      <c r="F86" s="21">
+        <f>0.8*(D86-B86)</f>
+        <v/>
+      </c>
+      <c r="G86" s="19">
+        <f>D26</f>
+        <v/>
+      </c>
+      <c r="H86" s="19">
+        <f>D44</f>
         <v/>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="17" t="inlineStr">
+      <c r="A87" s="18" t="inlineStr">
         <is>
           <t>Davidson</t>
         </is>
       </c>
-      <c r="B87" s="18">
+      <c r="B87" s="19">
         <f>E12+E19+E36+E51+E58+E64</f>
         <v/>
       </c>
-      <c r="C87" s="18">
+      <c r="C87" s="19">
         <f>F12+F19+F36+F51+F58+F64</f>
         <v/>
       </c>
-      <c r="D87" s="18">
-        <f>(F12+F19+F36+F51+F58+F64)-(E12+E19+E36+E51+E58+E64)</f>
-        <v/>
-      </c>
-      <c r="E87" s="19">
-        <f>0.8*D87</f>
-        <v/>
-      </c>
-      <c r="F87" s="18">
-        <f>F26</f>
-        <v/>
-      </c>
-      <c r="G87" s="18">
-        <f>F44</f>
-        <v/>
-      </c>
-      <c r="H87" s="18">
-        <f>F73</f>
-        <v/>
-      </c>
-      <c r="I87" s="18">
-        <f>F79</f>
+      <c r="D87" s="19">
+        <f>G12+G19+G36+G51+G58+G64</f>
+        <v/>
+      </c>
+      <c r="E87" s="20">
+        <f>0.8*(C87-B87)</f>
+        <v/>
+      </c>
+      <c r="F87" s="21">
+        <f>0.8*(D87-B87)</f>
+        <v/>
+      </c>
+      <c r="G87" s="19">
+        <f>G26</f>
+        <v/>
+      </c>
+      <c r="H87" s="19">
+        <f>G44</f>
         <v/>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="17" t="inlineStr">
+      <c r="A88" s="18" t="inlineStr">
         <is>
           <t>Hawaii</t>
         </is>
       </c>
-      <c r="B88" s="18">
+      <c r="B88" s="19">
         <f>H12+H19+H36+H51+H58+H64</f>
         <v/>
       </c>
-      <c r="C88" s="18">
+      <c r="C88" s="19">
         <f>I12+I19+I36+I51+I58+I64</f>
         <v/>
       </c>
-      <c r="D88" s="18">
-        <f>(I12+I19+I36+I51+I58+I64)-(H12+H19+H36+H51+H58+H64)</f>
-        <v/>
-      </c>
-      <c r="E88" s="19">
-        <f>0.8*D88</f>
-        <v/>
-      </c>
-      <c r="F88" s="18">
-        <f>I26</f>
-        <v/>
-      </c>
-      <c r="G88" s="18">
-        <f>I44</f>
-        <v/>
-      </c>
-      <c r="H88" s="18">
-        <f>I73</f>
-        <v/>
-      </c>
-      <c r="I88" s="18">
-        <f>I79</f>
+      <c r="D88" s="19">
+        <f>J12+J19+J36+J51+J58+J64</f>
+        <v/>
+      </c>
+      <c r="E88" s="20">
+        <f>0.8*(C88-B88)</f>
+        <v/>
+      </c>
+      <c r="F88" s="21">
+        <f>0.8*(D88-B88)</f>
+        <v/>
+      </c>
+      <c r="G88" s="19">
+        <f>J26</f>
+        <v/>
+      </c>
+      <c r="H88" s="19">
+        <f>J44</f>
         <v/>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="20" t="inlineStr">
+      <c r="A90" s="22" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
-      <c r="B90" s="21" t="n"/>
-      <c r="C90" s="21" t="n"/>
-      <c r="D90" s="21" t="n"/>
-      <c r="E90" s="21" t="n"/>
-      <c r="F90" s="21" t="n"/>
-      <c r="G90" s="21" t="n"/>
-      <c r="H90" s="21" t="n"/>
-      <c r="I90" s="21" t="n"/>
-      <c r="J90" s="21" t="n"/>
+      <c r="B90" s="23" t="n"/>
+      <c r="C90" s="23" t="n"/>
+      <c r="D90" s="23" t="n"/>
+      <c r="E90" s="23" t="n"/>
+      <c r="F90" s="23" t="n"/>
+      <c r="G90" s="23" t="n"/>
+      <c r="H90" s="23" t="n"/>
+      <c r="I90" s="23" t="n"/>
+      <c r="J90" s="23" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="22" t="inlineStr">
-        <is>
-          <t>Bucket 1 (commercial: Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps) is the rev-share base. School keeps its baseline (the 'Current' column); 80% of the increase → SPV, 20% → school.</t>
+      <c r="A91" s="24" t="inlineStr">
+        <is>
+          <t>Reach = full-attachment estimate (celebrity + Netflix + top-10 roster + deep tournament run all landing). Base = Current + a conservative fraction of that uplift (55-65% on commercial lines).</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="22" t="inlineStr">
-        <is>
-          <t>Structural (Conference &amp; NCAA distributions): 100% to the school. NCAA units spike with a deep tournament run but are conference-mediated/shared.</t>
+      <c r="A92" s="24" t="inlineStr">
+        <is>
+          <t>Bucket 1 (commercial: Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps) is the rev-share base. School keeps its baseline (Current); 80% of the increase over baseline -&gt; SPV, 20% -&gt; school.</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="22" t="inlineStr">
-        <is>
-          <t>Donor (Philanthropy): baseline stays 100% with the school; the MC-driven uplift is worked separately — conversion to SPV investment (capital) + 50/50 on the philanthropic remainder.</t>
+      <c r="A93" s="24" t="inlineStr">
+        <is>
+          <t>Structural (Conference &amp; NCAA): 100% to the school; NCAA units rise with a run but are conference-mediated/shared. Donor (Philanthropy): baseline stays with school; uplift worked separately (conversion to SPV investment + 50/50).</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="22" t="inlineStr">
-        <is>
-          <t>Institutional &amp; state support DECLINES with MC — the program self-funds, cutting subsidy reliance (a positive optics point for the AD).</t>
+      <c r="A94" s="24" t="inlineStr">
+        <is>
+          <t>Institutional &amp; state support DECLINES with MC (base declines half as far as reach) — the program self-funds. NIL (memo): athlete funding paid BY the SPV — a cost, not revenue.</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="22" t="inlineStr">
-        <is>
-          <t>NIL / rev-share (memo): athlete funding paid BY the SPV — a cost, not program revenue. Shown for completeness only.</t>
+      <c r="A95" s="24" t="inlineStr">
+        <is>
+          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, international + format. Roughly recoups the $15M SPV cost.</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="22" t="inlineStr">
-        <is>
-          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost = $4M margin), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, international + format windows. Roughly recoups the $15M SPV cost.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="22" t="inlineStr">
-        <is>
-          <t>Marquee-game relocation assumed: St. Joe's → Wells Fargo Center (19k); Davidson → Spectrum Center (19k); Hawaii carried by its 10,300 home arena + Diamond Head Classic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="22" t="inlineStr">
-        <is>
-          <t>All figures are ESTIMATES in $000s. This is the full-attachment ('reach') projection; a conservative base dials the With-MC commercial column down ~15-20%.</t>
+      <c r="A96" s="24" t="inlineStr">
+        <is>
+          <t>Marquee-game relocation assumed: St. Joe's -&gt; Wells Fargo Center (19k); Davidson -&gt; Spectrum Center (19k); Hawaii carried by its 10,300 arena + Diamond Head Classic. All figures ESTIMATES in $000s.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="10">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="A93:J93"/>
     <mergeCell ref="A94:J94"/>
-    <mergeCell ref="A97:J97"/>
     <mergeCell ref="A92:J92"/>
     <mergeCell ref="A91:J91"/>
     <mergeCell ref="A95:J95"/>
     <mergeCell ref="A96:J96"/>
     <mergeCell ref="H2:J2"/>
-    <mergeCell ref="A98:J98"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Scale down current MBB revenue estimates (0.42x) across all three schools
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -634,28 +634,28 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>700</v>
+        <v>290</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1380</v>
+        <v>1230</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>1800</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>900</v>
+        <v>380</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1710</v>
+        <v>1510</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>2200</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>1500</v>
+        <v>630</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>2430</v>
+        <v>2100</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>3000</v>
@@ -668,28 +668,28 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>400</v>
+        <v>170</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>2320</v>
+        <v>2230</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>3500</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>500</v>
+        <v>210</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>2360</v>
+        <v>2250</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>3500</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>700</v>
+        <v>290</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>1820</v>
+        <v>1660</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>2500</v>
@@ -702,28 +702,28 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>550</v>
+        <v>520</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>720</v>
+        <v>660</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>1000</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>670</v>
+        <v>610</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>900</v>
@@ -736,28 +736,28 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>500</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>350</v>
@@ -770,28 +770,28 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>360</v>
+        <v>330</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>500</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>400</v>
+        <v>360</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>550</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>550</v>
+        <v>480</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>700</v>
@@ -804,28 +804,28 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>300</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>350</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>270</v>
+        <v>240</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>350</v>
@@ -838,28 +838,28 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>340</v>
+        <v>320</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>500</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>420</v>
+        <v>390</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>600</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>370</v>
+        <v>330</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>500</v>
@@ -931,28 +931,28 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>500</v>
+        <v>210</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>530</v>
+        <v>410</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>550</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>500</v>
+        <v>210</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>530</v>
+        <v>410</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>550</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>330</v>
+        <v>260</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>350</v>
@@ -965,28 +965,28 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="D16" s="7" t="n">
         <v>250</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>300</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>200</v>
@@ -999,28 +999,28 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>450</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>350</v>
@@ -1033,28 +1033,28 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D18" s="7" t="n">
         <v>120</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>150</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>100</v>
@@ -1126,28 +1126,28 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>400</v>
+        <v>170</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>440</v>
+        <v>390</v>
       </c>
       <c r="D22" s="7" t="n">
         <v>450</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>400</v>
+        <v>170</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>440</v>
+        <v>390</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>450</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>290</v>
+        <v>260</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>300</v>
@@ -1160,25 +1160,25 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D23" s="7" t="n">
         <v>150</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>180</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I23" s="8" t="n">
         <v>100</v>
@@ -1194,28 +1194,28 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="C24" s="8" t="n">
-        <v>590</v>
+        <v>570</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>700</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>680</v>
+        <v>660</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>800</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I24" s="8" t="n">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>600</v>
@@ -1228,28 +1228,28 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C25" s="8" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>220</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>220</v>
       </c>
       <c r="H25" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="I25" s="8" t="n">
         <v>180</v>
-      </c>
-      <c r="I25" s="8" t="n">
-        <v>200</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>200</v>
@@ -1321,28 +1321,28 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="C29" s="8" t="n">
-        <v>600</v>
+        <v>530</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>680</v>
+        <v>600</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>900</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>400</v>
+        <v>170</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>640</v>
+        <v>550</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>800</v>
@@ -1355,28 +1355,28 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="C30" s="8" t="n">
-        <v>700</v>
+        <v>640</v>
       </c>
       <c r="D30" s="7" t="n">
         <v>1000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>840</v>
+        <v>770</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="I30" s="8" t="n">
-        <v>740</v>
+        <v>660</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1000</v>
@@ -1389,28 +1389,28 @@
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C31" s="8" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>200</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>300</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>250</v>
@@ -1423,28 +1423,28 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="C32" s="8" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="D32" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>320</v>
+        <v>290</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>450</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>300</v>
+        <v>260</v>
       </c>
       <c r="J32" s="7" t="n">
         <v>400</v>
@@ -1491,28 +1491,28 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C34" s="8" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D34" s="7" t="n">
         <v>150</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="G34" s="7" t="n">
         <v>180</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>120</v>
@@ -1525,28 +1525,28 @@
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C35" s="8" t="n">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>500</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>600</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>450</v>
@@ -1618,28 +1618,28 @@
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>600</v>
+        <v>250</v>
       </c>
       <c r="C39" s="8" t="n">
-        <v>930</v>
+        <v>770</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>900</v>
+        <v>380</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>1400</v>
+        <v>1160</v>
       </c>
       <c r="G39" s="7" t="n">
         <v>1800</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>500</v>
+        <v>210</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>780</v>
+        <v>640</v>
       </c>
       <c r="J39" s="7" t="n">
         <v>1000</v>
@@ -1652,28 +1652,28 @@
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="C40" s="8" t="n">
-        <v>580</v>
+        <v>500</v>
       </c>
       <c r="D40" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>500</v>
+        <v>210</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>880</v>
+        <v>750</v>
       </c>
       <c r="G40" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="I40" s="8" t="n">
-        <v>480</v>
+        <v>420</v>
       </c>
       <c r="J40" s="7" t="n">
         <v>700</v>
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C41" s="8" t="n">
-        <v>640</v>
+        <v>590</v>
       </c>
       <c r="D41" s="7" t="n">
         <v>1000</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>400</v>
+        <v>170</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>1500</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>560</v>
+        <v>520</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>900</v>
@@ -1720,28 +1720,28 @@
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="C42" s="8" t="n">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="D42" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>480</v>
+        <v>420</v>
       </c>
       <c r="G42" s="7" t="n">
         <v>700</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I42" s="8" t="n">
-        <v>320</v>
+        <v>290</v>
       </c>
       <c r="J42" s="7" t="n">
         <v>500</v>
@@ -1754,28 +1754,28 @@
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="C43" s="8" t="n">
-        <v>800</v>
+        <v>720</v>
       </c>
       <c r="D43" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>500</v>
+        <v>210</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>1050</v>
+        <v>920</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>1500</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>660</v>
+        <v>600</v>
       </c>
       <c r="J43" s="7" t="n">
         <v>1000</v>
@@ -1847,28 +1847,28 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="C47" s="8" t="n">
-        <v>520</v>
+        <v>460</v>
       </c>
       <c r="D47" s="7" t="n">
         <v>700</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>660</v>
+        <v>590</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>900</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="I47" s="8" t="n">
-        <v>380</v>
+        <v>330</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>500</v>
@@ -1881,28 +1881,28 @@
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C48" s="8" t="n">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="D48" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>390</v>
+        <v>370</v>
       </c>
       <c r="G48" s="7" t="n">
         <v>600</v>
       </c>
       <c r="H48" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I48" s="8" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="J48" s="7" t="n">
         <v>300</v>
@@ -1915,28 +1915,28 @@
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="C49" s="8" t="n">
-        <v>520</v>
+        <v>500</v>
       </c>
       <c r="D49" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>660</v>
+        <v>620</v>
       </c>
       <c r="G49" s="7" t="n">
         <v>1000</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>410</v>
+        <v>380</v>
       </c>
       <c r="J49" s="7" t="n">
         <v>600</v>
@@ -1949,28 +1949,28 @@
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C50" s="8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D50" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="G50" s="7" t="n">
         <v>150</v>
       </c>
       <c r="H50" s="7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="I50" s="8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J50" s="7" t="n">
         <v>80</v>
@@ -2042,28 +2042,28 @@
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="C54" s="8" t="n">
-        <v>490</v>
+        <v>420</v>
       </c>
       <c r="D54" s="7" t="n">
         <v>600</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>490</v>
+        <v>420</v>
       </c>
       <c r="G54" s="7" t="n">
         <v>600</v>
       </c>
       <c r="H54" s="7" t="n">
-        <v>400</v>
+        <v>170</v>
       </c>
       <c r="I54" s="8" t="n">
-        <v>460</v>
+        <v>370</v>
       </c>
       <c r="J54" s="7" t="n">
         <v>500</v>
@@ -2076,28 +2076,28 @@
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="C55" s="8" t="n">
-        <v>530</v>
+        <v>510</v>
       </c>
       <c r="D55" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>620</v>
+        <v>580</v>
       </c>
       <c r="G55" s="7" t="n">
         <v>900</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="I55" s="8" t="n">
-        <v>550</v>
+        <v>480</v>
       </c>
       <c r="J55" s="7" t="n">
         <v>700</v>
@@ -2110,28 +2110,28 @@
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="C56" s="8" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="D56" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="F56" s="8" t="n">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="G56" s="7" t="n">
         <v>500</v>
       </c>
       <c r="H56" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="I56" s="8" t="n">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="J56" s="7" t="n">
         <v>400</v>
@@ -2144,7 +2144,7 @@
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C57" s="8" t="n">
         <v>70</v>
@@ -2153,19 +2153,19 @@
         <v>100</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F57" s="8" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G57" s="7" t="n">
         <v>120</v>
       </c>
       <c r="H57" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I57" s="8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>80</v>
@@ -2237,28 +2237,28 @@
         </is>
       </c>
       <c r="B61" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="C61" s="8" t="n">
-        <v>310</v>
+        <v>280</v>
       </c>
       <c r="D61" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="F61" s="8" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="G61" s="7" t="n">
         <v>500</v>
       </c>
       <c r="H61" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="I61" s="8" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>350</v>
@@ -2271,28 +2271,28 @@
         </is>
       </c>
       <c r="B62" s="7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="C62" s="8" t="n">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="D62" s="7" t="n">
         <v>200</v>
       </c>
       <c r="E62" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="G62" s="7" t="n">
         <v>250</v>
       </c>
       <c r="H62" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="I62" s="8" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="J62" s="7" t="n">
         <v>150</v>
@@ -2305,28 +2305,28 @@
         </is>
       </c>
       <c r="B63" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C63" s="8" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D63" s="7" t="n">
         <v>150</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F63" s="8" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="G63" s="7" t="n">
         <v>180</v>
       </c>
       <c r="H63" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I63" s="8" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>250</v>
@@ -2398,28 +2398,28 @@
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>800</v>
+        <v>340</v>
       </c>
       <c r="C67" s="8" t="n">
-        <v>600</v>
+        <v>370</v>
       </c>
       <c r="D67" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>600</v>
+        <v>250</v>
       </c>
       <c r="F67" s="8" t="n">
-        <v>450</v>
+        <v>280</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>300</v>
       </c>
       <c r="H67" s="7" t="n">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="I67" s="8" t="n">
-        <v>950</v>
+        <v>600</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>700</v>
@@ -2432,28 +2432,28 @@
         </is>
       </c>
       <c r="B68" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C68" s="8" t="n">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="D68" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="F68" s="8" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="G68" s="7" t="n">
         <v>50</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>600</v>
+        <v>250</v>
       </c>
       <c r="I68" s="8" t="n">
-        <v>500</v>
+        <v>320</v>
       </c>
       <c r="J68" s="7" t="n">
         <v>400</v>
@@ -2484,10 +2484,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>800</v>
+        <v>340</v>
       </c>
       <c r="I69" s="8" t="n">
-        <v>700</v>
+        <v>470</v>
       </c>
       <c r="J69" s="7" t="n">
         <v>600</v>
@@ -2500,28 +2500,28 @@
         </is>
       </c>
       <c r="B70" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="C70" s="8" t="n">
         <v>100</v>
-      </c>
-      <c r="C70" s="8" t="n">
-        <v>120</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>150</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>350</v>
+        <v>260</v>
       </c>
       <c r="G70" s="7" t="n">
         <v>400</v>
       </c>
       <c r="H70" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="I70" s="8" t="n">
         <v>50</v>
-      </c>
-      <c r="I70" s="8" t="n">
-        <v>60</v>
       </c>
       <c r="J70" s="7" t="n">
         <v>80</v>
@@ -2534,28 +2534,28 @@
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C71" s="8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D71" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="G71" s="7" t="n">
         <v>150</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="I71" s="8" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="J71" s="7" t="n">
         <v>120</v>
@@ -2568,28 +2568,28 @@
         </is>
       </c>
       <c r="B72" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C72" s="8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G72" s="7" t="n">
         <v>120</v>
       </c>
       <c r="H72" s="7" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="I72" s="8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="J72" s="7" t="n">
         <v>100</v>
@@ -2661,28 +2661,28 @@
         </is>
       </c>
       <c r="B76" s="7" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C76" s="8" t="n">
-        <v>2020</v>
+        <v>1980</v>
       </c>
       <c r="D76" s="7" t="n">
         <v>3000</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>400</v>
+        <v>170</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>2420</v>
+        <v>2330</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>3500</v>
       </c>
       <c r="H76" s="7" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="I76" s="8" t="n">
-        <v>1680</v>
+        <v>1650</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>2500</v>
@@ -2695,25 +2695,25 @@
         </is>
       </c>
       <c r="B77" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C77" s="8" t="n">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="D77" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>680</v>
+        <v>660</v>
       </c>
       <c r="G77" s="7" t="n">
         <v>1000</v>
       </c>
       <c r="H77" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I77" s="8" t="n">
         <v>400</v>

</xml_diff>

<commit_message>
Simplify SPV mechanic: single lump baseline (total current revenue) subtracted once, 80/20 above
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -146,7 +146,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2802,7 +2802,7 @@
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
         <is>
-          <t>PROGRAM REVENUE  (categories 1–9, excl. NIL)</t>
+          <t>PROGRAM REVENUE  (categories 1–9, excl. NIL)  = the total baseline</t>
         </is>
       </c>
       <c r="B81" s="12">
@@ -2888,7 +2888,7 @@
     <row r="84">
       <c r="A84" s="15" t="inlineStr">
         <is>
-          <t>RECONCILIATION TO DEAL BUCKETS  (SPV = Making Cinderella)</t>
+          <t>SPV ECONOMICS  (Bucket 1 above baseline, 80/20; baseline = total current revenue, one lump)</t>
         </is>
       </c>
       <c r="B84" s="16" t="n"/>
@@ -2901,41 +2901,41 @@
       <c r="I84" s="16" t="n"/>
       <c r="J84" s="16" t="n"/>
     </row>
-    <row r="85">
+    <row r="85" ht="26" customHeight="1">
       <c r="A85" s="17" t="inlineStr"/>
       <c r="B85" s="17" t="inlineStr">
         <is>
-          <t>B1 Cur</t>
+          <t>Baseline (total curr.)</t>
         </is>
       </c>
       <c r="C85" s="17" t="inlineStr">
         <is>
-          <t>B1 Base</t>
+          <t>Bucket 1 Base w/MC</t>
         </is>
       </c>
       <c r="D85" s="17" t="inlineStr">
         <is>
-          <t>B1 Reach</t>
+          <t>Bucket 1 Reach w/MC</t>
         </is>
       </c>
       <c r="E85" s="17" t="inlineStr">
         <is>
-          <t>SPV80% Base</t>
+          <t>SPV 80% Base</t>
         </is>
       </c>
       <c r="F85" s="17" t="inlineStr">
         <is>
-          <t>SPV80% Reach</t>
+          <t>SPV 80% Reach</t>
         </is>
       </c>
       <c r="G85" s="17" t="inlineStr">
         <is>
-          <t>Struct (100% sch)</t>
+          <t>School keeps Base</t>
         </is>
       </c>
       <c r="H85" s="17" t="inlineStr">
         <is>
-          <t>Donor Reach</t>
+          <t>School keeps Reach</t>
         </is>
       </c>
       <c r="I85" s="17" t="inlineStr"/>
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="B86" s="19">
-        <f>B12+B19+B36+B51+B58+B64</f>
+        <f>B81</f>
         <v/>
       </c>
       <c r="C86" s="19">
@@ -2968,11 +2968,11 @@
         <v/>
       </c>
       <c r="G86" s="19">
-        <f>D26</f>
+        <f>B86+0.2*(C86-B86)</f>
         <v/>
       </c>
       <c r="H86" s="19">
-        <f>D44</f>
+        <f>B86+0.2*(D86-B86)</f>
         <v/>
       </c>
     </row>
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="B87" s="19">
-        <f>E12+E19+E36+E51+E58+E64</f>
+        <f>E81</f>
         <v/>
       </c>
       <c r="C87" s="19">
@@ -3003,11 +3003,11 @@
         <v/>
       </c>
       <c r="G87" s="19">
-        <f>G26</f>
+        <f>B87+0.2*(C87-B87)</f>
         <v/>
       </c>
       <c r="H87" s="19">
-        <f>G44</f>
+        <f>B87+0.2*(D87-B87)</f>
         <v/>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="B88" s="19">
-        <f>H12+H19+H36+H51+H58+H64</f>
+        <f>H81</f>
         <v/>
       </c>
       <c r="C88" s="19">
@@ -3038,11 +3038,11 @@
         <v/>
       </c>
       <c r="G88" s="19">
-        <f>J26</f>
+        <f>B88+0.2*(C88-B88)</f>
         <v/>
       </c>
       <c r="H88" s="19">
-        <f>J44</f>
+        <f>B88+0.2*(D88-B88)</f>
         <v/>
       </c>
     </row>
@@ -3072,14 +3072,14 @@
     <row r="92">
       <c r="A92" s="24" t="inlineStr">
         <is>
-          <t>Bucket 1 (commercial: Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps) is the rev-share base. School keeps its baseline (Current); 80% of the increase over baseline -&gt; SPV, 20% -&gt; school.</t>
+          <t>MECHANIC (simplified): baseline = the school's TOTAL current program revenue (one lump, the green PROGRAM REVENUE row). The school keeps the first [baseline] dollars; everything in Bucket 1 above the baseline splits 80/20 (SPV 80, school 20). Not itemized line-by-line.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="24" t="inlineStr">
         <is>
-          <t>Structural (Conference &amp; NCAA): 100% to the school; NCAA units rise with a run but are conference-mediated/shared. Donor (Philanthropy): baseline stays with school; uplift worked separately (conversion to SPV investment + 50/50).</t>
+          <t>Bucket 1 = the school's commercial revenue with MC (Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps). SPV 80% = 0.8 x (Bucket 1 w/MC - total baseline). School keeps baseline + 20% of the excess.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hold fixed structural conference/NCAA lines flat; correct conference media baselines
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -931,31 +931,31 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>210</v>
+        <v>450</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>410</v>
+        <v>450</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>550</v>
+        <v>450</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>210</v>
+        <v>450</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>410</v>
+        <v>450</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>550</v>
+        <v>450</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>130</v>
+        <v>250</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16">
@@ -1122,35 +1122,35 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Conference revenue distribution</t>
+          <t xml:space="preserve">   Conference revenue distribution (non-media share)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>170</v>
+        <v>350</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>390</v>
+        <v>350</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>170</v>
+        <v>350</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>390</v>
+        <v>350</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>260</v>
+        <v>200</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23">
@@ -1160,31 +1160,31 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>180</v>
+        <v>80</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24">
@@ -1228,31 +1228,31 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>80</v>
+        <v>210</v>
       </c>
       <c r="C25" s="8" t="n">
+        <v>210</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>210</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="H25" s="7" t="n">
         <v>190</v>
       </c>
-      <c r="D25" s="7" t="n">
-        <v>220</v>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="F25" s="8" t="n">
+      <c r="I25" s="8" t="n">
         <v>190</v>
       </c>
-      <c r="G25" s="7" t="n">
-        <v>220</v>
-      </c>
-      <c r="H25" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="I25" s="8" t="n">
-        <v>180</v>
-      </c>
       <c r="J25" s="7" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
Lower current-scale factor to 0.33 so all-in baselines land in $3-4M
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -634,28 +634,28 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>290</v>
+        <v>230</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1230</v>
+        <v>1200</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>1800</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1510</v>
+        <v>1480</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>2200</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>630</v>
+        <v>500</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>2100</v>
+        <v>2050</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>3000</v>
@@ -668,28 +668,28 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>2230</v>
+        <v>2220</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>3500</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>210</v>
+        <v>160</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>2250</v>
+        <v>2230</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>3500</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>290</v>
+        <v>230</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>1660</v>
+        <v>1640</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>2500</v>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>520</v>
@@ -711,19 +711,19 @@
         <v>800</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>660</v>
+        <v>650</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>1000</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>610</v>
+        <v>600</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>900</v>
@@ -745,7 +745,7 @@
         <v>400</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>320</v>
@@ -754,7 +754,7 @@
         <v>500</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I8" s="8" t="n">
         <v>220</v>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>330</v>
@@ -779,7 +779,7 @@
         <v>500</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>360</v>
@@ -788,10 +788,10 @@
         <v>550</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>480</v>
+        <v>470</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>700</v>
@@ -804,10 +804,10 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>300</v>
@@ -822,7 +822,7 @@
         <v>350</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I10" s="8" t="n">
         <v>240</v>
@@ -847,7 +847,7 @@
         <v>500</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F11" s="8" t="n">
         <v>390</v>
@@ -856,7 +856,7 @@
         <v>600</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I11" s="8" t="n">
         <v>330</v>
@@ -974,7 +974,7 @@
         <v>250</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>190</v>
@@ -1017,10 +1017,10 @@
         <v>450</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>350</v>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>80</v>
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C24" s="8" t="n">
         <v>570</v>
@@ -1203,16 +1203,16 @@
         <v>700</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>660</v>
+        <v>650</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>800</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I24" s="8" t="n">
         <v>490</v>
@@ -1321,28 +1321,28 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="C29" s="8" t="n">
-        <v>530</v>
+        <v>520</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>900</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>550</v>
+        <v>530</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>800</v>
@@ -1355,28 +1355,28 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C30" s="8" t="n">
-        <v>640</v>
+        <v>630</v>
       </c>
       <c r="D30" s="7" t="n">
         <v>1000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>770</v>
+        <v>760</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="I30" s="8" t="n">
-        <v>660</v>
+        <v>650</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1000</v>
@@ -1407,10 +1407,10 @@
         <v>300</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>250</v>
@@ -1423,16 +1423,16 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C32" s="8" t="n">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="D32" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>290</v>
@@ -1441,7 +1441,7 @@
         <v>450</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I32" s="8" t="n">
         <v>260</v>
@@ -1491,10 +1491,10 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C34" s="8" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D34" s="7" t="n">
         <v>150</v>
@@ -1509,7 +1509,7 @@
         <v>180</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I34" s="8" t="n">
         <v>80</v>
@@ -1534,10 +1534,10 @@
         <v>500</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>600</v>
@@ -1618,28 +1618,28 @@
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="C39" s="8" t="n">
-        <v>770</v>
+        <v>750</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>1160</v>
+        <v>1120</v>
       </c>
       <c r="G39" s="7" t="n">
         <v>1800</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>210</v>
+        <v>160</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>640</v>
+        <v>620</v>
       </c>
       <c r="J39" s="7" t="n">
         <v>1000</v>
@@ -1652,25 +1652,25 @@
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="C40" s="8" t="n">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="D40" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>210</v>
+        <v>160</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>750</v>
+        <v>730</v>
       </c>
       <c r="G40" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I40" s="8" t="n">
         <v>420</v>
@@ -1686,25 +1686,25 @@
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C41" s="8" t="n">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="D41" s="7" t="n">
         <v>1000</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>900</v>
+        <v>880</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>1500</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I41" s="8" t="n">
         <v>520</v>
@@ -1720,16 +1720,16 @@
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C42" s="8" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="D42" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F42" s="8" t="n">
         <v>420</v>
@@ -1738,7 +1738,7 @@
         <v>700</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I42" s="8" t="n">
         <v>290</v>
@@ -1754,28 +1754,28 @@
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="C43" s="8" t="n">
-        <v>720</v>
+        <v>700</v>
       </c>
       <c r="D43" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>210</v>
+        <v>160</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>920</v>
+        <v>900</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>1500</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="J43" s="7" t="n">
         <v>1000</v>
@@ -1847,25 +1847,25 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C47" s="8" t="n">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="D47" s="7" t="n">
         <v>700</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>900</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I47" s="8" t="n">
         <v>330</v>
@@ -1881,10 +1881,10 @@
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C48" s="8" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="D48" s="7" t="n">
         <v>400</v>
@@ -1899,10 +1899,10 @@
         <v>600</v>
       </c>
       <c r="H48" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I48" s="8" t="n">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="J48" s="7" t="n">
         <v>300</v>
@@ -1915,16 +1915,16 @@
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C49" s="8" t="n">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="D49" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F49" s="8" t="n">
         <v>620</v>
@@ -1933,7 +1933,7 @@
         <v>1000</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I49" s="8" t="n">
         <v>380</v>
@@ -1958,10 +1958,10 @@
         <v>100</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G50" s="7" t="n">
         <v>150</v>
@@ -2042,28 +2042,28 @@
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="C54" s="8" t="n">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="D54" s="7" t="n">
         <v>600</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="G54" s="7" t="n">
         <v>600</v>
       </c>
       <c r="H54" s="7" t="n">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="I54" s="8" t="n">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="J54" s="7" t="n">
         <v>500</v>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C55" s="8" t="n">
         <v>510</v>
@@ -2085,7 +2085,7 @@
         <v>800</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F55" s="8" t="n">
         <v>580</v>
@@ -2094,10 +2094,10 @@
         <v>900</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="I55" s="8" t="n">
-        <v>480</v>
+        <v>470</v>
       </c>
       <c r="J55" s="7" t="n">
         <v>700</v>
@@ -2119,16 +2119,16 @@
         <v>400</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F56" s="8" t="n">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="G56" s="7" t="n">
         <v>500</v>
       </c>
       <c r="H56" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I56" s="8" t="n">
         <v>270</v>
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="B61" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C61" s="8" t="n">
         <v>280</v>
@@ -2246,7 +2246,7 @@
         <v>400</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F61" s="8" t="n">
         <v>350</v>
@@ -2255,10 +2255,10 @@
         <v>500</v>
       </c>
       <c r="H61" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I61" s="8" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>350</v>
@@ -2280,19 +2280,19 @@
         <v>200</v>
       </c>
       <c r="E62" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="G62" s="7" t="n">
         <v>250</v>
       </c>
       <c r="H62" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="I62" s="8" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="J62" s="7" t="n">
         <v>150</v>
@@ -2314,19 +2314,19 @@
         <v>150</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F63" s="8" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="G63" s="7" t="n">
         <v>180</v>
       </c>
       <c r="H63" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I63" s="8" t="n">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>250</v>
@@ -2398,28 +2398,28 @@
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>340</v>
+        <v>260</v>
       </c>
       <c r="C67" s="8" t="n">
-        <v>370</v>
+        <v>330</v>
       </c>
       <c r="D67" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E67" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="F67" s="8" t="n">
         <v>250</v>
-      </c>
-      <c r="F67" s="8" t="n">
-        <v>280</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>300</v>
       </c>
       <c r="H67" s="7" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="I67" s="8" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>700</v>
@@ -2432,16 +2432,16 @@
         </is>
       </c>
       <c r="B68" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="C68" s="8" t="n">
         <v>80</v>
-      </c>
-      <c r="C68" s="8" t="n">
-        <v>90</v>
       </c>
       <c r="D68" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F68" s="8" t="n">
         <v>40</v>
@@ -2450,10 +2450,10 @@
         <v>50</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="I68" s="8" t="n">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="J68" s="7" t="n">
         <v>400</v>
@@ -2484,10 +2484,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>340</v>
+        <v>260</v>
       </c>
       <c r="I69" s="8" t="n">
-        <v>470</v>
+        <v>430</v>
       </c>
       <c r="J69" s="7" t="n">
         <v>600</v>
@@ -2500,19 +2500,19 @@
         </is>
       </c>
       <c r="B70" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C70" s="8" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>150</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="G70" s="7" t="n">
         <v>400</v>
@@ -2552,10 +2552,10 @@
         <v>150</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="I71" s="8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J71" s="7" t="n">
         <v>120</v>
@@ -2577,16 +2577,16 @@
         <v>100</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G72" s="7" t="n">
         <v>120</v>
       </c>
       <c r="H72" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="I72" s="8" t="n">
         <v>60</v>
@@ -2661,28 +2661,28 @@
         </is>
       </c>
       <c r="B76" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C76" s="8" t="n">
-        <v>1980</v>
+        <v>1970</v>
       </c>
       <c r="D76" s="7" t="n">
         <v>3000</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>2330</v>
+        <v>2320</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>3500</v>
       </c>
       <c r="H76" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I76" s="8" t="n">
-        <v>1650</v>
+        <v>1640</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>2500</v>
@@ -2704,7 +2704,7 @@
         <v>800</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F77" s="8" t="n">
         <v>660</v>
@@ -2713,10 +2713,10 @@
         <v>1000</v>
       </c>
       <c r="H77" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I77" s="8" t="n">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>600</v>

</xml_diff>

<commit_message>
Apply revenue-line corrections: cut postseason gate, MMR-constrain Bkt1 sponsorship, flat apparel, NIL memo reframe
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>1200</v>
@@ -643,19 +643,19 @@
         <v>1800</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1480</v>
+        <v>1470</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>2200</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>500</v>
+        <v>450</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>2050</v>
+        <v>2030</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>3000</v>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>2220</v>
@@ -677,7 +677,7 @@
         <v>3500</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>2230</v>
@@ -686,10 +686,10 @@
         <v>3500</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>1640</v>
+        <v>1630</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>2500</v>
@@ -702,10 +702,10 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>520</v>
+        <v>510</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>800</v>
@@ -720,10 +720,10 @@
         <v>1000</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>900</v>
@@ -732,35 +732,35 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Postseason ticket revenue (conf tourn/NCAA)</t>
+          <t xml:space="preserve">   Postseason ticket (allotment margin — conf/NCAA keep the gate)</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
         <v>10</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>250</v>
+        <v>40</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>400</v>
+        <v>60</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>20</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>320</v>
+        <v>60</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>500</v>
+        <v>80</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>10</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>220</v>
+        <v>30</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>350</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -779,7 +779,7 @@
         <v>500</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>360</v>
@@ -788,7 +788,7 @@
         <v>550</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="I9" s="8" t="n">
         <v>470</v>
@@ -813,19 +813,19 @@
         <v>300</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>350</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>350</v>
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C11" s="8" t="n">
         <v>320</v>
@@ -856,7 +856,7 @@
         <v>600</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I11" s="8" t="n">
         <v>330</v>
@@ -983,7 +983,7 @@
         <v>300</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="I16" s="8" t="n">
         <v>130</v>
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C24" s="8" t="n">
         <v>570</v>
@@ -1203,7 +1203,7 @@
         <v>700</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>650</v>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C29" s="8" t="n">
         <v>520</v>
@@ -1330,16 +1330,16 @@
         <v>800</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>900</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="I29" s="8" t="n">
         <v>530</v>
@@ -1351,35 +1351,35 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Corporate / category sponsorships</t>
+          <t xml:space="preserve">   Corporate / category sponsorships (school)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
         <v>80</v>
       </c>
       <c r="C30" s="8" t="n">
-        <v>630</v>
+        <v>450</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>1000</v>
+        <v>700</v>
       </c>
       <c r="E30" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F30" s="8" t="n">
+        <v>550</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>850</v>
+      </c>
+      <c r="H30" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="F30" s="8" t="n">
-        <v>760</v>
-      </c>
-      <c r="G30" s="7" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H30" s="7" t="n">
-        <v>120</v>
-      </c>
       <c r="I30" s="8" t="n">
-        <v>650</v>
+        <v>460</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>1000</v>
+        <v>700</v>
       </c>
     </row>
     <row r="31">
@@ -1398,7 +1398,7 @@
         <v>200</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F31" s="8" t="n">
         <v>190</v>
@@ -1426,62 +1426,62 @@
         <v>30</v>
       </c>
       <c r="C32" s="8" t="n">
-        <v>250</v>
+        <v>190</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>40</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>290</v>
+        <v>230</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>260</v>
+        <v>200</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Jersey patch / uniform sponsorship</t>
+          <t xml:space="preserve">   Jersey patch (school; national patch = Bkt2)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C33" s="8" t="n">
-        <v>480</v>
+        <v>90</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>800</v>
+        <v>150</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>420</v>
+        <v>70</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>700</v>
+        <v>120</v>
       </c>
     </row>
     <row r="34">
@@ -1521,35 +1521,35 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Digital &amp; social sponsorship / content</t>
+          <t xml:space="preserve">   Digital &amp; social sponsorship (national = Bkt2)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
         <v>10</v>
       </c>
       <c r="C35" s="8" t="n">
-        <v>300</v>
+        <v>90</v>
       </c>
       <c r="D35" s="7" t="n">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>10</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>360</v>
+        <v>120</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>10</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>270</v>
+        <v>80</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>450</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36">
@@ -1618,25 +1618,25 @@
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="C39" s="8" t="n">
-        <v>750</v>
+        <v>740</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>1200</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>1120</v>
+        <v>1110</v>
       </c>
       <c r="G39" s="7" t="n">
         <v>1800</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="I39" s="8" t="n">
         <v>620</v>
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C40" s="8" t="n">
-        <v>490</v>
+        <v>480</v>
       </c>
       <c r="D40" s="7" t="n">
         <v>800</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="F40" s="8" t="n">
         <v>730</v>
@@ -1670,10 +1670,10 @@
         <v>1200</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I40" s="8" t="n">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="J40" s="7" t="n">
         <v>700</v>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C41" s="8" t="n">
         <v>580</v>
@@ -1695,7 +1695,7 @@
         <v>1000</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F41" s="8" t="n">
         <v>880</v>
@@ -1704,10 +1704,10 @@
         <v>1500</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>520</v>
+        <v>510</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>900</v>
@@ -1729,10 +1729,10 @@
         <v>400</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="G42" s="7" t="n">
         <v>700</v>
@@ -1754,7 +1754,7 @@
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C43" s="8" t="n">
         <v>700</v>
@@ -1763,10 +1763,10 @@
         <v>1200</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>900</v>
+        <v>890</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>1500</v>
@@ -1847,31 +1847,31 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="C47" s="8" t="n">
-        <v>450</v>
+        <v>200</v>
       </c>
       <c r="D47" s="7" t="n">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>580</v>
+        <v>300</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="I47" s="8" t="n">
-        <v>330</v>
+        <v>150</v>
       </c>
       <c r="J47" s="7" t="n">
-        <v>500</v>
+        <v>150</v>
       </c>
     </row>
     <row r="48">
@@ -1890,7 +1890,7 @@
         <v>400</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F48" s="8" t="n">
         <v>370</v>
@@ -1924,7 +1924,7 @@
         <v>800</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F49" s="8" t="n">
         <v>620</v>
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C54" s="8" t="n">
         <v>410</v>
@@ -2051,7 +2051,7 @@
         <v>600</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F54" s="8" t="n">
         <v>410</v>
@@ -2060,7 +2060,7 @@
         <v>600</v>
       </c>
       <c r="H54" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="I54" s="8" t="n">
         <v>360</v>
@@ -2085,16 +2085,16 @@
         <v>800</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>580</v>
+        <v>570</v>
       </c>
       <c r="G55" s="7" t="n">
         <v>900</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="I55" s="8" t="n">
         <v>470</v>
@@ -2110,7 +2110,7 @@
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C56" s="8" t="n">
         <v>260</v>
@@ -2128,10 +2128,10 @@
         <v>500</v>
       </c>
       <c r="H56" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I56" s="8" t="n">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="J56" s="7" t="n">
         <v>400</v>
@@ -2237,16 +2237,16 @@
         </is>
       </c>
       <c r="B61" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C61" s="8" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="D61" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F61" s="8" t="n">
         <v>350</v>
@@ -2255,7 +2255,7 @@
         <v>500</v>
       </c>
       <c r="H61" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I61" s="8" t="n">
         <v>240</v>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="B62" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C62" s="8" t="n">
         <v>140</v>
@@ -2398,28 +2398,28 @@
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="C67" s="8" t="n">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="D67" s="7" t="n">
         <v>400</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="F67" s="8" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>300</v>
       </c>
       <c r="H67" s="7" t="n">
-        <v>400</v>
+        <v>360</v>
       </c>
       <c r="I67" s="8" t="n">
-        <v>550</v>
+        <v>530</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>700</v>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="B68" s="7" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C68" s="8" t="n">
         <v>80</v>
@@ -2450,10 +2450,10 @@
         <v>50</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="I68" s="8" t="n">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="J68" s="7" t="n">
         <v>400</v>
@@ -2484,10 +2484,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="I69" s="8" t="n">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="J69" s="7" t="n">
         <v>600</v>
@@ -2509,10 +2509,10 @@
         <v>150</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="G70" s="7" t="n">
         <v>400</v>
@@ -2543,10 +2543,10 @@
         <v>100</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G71" s="7" t="n">
         <v>150</v>
@@ -2641,7 +2641,7 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>NIL / revenue-share era  (memo — cost-side funding, not program revenue)</t>
+          <t>NIL / rev-share era  (memo — NOT program revenue; see per-line notes)</t>
         </is>
       </c>
       <c r="B75" s="6" t="n"/>
@@ -2657,41 +2657,41 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">   NIL collective revenue (third-party)</t>
+          <t xml:space="preserve">   Third-party athlete NIL income (memo — athletes' own $, not SPV rev/cost)</t>
         </is>
       </c>
       <c r="B76" s="7" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="C76" s="8" t="n">
-        <v>1970</v>
+        <v>990</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>130</v>
+        <v>40</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>2320</v>
+        <v>1310</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="H76" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="I76" s="8" t="n">
-        <v>1640</v>
+        <v>660</v>
       </c>
       <c r="J76" s="7" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Athlete marketing / activation revenue</t>
+          <t xml:space="preserve">   Athlete marketing / activation (SPV-produced = Bucket 2)</t>
         </is>
       </c>
       <c r="B77" s="7" t="n">
@@ -2725,7 +2725,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">   House-settlement revenue-share pool</t>
+          <t xml:space="preserve">   House-settlement rev-share pool (SPV-funded roster COST)</t>
         </is>
       </c>
       <c r="B78" s="7" t="n">
@@ -2759,7 +2759,7 @@
     <row r="79">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Subtotal — NIL / revenue-share era</t>
+          <t xml:space="preserve">   Subtotal — NIL / rev-share era</t>
         </is>
       </c>
       <c r="B79" s="10">
@@ -3086,35 +3086,67 @@
     <row r="94">
       <c r="A94" s="24" t="inlineStr">
         <is>
-          <t>Institutional &amp; state support DECLINES with MC (base declines half as far as reach) — the program self-funds. NIL (memo): athlete funding paid BY the SPV — a cost, not revenue.</t>
+          <t>Postseason gate: conf tournament &amp; NCAA tournament ticket revenue goes to the CONFERENCE / NCAA, not the school — line reduced to a small allotment margin only.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="24" t="inlineStr">
         <is>
-          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, international + format. Roughly recoups the $15M SPV cost.</t>
+          <t>Concessions &amp; parking DO grow: marquee home games are relocated to big arenas (St. Joe's -&gt; Xfinity Mobile Arena) where the school is the home promoter and keeps/splits the ancillaries.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="24" t="inlineStr">
         <is>
-          <t>Marquee-game relocation assumed: St. Joe's -&gt; Wells Fargo Center (19k); Davidson -&gt; Spectrum Center (19k); Hawaii carried by its 10,300 arena + Diamond Head Classic. All figures ESTIMATES in $000s.</t>
+          <t>MMR constraint (Learfield/Playfly own school inventory): Bucket 1 sponsorship kept modest. National / Netflix-grade sponsor + patch = SPV IP (Bucket 2, off this sheet), not school MMR inventory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="24" t="inlineStr">
+        <is>
+          <t>Apparel shoe contract held FLAT — multi-year locked deal, no mid-term jump (renewal upside later). Licensing/merch/retail still grow (flexible).</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="24" t="inlineStr">
+        <is>
+          <t>NIL memo lines are NOT program revenue: (1) third-party athlete NIL income = athletes' own earnings (a recruiting benefit, not SPV rev/cost); (2) athlete marketing/activation = SPV-produced Bucket 2; (3) House rev-share pool = SPV-funded roster COST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="24" t="inlineStr">
+        <is>
+          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, athlete-marketing/activation, international + format. Roughly recoups the $15M SPV cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="24" t="inlineStr">
+        <is>
+          <t>Marquee-game relocation assumed: St. Joe's -&gt; Xfinity Mobile Arena (19k); Davidson -&gt; Spectrum Center (19k); Hawaii carried by its 10,300 arena + Diamond Head Classic. All figures ESTIMATES in $000s.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="14">
+    <mergeCell ref="A99:J99"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="A93:J93"/>
     <mergeCell ref="A94:J94"/>
+    <mergeCell ref="A97:J97"/>
+    <mergeCell ref="A100:J100"/>
     <mergeCell ref="A92:J92"/>
     <mergeCell ref="A91:J91"/>
     <mergeCell ref="A95:J95"/>
     <mergeCell ref="A96:J96"/>
     <mergeCell ref="H2:J2"/>
+    <mergeCell ref="A98:J98"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Bucket 2 (SPV) tab: series/live/sponsor economics + MC-originated sponsorship (85%), full SPV picture
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Three-School Projection" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bucket 2 (SPV)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;–&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +57,11 @@
     <font>
       <i val="1"/>
       <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -155,6 +161,8 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3151,4 +3159,404 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bucket 2 — SPV-only revenue (100% SPV, off the school sheet)   ($000s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Streaming series (10 hrs @ $1.0M sold / $0.6M cost)</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>$400k/hr margin before intl/format</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   International + format windows</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>durable franchise asset; grows w/ library</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Live games (3 @ &gt;$1.0M rev / $0.3M cost each)</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>2100</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>school-owned neutral/non-conf games</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   National presenting sponsor + premium patch</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>priced off Netflix eyeballs; SPV IP, not school MMR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MC-originated sponsorship (signage/MMR-scope, ~85% SPV)</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>MC sources it, keeps ~85% via originator deal; Learfield ~15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Content engine / athlete marketing &amp; activation</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>500</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>SPV-produced branded content; players' NIL contracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Bucket 2 total (SPV)</t>
+        </is>
+      </c>
+      <c r="B10" s="10">
+        <f>SUM(B4:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="10">
+        <f>SUM(C4:C9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>FULL SPV PICTURE — single season  (Bucket 1 share + Bucket 2 − $15M SPV cost)</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n"/>
+      <c r="C12" s="16" t="n"/>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="16" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Bkt1 SPV Base</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>+ Bkt2 Base</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>− SPV cost</t>
+        </is>
+      </c>
+      <c r="E13" s="17">
+        <f> SPV net Base</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>St. Joseph's</t>
+        </is>
+      </c>
+      <c r="B14" s="19">
+        <f>'Three-School Projection'!E86</f>
+        <v/>
+      </c>
+      <c r="C14" s="19">
+        <f>B10</f>
+        <v/>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E14" s="21">
+        <f>B14+C14+D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Davidson</t>
+        </is>
+      </c>
+      <c r="B15" s="19">
+        <f>'Three-School Projection'!E87</f>
+        <v/>
+      </c>
+      <c r="C15" s="19">
+        <f>B10</f>
+        <v/>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E15" s="21">
+        <f>B15+C15+D15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Hawaii</t>
+        </is>
+      </c>
+      <c r="B16" s="19">
+        <f>'Three-School Projection'!E88</f>
+        <v/>
+      </c>
+      <c r="C16" s="19">
+        <f>B10</f>
+        <v/>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E16" s="21">
+        <f>B16+C16+D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Bkt1 SPV Reach</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>+ Bkt2 Reach</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>− SPV cost</t>
+        </is>
+      </c>
+      <c r="E18" s="17">
+        <f> SPV net Reach</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>St. Joseph's</t>
+        </is>
+      </c>
+      <c r="B19" s="19">
+        <f>'Three-School Projection'!F86</f>
+        <v/>
+      </c>
+      <c r="C19" s="19">
+        <f>C10</f>
+        <v/>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E19" s="21">
+        <f>B19+C19+D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Davidson</t>
+        </is>
+      </c>
+      <c r="B20" s="19">
+        <f>'Three-School Projection'!F87</f>
+        <v/>
+      </c>
+      <c r="C20" s="19">
+        <f>C10</f>
+        <v/>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E20" s="21">
+        <f>B20+C20+D20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Hawaii</t>
+        </is>
+      </c>
+      <c r="B21" s="19">
+        <f>'Three-School Projection'!F88</f>
+        <v/>
+      </c>
+      <c r="C21" s="19">
+        <f>C10</f>
+        <v/>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E21" s="21">
+        <f>B21+C21+D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>Bucket 2 is 100% SPV and never touches the school sheet or the 80/20 split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Series &amp; live-game costs are already netted in their lines (EverWonder finances production, recoups cost+10%). The $15M SPV cost = roster/NIL + ops.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>MC-originated sponsorship: rather than routing MC-sourced signage/MMR-scope deals through Learfield's fixed guarantee (where the upside gets trapped), MC originates and keeps ~85%. Safer and higher than the 80/20 team-revenue path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>Per-school variance is minor (national platform) — Davidson skews high via the Curry anchor. Reach is the optimistic ceiling; underwrite on Base.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Move MC-originated MMR/signage sponsorship to Bucket 1 (85% kept, runs through 80/20); Bucket 2 = on-screen only
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1561,1018 +1561,1018 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MC-originated MMR/signage (85% kept; 15% Learfield)</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="J36" s="7" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Corporate sponsorship &amp; multimedia rights</t>
         </is>
       </c>
-      <c r="B36" s="10">
-        <f>SUM(B29:B35)</f>
-        <v/>
-      </c>
-      <c r="C36" s="10">
-        <f>SUM(C29:C35)</f>
-        <v/>
-      </c>
-      <c r="D36" s="10">
-        <f>SUM(D29:D35)</f>
-        <v/>
-      </c>
-      <c r="E36" s="10">
-        <f>SUM(E29:E35)</f>
-        <v/>
-      </c>
-      <c r="F36" s="10">
-        <f>SUM(F29:F35)</f>
-        <v/>
-      </c>
-      <c r="G36" s="10">
-        <f>SUM(G29:G35)</f>
-        <v/>
-      </c>
-      <c r="H36" s="10">
-        <f>SUM(H29:H35)</f>
-        <v/>
-      </c>
-      <c r="I36" s="10">
-        <f>SUM(I29:I35)</f>
-        <v/>
-      </c>
-      <c r="J36" s="10">
-        <f>SUM(J29:J35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="B37" s="10">
+        <f>SUM(B29:B36)</f>
+        <v/>
+      </c>
+      <c r="C37" s="10">
+        <f>SUM(C29:C36)</f>
+        <v/>
+      </c>
+      <c r="D37" s="10">
+        <f>SUM(D29:D36)</f>
+        <v/>
+      </c>
+      <c r="E37" s="10">
+        <f>SUM(E29:E36)</f>
+        <v/>
+      </c>
+      <c r="F37" s="10">
+        <f>SUM(F29:F36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="10">
+        <f>SUM(G29:G36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="10">
+        <f>SUM(H29:H36)</f>
+        <v/>
+      </c>
+      <c r="I37" s="10">
+        <f>SUM(I29:I36)</f>
+        <v/>
+      </c>
+      <c r="J37" s="10">
+        <f>SUM(J29:J36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>Philanthropy &amp; donor</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="6" t="n"/>
-      <c r="J38" s="6" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Annual fund / booster donations</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="n">
-        <v>180</v>
-      </c>
-      <c r="C39" s="8" t="n">
-        <v>740</v>
-      </c>
-      <c r="D39" s="7" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E39" s="7" t="n">
-        <v>270</v>
-      </c>
-      <c r="F39" s="8" t="n">
-        <v>1110</v>
-      </c>
-      <c r="G39" s="7" t="n">
-        <v>1800</v>
-      </c>
-      <c r="H39" s="7" t="n">
-        <v>150</v>
-      </c>
-      <c r="I39" s="8" t="n">
-        <v>620</v>
-      </c>
-      <c r="J39" s="7" t="n">
-        <v>1000</v>
-      </c>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Seat-related required donations (PSLs)</t>
+          <t xml:space="preserve">   Annual fund / booster donations</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="C40" s="8" t="n">
-        <v>480</v>
+        <v>740</v>
       </c>
       <c r="D40" s="7" t="n">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="E40" s="7" t="n">
+        <v>270</v>
+      </c>
+      <c r="F40" s="8" t="n">
+        <v>1110</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H40" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="F40" s="8" t="n">
-        <v>730</v>
-      </c>
-      <c r="G40" s="7" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H40" s="7" t="n">
-        <v>60</v>
-      </c>
       <c r="I40" s="8" t="n">
-        <v>410</v>
+        <v>620</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>700</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Major gifts &amp; endowment (MBB-specific)</t>
+          <t xml:space="preserve">   Seat-related required donations (PSLs)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="C41" s="8" t="n">
+        <v>480</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="F41" s="8" t="n">
+        <v>730</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H41" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="C41" s="8" t="n">
-        <v>580</v>
-      </c>
-      <c r="D41" s="7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E41" s="7" t="n">
-        <v>120</v>
-      </c>
-      <c r="F41" s="8" t="n">
-        <v>880</v>
-      </c>
-      <c r="G41" s="7" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H41" s="7" t="n">
-        <v>40</v>
-      </c>
       <c r="I41" s="8" t="n">
-        <v>510</v>
+        <v>410</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>900</v>
+        <v>700</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Capital-campaign gifts (facilities)</t>
+          <t xml:space="preserve">   Major gifts &amp; endowment (MBB-specific)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C42" s="8" t="n">
-        <v>230</v>
+        <v>580</v>
       </c>
       <c r="D42" s="7" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>410</v>
+        <v>880</v>
       </c>
       <c r="G42" s="7" t="n">
-        <v>700</v>
+        <v>1500</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I42" s="8" t="n">
-        <v>290</v>
+        <v>510</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Capital-campaign gifts (facilities)</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C43" s="8" t="n">
+        <v>230</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>410</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>700</v>
+      </c>
+      <c r="H43" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="I43" s="8" t="n">
+        <v>290</v>
+      </c>
+      <c r="J43" s="7" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Collective / NIL donor contributions</t>
         </is>
       </c>
-      <c r="B43" s="7" t="n">
+      <c r="B44" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="C43" s="8" t="n">
+      <c r="C44" s="8" t="n">
         <v>700</v>
       </c>
-      <c r="D43" s="7" t="n">
+      <c r="D44" s="7" t="n">
         <v>1200</v>
       </c>
-      <c r="E43" s="7" t="n">
+      <c r="E44" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="F43" s="8" t="n">
+      <c r="F44" s="8" t="n">
         <v>890</v>
       </c>
-      <c r="G43" s="7" t="n">
+      <c r="G44" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="H43" s="7" t="n">
+      <c r="H44" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="I43" s="8" t="n">
+      <c r="I44" s="8" t="n">
         <v>590</v>
       </c>
-      <c r="J43" s="7" t="n">
+      <c r="J44" s="7" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="9" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Philanthropy &amp; donor</t>
         </is>
       </c>
-      <c r="B44" s="10">
-        <f>SUM(B39:B43)</f>
-        <v/>
-      </c>
-      <c r="C44" s="10">
-        <f>SUM(C39:C43)</f>
-        <v/>
-      </c>
-      <c r="D44" s="10">
-        <f>SUM(D39:D43)</f>
-        <v/>
-      </c>
-      <c r="E44" s="10">
-        <f>SUM(E39:E43)</f>
-        <v/>
-      </c>
-      <c r="F44" s="10">
-        <f>SUM(F39:F43)</f>
-        <v/>
-      </c>
-      <c r="G44" s="10">
-        <f>SUM(G39:G43)</f>
-        <v/>
-      </c>
-      <c r="H44" s="10">
-        <f>SUM(H39:H43)</f>
-        <v/>
-      </c>
-      <c r="I44" s="10">
-        <f>SUM(I39:I43)</f>
-        <v/>
-      </c>
-      <c r="J44" s="10">
-        <f>SUM(J39:J43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="B45" s="10">
+        <f>SUM(B40:B44)</f>
+        <v/>
+      </c>
+      <c r="C45" s="10">
+        <f>SUM(C40:C44)</f>
+        <v/>
+      </c>
+      <c r="D45" s="10">
+        <f>SUM(D40:D44)</f>
+        <v/>
+      </c>
+      <c r="E45" s="10">
+        <f>SUM(E40:E44)</f>
+        <v/>
+      </c>
+      <c r="F45" s="10">
+        <f>SUM(F40:F44)</f>
+        <v/>
+      </c>
+      <c r="G45" s="10">
+        <f>SUM(G40:G44)</f>
+        <v/>
+      </c>
+      <c r="H45" s="10">
+        <f>SUM(H40:H44)</f>
+        <v/>
+      </c>
+      <c r="I45" s="10">
+        <f>SUM(I40:I44)</f>
+        <v/>
+      </c>
+      <c r="J45" s="10">
+        <f>SUM(J40:J44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>Apparel &amp; licensing</t>
         </is>
       </c>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="6" t="n"/>
-      <c r="D46" s="6" t="n"/>
-      <c r="E46" s="6" t="n"/>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="6" t="n"/>
-      <c r="H46" s="6" t="n"/>
-      <c r="I46" s="6" t="n"/>
-      <c r="J46" s="6" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Shoe/apparel contract (cash + product)</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="C47" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D47" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="E47" s="7" t="n">
-        <v>300</v>
-      </c>
-      <c r="F47" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G47" s="7" t="n">
-        <v>300</v>
-      </c>
-      <c r="H47" s="7" t="n">
-        <v>150</v>
-      </c>
-      <c r="I47" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="J47" s="7" t="n">
-        <v>150</v>
-      </c>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
+      <c r="J47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Trademark / logo licensing royalties</t>
+          <t xml:space="preserve">   Shoe/apparel contract (cash + product)</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="C48" s="8" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="D48" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>20</v>
+        <v>300</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>370</v>
+        <v>300</v>
       </c>
       <c r="G48" s="7" t="n">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="H48" s="7" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="I48" s="8" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="J48" s="7" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Team retail merchandise sales</t>
+          <t xml:space="preserve">   Trademark / logo licensing royalties</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C49" s="8" t="n">
-        <v>490</v>
+        <v>240</v>
       </c>
       <c r="D49" s="7" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>620</v>
+        <v>370</v>
       </c>
       <c r="G49" s="7" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>380</v>
+        <v>180</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>600</v>
+        <v>300</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Team retail merchandise sales</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C50" s="8" t="n">
+        <v>490</v>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="F50" s="8" t="n">
+        <v>620</v>
+      </c>
+      <c r="G50" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H50" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="I50" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="J50" s="7" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Video-game / EA royalties</t>
         </is>
       </c>
-      <c r="B50" s="7" t="n">
+      <c r="B51" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C50" s="8" t="n">
+      <c r="C51" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="D50" s="7" t="n">
+      <c r="D51" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="E50" s="7" t="n">
+      <c r="E51" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F50" s="8" t="n">
+      <c r="F51" s="8" t="n">
         <v>90</v>
       </c>
-      <c r="G50" s="7" t="n">
+      <c r="G51" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="H50" s="7" t="n">
+      <c r="H51" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="I50" s="8" t="n">
+      <c r="I51" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="J50" s="7" t="n">
+      <c r="J51" s="7" t="n">
         <v>80</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="9" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Apparel &amp; licensing</t>
         </is>
       </c>
-      <c r="B51" s="10">
-        <f>SUM(B47:B50)</f>
-        <v/>
-      </c>
-      <c r="C51" s="10">
-        <f>SUM(C47:C50)</f>
-        <v/>
-      </c>
-      <c r="D51" s="10">
-        <f>SUM(D47:D50)</f>
-        <v/>
-      </c>
-      <c r="E51" s="10">
-        <f>SUM(E47:E50)</f>
-        <v/>
-      </c>
-      <c r="F51" s="10">
-        <f>SUM(F47:F50)</f>
-        <v/>
-      </c>
-      <c r="G51" s="10">
-        <f>SUM(G47:G50)</f>
-        <v/>
-      </c>
-      <c r="H51" s="10">
-        <f>SUM(H47:H50)</f>
-        <v/>
-      </c>
-      <c r="I51" s="10">
-        <f>SUM(I47:I50)</f>
-        <v/>
-      </c>
-      <c r="J51" s="10">
-        <f>SUM(J47:J50)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="B52" s="10">
+        <f>SUM(B48:B51)</f>
+        <v/>
+      </c>
+      <c r="C52" s="10">
+        <f>SUM(C48:C51)</f>
+        <v/>
+      </c>
+      <c r="D52" s="10">
+        <f>SUM(D48:D51)</f>
+        <v/>
+      </c>
+      <c r="E52" s="10">
+        <f>SUM(E48:E51)</f>
+        <v/>
+      </c>
+      <c r="F52" s="10">
+        <f>SUM(F48:F51)</f>
+        <v/>
+      </c>
+      <c r="G52" s="10">
+        <f>SUM(G48:G51)</f>
+        <v/>
+      </c>
+      <c r="H52" s="10">
+        <f>SUM(H48:H51)</f>
+        <v/>
+      </c>
+      <c r="I52" s="10">
+        <f>SUM(I48:I51)</f>
+        <v/>
+      </c>
+      <c r="J52" s="10">
+        <f>SUM(J48:J51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>Guarantees &amp; scheduling</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="6" t="n"/>
-      <c r="H53" s="6" t="n"/>
-      <c r="I53" s="6" t="n"/>
-      <c r="J53" s="6" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Guarantee ('buy') game income</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="C54" s="8" t="n">
-        <v>410</v>
-      </c>
-      <c r="D54" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="E54" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="F54" s="8" t="n">
-        <v>410</v>
-      </c>
-      <c r="G54" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="H54" s="7" t="n">
-        <v>120</v>
-      </c>
-      <c r="I54" s="8" t="n">
-        <v>360</v>
-      </c>
-      <c r="J54" s="7" t="n">
-        <v>500</v>
-      </c>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="6" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="6" t="n"/>
+      <c r="H54" s="6" t="n"/>
+      <c r="I54" s="6" t="n"/>
+      <c r="J54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Neutral-site / MTE appearance fees</t>
+          <t xml:space="preserve">   Guarantee ('buy') game income</t>
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="C55" s="8" t="n">
-        <v>510</v>
+        <v>410</v>
       </c>
       <c r="D55" s="7" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>570</v>
+        <v>410</v>
       </c>
       <c r="G55" s="7" t="n">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="I55" s="8" t="n">
-        <v>470</v>
+        <v>360</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Early-season / holiday tournament payouts</t>
+          <t xml:space="preserve">   Neutral-site / MTE appearance fees</t>
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C56" s="8" t="n">
-        <v>260</v>
+        <v>510</v>
       </c>
       <c r="D56" s="7" t="n">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F56" s="8" t="n">
-        <v>320</v>
+        <v>570</v>
       </c>
       <c r="G56" s="7" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="H56" s="7" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="I56" s="8" t="n">
-        <v>260</v>
+        <v>470</v>
       </c>
       <c r="J56" s="7" t="n">
-        <v>400</v>
+        <v>700</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Early-season / holiday tournament payouts</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C57" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F57" s="8" t="n">
+        <v>320</v>
+      </c>
+      <c r="G57" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="H57" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="I57" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="J57" s="7" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Exhibition / charity game revenue</t>
         </is>
       </c>
-      <c r="B57" s="7" t="n">
+      <c r="B58" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C57" s="8" t="n">
+      <c r="C58" s="8" t="n">
         <v>70</v>
       </c>
-      <c r="D57" s="7" t="n">
+      <c r="D58" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="E57" s="7" t="n">
+      <c r="E58" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F57" s="8" t="n">
+      <c r="F58" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="G57" s="7" t="n">
+      <c r="G58" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="H57" s="7" t="n">
+      <c r="H58" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="I57" s="8" t="n">
+      <c r="I58" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="J57" s="7" t="n">
+      <c r="J58" s="7" t="n">
         <v>80</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="9" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Guarantees &amp; scheduling</t>
         </is>
       </c>
-      <c r="B58" s="10">
-        <f>SUM(B54:B57)</f>
-        <v/>
-      </c>
-      <c r="C58" s="10">
-        <f>SUM(C54:C57)</f>
-        <v/>
-      </c>
-      <c r="D58" s="10">
-        <f>SUM(D54:D57)</f>
-        <v/>
-      </c>
-      <c r="E58" s="10">
-        <f>SUM(E54:E57)</f>
-        <v/>
-      </c>
-      <c r="F58" s="10">
-        <f>SUM(F54:F57)</f>
-        <v/>
-      </c>
-      <c r="G58" s="10">
-        <f>SUM(G54:G57)</f>
-        <v/>
-      </c>
-      <c r="H58" s="10">
-        <f>SUM(H54:H57)</f>
-        <v/>
-      </c>
-      <c r="I58" s="10">
-        <f>SUM(I54:I57)</f>
-        <v/>
-      </c>
-      <c r="J58" s="10">
-        <f>SUM(J54:J57)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="B59" s="10">
+        <f>SUM(B55:B58)</f>
+        <v/>
+      </c>
+      <c r="C59" s="10">
+        <f>SUM(C55:C58)</f>
+        <v/>
+      </c>
+      <c r="D59" s="10">
+        <f>SUM(D55:D58)</f>
+        <v/>
+      </c>
+      <c r="E59" s="10">
+        <f>SUM(E55:E58)</f>
+        <v/>
+      </c>
+      <c r="F59" s="10">
+        <f>SUM(F55:F58)</f>
+        <v/>
+      </c>
+      <c r="G59" s="10">
+        <f>SUM(G55:G58)</f>
+        <v/>
+      </c>
+      <c r="H59" s="10">
+        <f>SUM(H55:H58)</f>
+        <v/>
+      </c>
+      <c r="I59" s="10">
+        <f>SUM(I55:I58)</f>
+        <v/>
+      </c>
+      <c r="J59" s="10">
+        <f>SUM(J55:J58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>Camps, clinics &amp; operations</t>
         </is>
       </c>
-      <c r="B60" s="6" t="n"/>
-      <c r="C60" s="6" t="n"/>
-      <c r="D60" s="6" t="n"/>
-      <c r="E60" s="6" t="n"/>
-      <c r="F60" s="6" t="n"/>
-      <c r="G60" s="6" t="n"/>
-      <c r="H60" s="6" t="n"/>
-      <c r="I60" s="6" t="n"/>
-      <c r="J60" s="6" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Basketball camps &amp; clinics revenue</t>
-        </is>
-      </c>
-      <c r="B61" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="C61" s="8" t="n">
-        <v>270</v>
-      </c>
-      <c r="D61" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="E61" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="F61" s="8" t="n">
-        <v>350</v>
-      </c>
-      <c r="G61" s="7" t="n">
-        <v>500</v>
-      </c>
-      <c r="H61" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="I61" s="8" t="n">
-        <v>240</v>
-      </c>
-      <c r="J61" s="7" t="n">
-        <v>350</v>
-      </c>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="6" t="n"/>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="6" t="n"/>
+      <c r="F61" s="6" t="n"/>
+      <c r="G61" s="6" t="n"/>
+      <c r="H61" s="6" t="n"/>
+      <c r="I61" s="6" t="n"/>
+      <c r="J61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Coach's camps</t>
+          <t xml:space="preserve">   Basketball camps &amp; clinics revenue</t>
         </is>
       </c>
       <c r="B62" s="7" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C62" s="8" t="n">
-        <v>140</v>
+        <v>270</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="E62" s="7" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>170</v>
+        <v>350</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="H62" s="7" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="I62" s="8" t="n">
-        <v>100</v>
+        <v>240</v>
       </c>
       <c r="J62" s="7" t="n">
-        <v>150</v>
+        <v>350</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Facility rentals (MBB-allocated)</t>
+          <t xml:space="preserve">   Coach's camps</t>
         </is>
       </c>
       <c r="B63" s="7" t="n">
         <v>20</v>
       </c>
       <c r="C63" s="8" t="n">
+        <v>140</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F63" s="8" t="n">
+        <v>170</v>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="H63" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="I63" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="D63" s="7" t="n">
+      <c r="J63" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="E63" s="7" t="n">
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Facility rentals (MBB-allocated)</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F63" s="8" t="n">
+      <c r="C64" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F64" s="8" t="n">
         <v>120</v>
       </c>
-      <c r="G63" s="7" t="n">
+      <c r="G64" s="7" t="n">
         <v>180</v>
       </c>
-      <c r="H63" s="7" t="n">
+      <c r="H64" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="I63" s="8" t="n">
+      <c r="I64" s="8" t="n">
         <v>170</v>
       </c>
-      <c r="J63" s="7" t="n">
+      <c r="J64" s="7" t="n">
         <v>250</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="9" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Camps, clinics &amp; operations</t>
         </is>
       </c>
-      <c r="B64" s="10">
-        <f>SUM(B61:B63)</f>
-        <v/>
-      </c>
-      <c r="C64" s="10">
-        <f>SUM(C61:C63)</f>
-        <v/>
-      </c>
-      <c r="D64" s="10">
-        <f>SUM(D61:D63)</f>
-        <v/>
-      </c>
-      <c r="E64" s="10">
-        <f>SUM(E61:E63)</f>
-        <v/>
-      </c>
-      <c r="F64" s="10">
-        <f>SUM(F61:F63)</f>
-        <v/>
-      </c>
-      <c r="G64" s="10">
-        <f>SUM(G61:G63)</f>
-        <v/>
-      </c>
-      <c r="H64" s="10">
-        <f>SUM(H61:H63)</f>
-        <v/>
-      </c>
-      <c r="I64" s="10">
-        <f>SUM(I61:I63)</f>
-        <v/>
-      </c>
-      <c r="J64" s="10">
-        <f>SUM(J61:J63)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="B65" s="10">
+        <f>SUM(B62:B64)</f>
+        <v/>
+      </c>
+      <c r="C65" s="10">
+        <f>SUM(C62:C64)</f>
+        <v/>
+      </c>
+      <c r="D65" s="10">
+        <f>SUM(D62:D64)</f>
+        <v/>
+      </c>
+      <c r="E65" s="10">
+        <f>SUM(E62:E64)</f>
+        <v/>
+      </c>
+      <c r="F65" s="10">
+        <f>SUM(F62:F64)</f>
+        <v/>
+      </c>
+      <c r="G65" s="10">
+        <f>SUM(G62:G64)</f>
+        <v/>
+      </c>
+      <c r="H65" s="10">
+        <f>SUM(H62:H64)</f>
+        <v/>
+      </c>
+      <c r="I65" s="10">
+        <f>SUM(I62:I64)</f>
+        <v/>
+      </c>
+      <c r="J65" s="10">
+        <f>SUM(J62:J64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>Institutional &amp; other support</t>
         </is>
       </c>
-      <c r="B66" s="6" t="n"/>
-      <c r="C66" s="6" t="n"/>
-      <c r="D66" s="6" t="n"/>
-      <c r="E66" s="6" t="n"/>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="6" t="n"/>
-      <c r="H66" s="6" t="n"/>
-      <c r="I66" s="6" t="n"/>
-      <c r="J66" s="6" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Direct institutional / university support</t>
-        </is>
-      </c>
-      <c r="B67" s="7" t="n">
-        <v>240</v>
-      </c>
-      <c r="C67" s="8" t="n">
-        <v>320</v>
-      </c>
-      <c r="D67" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="E67" s="7" t="n">
-        <v>180</v>
-      </c>
-      <c r="F67" s="8" t="n">
-        <v>240</v>
-      </c>
-      <c r="G67" s="7" t="n">
-        <v>300</v>
-      </c>
-      <c r="H67" s="7" t="n">
-        <v>360</v>
-      </c>
-      <c r="I67" s="8" t="n">
-        <v>530</v>
-      </c>
-      <c r="J67" s="7" t="n">
-        <v>700</v>
-      </c>
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="6" t="n"/>
+      <c r="G67" s="6" t="n"/>
+      <c r="H67" s="6" t="n"/>
+      <c r="I67" s="6" t="n"/>
+      <c r="J67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Student-fee allocation</t>
+          <t xml:space="preserve">   Direct institutional / university support</t>
         </is>
       </c>
       <c r="B68" s="7" t="n">
-        <v>60</v>
+        <v>240</v>
       </c>
       <c r="C68" s="8" t="n">
-        <v>80</v>
+        <v>320</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="F68" s="8" t="n">
-        <v>40</v>
+        <v>240</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>180</v>
+        <v>360</v>
       </c>
       <c r="I68" s="8" t="n">
-        <v>290</v>
+        <v>530</v>
       </c>
       <c r="J68" s="7" t="n">
-        <v>400</v>
+        <v>700</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Direct state / government support</t>
+          <t xml:space="preserve">   Student-fee allocation</t>
         </is>
       </c>
       <c r="B69" s="7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="C69" s="8" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="D69" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>240</v>
+        <v>180</v>
       </c>
       <c r="I69" s="8" t="n">
-        <v>420</v>
+        <v>290</v>
       </c>
       <c r="J69" s="7" t="n">
-        <v>600</v>
+        <v>400</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Athletics endowment / investment income</t>
+          <t xml:space="preserve">   Direct state / government support</t>
         </is>
       </c>
       <c r="B70" s="7" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C70" s="8" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F70" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="7" t="n">
         <v>240</v>
       </c>
-      <c r="G70" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="H70" s="7" t="n">
-        <v>20</v>
-      </c>
       <c r="I70" s="8" t="n">
-        <v>50</v>
+        <v>420</v>
       </c>
       <c r="J70" s="7" t="n">
-        <v>80</v>
+        <v>600</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Third-party in-kind &amp; third-party-paid comp</t>
+          <t xml:space="preserve">   Athletics endowment / investment income</t>
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C71" s="8" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="D71" s="7" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>80</v>
+        <v>240</v>
       </c>
       <c r="G71" s="7" t="n">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="H71" s="7" t="n">
         <v>20</v>
       </c>
       <c r="I71" s="8" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="J71" s="7" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Other / misc operating revenue</t>
+          <t xml:space="preserve">   Third-party in-kind &amp; third-party-paid comp</t>
         </is>
       </c>
       <c r="B72" s="7" t="n">
@@ -2588,418 +2588,417 @@
         <v>20</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="H72" s="7" t="n">
         <v>20</v>
       </c>
       <c r="I72" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="J72" s="7" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Other / misc operating revenue</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C73" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="J72" s="7" t="n">
+      <c r="D73" s="7" t="n">
         <v>100</v>
       </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="9" t="inlineStr">
+      <c r="E73" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F73" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="G73" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H73" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="I73" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J73" s="7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Institutional &amp; other support</t>
         </is>
       </c>
-      <c r="B73" s="10">
-        <f>SUM(B67:B72)</f>
-        <v/>
-      </c>
-      <c r="C73" s="10">
-        <f>SUM(C67:C72)</f>
-        <v/>
-      </c>
-      <c r="D73" s="10">
-        <f>SUM(D67:D72)</f>
-        <v/>
-      </c>
-      <c r="E73" s="10">
-        <f>SUM(E67:E72)</f>
-        <v/>
-      </c>
-      <c r="F73" s="10">
-        <f>SUM(F67:F72)</f>
-        <v/>
-      </c>
-      <c r="G73" s="10">
-        <f>SUM(G67:G72)</f>
-        <v/>
-      </c>
-      <c r="H73" s="10">
-        <f>SUM(H67:H72)</f>
-        <v/>
-      </c>
-      <c r="I73" s="10">
-        <f>SUM(I67:I72)</f>
-        <v/>
-      </c>
-      <c r="J73" s="10">
-        <f>SUM(J67:J72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+      <c r="B74" s="10">
+        <f>SUM(B68:B73)</f>
+        <v/>
+      </c>
+      <c r="C74" s="10">
+        <f>SUM(C68:C73)</f>
+        <v/>
+      </c>
+      <c r="D74" s="10">
+        <f>SUM(D68:D73)</f>
+        <v/>
+      </c>
+      <c r="E74" s="10">
+        <f>SUM(E68:E73)</f>
+        <v/>
+      </c>
+      <c r="F74" s="10">
+        <f>SUM(F68:F73)</f>
+        <v/>
+      </c>
+      <c r="G74" s="10">
+        <f>SUM(G68:G73)</f>
+        <v/>
+      </c>
+      <c r="H74" s="10">
+        <f>SUM(H68:H73)</f>
+        <v/>
+      </c>
+      <c r="I74" s="10">
+        <f>SUM(I68:I73)</f>
+        <v/>
+      </c>
+      <c r="J74" s="10">
+        <f>SUM(J68:J73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
         <is>
           <t>NIL / rev-share era  (memo — NOT program revenue; see per-line notes)</t>
         </is>
       </c>
-      <c r="B75" s="6" t="n"/>
-      <c r="C75" s="6" t="n"/>
-      <c r="D75" s="6" t="n"/>
-      <c r="E75" s="6" t="n"/>
-      <c r="F75" s="6" t="n"/>
-      <c r="G75" s="6" t="n"/>
-      <c r="H75" s="6" t="n"/>
-      <c r="I75" s="6" t="n"/>
-      <c r="J75" s="6" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Third-party athlete NIL income (memo — athletes' own $, not SPV rev/cost)</t>
-        </is>
-      </c>
-      <c r="B76" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="C76" s="8" t="n">
-        <v>990</v>
-      </c>
-      <c r="D76" s="7" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E76" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="F76" s="8" t="n">
-        <v>1310</v>
-      </c>
-      <c r="G76" s="7" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H76" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="I76" s="8" t="n">
-        <v>660</v>
-      </c>
-      <c r="J76" s="7" t="n">
-        <v>1000</v>
-      </c>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="6" t="n"/>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="6" t="n"/>
+      <c r="F76" s="6" t="n"/>
+      <c r="G76" s="6" t="n"/>
+      <c r="H76" s="6" t="n"/>
+      <c r="I76" s="6" t="n"/>
+      <c r="J76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Athlete marketing / activation (SPV-produced = Bucket 2)</t>
+          <t xml:space="preserve">   Third-party athlete NIL income (memo — athletes' own $, not SPV rev/cost)</t>
         </is>
       </c>
       <c r="B77" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C77" s="8" t="n">
+        <v>990</v>
+      </c>
+      <c r="D77" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E77" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="F77" s="8" t="n">
+        <v>1310</v>
+      </c>
+      <c r="G77" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H77" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C77" s="8" t="n">
-        <v>530</v>
-      </c>
-      <c r="D77" s="7" t="n">
-        <v>800</v>
-      </c>
-      <c r="E77" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="F77" s="8" t="n">
+      <c r="I77" s="8" t="n">
         <v>660</v>
       </c>
-      <c r="G77" s="7" t="n">
+      <c r="J77" s="7" t="n">
         <v>1000</v>
-      </c>
-      <c r="H77" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="I77" s="8" t="n">
-        <v>390</v>
-      </c>
-      <c r="J77" s="7" t="n">
-        <v>600</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Athlete marketing / activation (SPV-produced = Bucket 2)</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C78" s="8" t="n">
+        <v>530</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="E78" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F78" s="8" t="n">
+        <v>660</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H78" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I78" s="8" t="n">
+        <v>390</v>
+      </c>
+      <c r="J78" s="7" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t xml:space="preserve">   House-settlement rev-share pool (SPV-funded roster COST)</t>
         </is>
       </c>
-      <c r="B78" s="7" t="n">
+      <c r="B79" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C78" s="8" t="n">
+      <c r="C79" s="8" t="n">
         <v>1620</v>
       </c>
-      <c r="D78" s="7" t="n">
+      <c r="D79" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="E78" s="7" t="n">
+      <c r="E79" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F78" s="8" t="n">
+      <c r="F79" s="8" t="n">
         <v>1620</v>
       </c>
-      <c r="G78" s="7" t="n">
+      <c r="G79" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="H78" s="7" t="n">
+      <c r="H79" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I78" s="8" t="n">
+      <c r="I79" s="8" t="n">
         <v>1620</v>
       </c>
-      <c r="J78" s="7" t="n">
+      <c r="J79" s="7" t="n">
         <v>2500</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="9" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — NIL / rev-share era</t>
         </is>
       </c>
-      <c r="B79" s="10">
-        <f>SUM(B76:B78)</f>
-        <v/>
-      </c>
-      <c r="C79" s="10">
-        <f>SUM(C76:C78)</f>
-        <v/>
-      </c>
-      <c r="D79" s="10">
-        <f>SUM(D76:D78)</f>
-        <v/>
-      </c>
-      <c r="E79" s="10">
-        <f>SUM(E76:E78)</f>
-        <v/>
-      </c>
-      <c r="F79" s="10">
-        <f>SUM(F76:F78)</f>
-        <v/>
-      </c>
-      <c r="G79" s="10">
-        <f>SUM(G76:G78)</f>
-        <v/>
-      </c>
-      <c r="H79" s="10">
-        <f>SUM(H76:H78)</f>
-        <v/>
-      </c>
-      <c r="I79" s="10">
-        <f>SUM(I76:I78)</f>
-        <v/>
-      </c>
-      <c r="J79" s="10">
-        <f>SUM(J76:J78)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="11" t="inlineStr">
+      <c r="B80" s="10">
+        <f>SUM(B77:B79)</f>
+        <v/>
+      </c>
+      <c r="C80" s="10">
+        <f>SUM(C77:C79)</f>
+        <v/>
+      </c>
+      <c r="D80" s="10">
+        <f>SUM(D77:D79)</f>
+        <v/>
+      </c>
+      <c r="E80" s="10">
+        <f>SUM(E77:E79)</f>
+        <v/>
+      </c>
+      <c r="F80" s="10">
+        <f>SUM(F77:F79)</f>
+        <v/>
+      </c>
+      <c r="G80" s="10">
+        <f>SUM(G77:G79)</f>
+        <v/>
+      </c>
+      <c r="H80" s="10">
+        <f>SUM(H77:H79)</f>
+        <v/>
+      </c>
+      <c r="I80" s="10">
+        <f>SUM(I77:I79)</f>
+        <v/>
+      </c>
+      <c r="J80" s="10">
+        <f>SUM(J77:J79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
         <is>
           <t>PROGRAM REVENUE  (categories 1–9, excl. NIL)  = the total baseline</t>
         </is>
       </c>
-      <c r="B81" s="12">
-        <f>B12+B19+B26+B36+B44+B51+B58+B64+B73</f>
-        <v/>
-      </c>
-      <c r="C81" s="12">
-        <f>C12+C19+C26+C36+C44+C51+C58+C64+C73</f>
-        <v/>
-      </c>
-      <c r="D81" s="12">
-        <f>D12+D19+D26+D36+D44+D51+D58+D64+D73</f>
-        <v/>
-      </c>
-      <c r="E81" s="12">
-        <f>E12+E19+E26+E36+E44+E51+E58+E64+E73</f>
-        <v/>
-      </c>
-      <c r="F81" s="12">
-        <f>F12+F19+F26+F36+F44+F51+F58+F64+F73</f>
-        <v/>
-      </c>
-      <c r="G81" s="12">
-        <f>G12+G19+G26+G36+G44+G51+G58+G64+G73</f>
-        <v/>
-      </c>
-      <c r="H81" s="12">
-        <f>H12+H19+H26+H36+H44+H51+H58+H64+H73</f>
-        <v/>
-      </c>
-      <c r="I81" s="12">
-        <f>I12+I19+I26+I36+I44+I51+I58+I64+I73</f>
-        <v/>
-      </c>
-      <c r="J81" s="12">
-        <f>J12+J19+J26+J36+J44+J51+J58+J64+J73</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="13" t="inlineStr">
+      <c r="B82" s="12">
+        <f>B12+B19+B26+B37+B45+B52+B59+B65+B74</f>
+        <v/>
+      </c>
+      <c r="C82" s="12">
+        <f>C12+C19+C26+C37+C45+C52+C59+C65+C74</f>
+        <v/>
+      </c>
+      <c r="D82" s="12">
+        <f>D12+D19+D26+D37+D45+D52+D59+D65+D74</f>
+        <v/>
+      </c>
+      <c r="E82" s="12">
+        <f>E12+E19+E26+E37+E45+E52+E59+E65+E74</f>
+        <v/>
+      </c>
+      <c r="F82" s="12">
+        <f>F12+F19+F26+F37+F45+F52+F59+F65+F74</f>
+        <v/>
+      </c>
+      <c r="G82" s="12">
+        <f>G12+G19+G26+G37+G45+G52+G59+G65+G74</f>
+        <v/>
+      </c>
+      <c r="H82" s="12">
+        <f>H12+H19+H26+H37+H45+H52+H59+H65+H74</f>
+        <v/>
+      </c>
+      <c r="I82" s="12">
+        <f>I12+I19+I26+I37+I45+I52+I59+I65+I74</f>
+        <v/>
+      </c>
+      <c r="J82" s="12">
+        <f>J12+J19+J26+J37+J45+J52+J59+J65+J74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="13" t="inlineStr">
         <is>
           <t>NIL / rev-share funding  (memo — SPV-funded cost)</t>
         </is>
       </c>
-      <c r="B82" s="14">
-        <f>B79</f>
-        <v/>
-      </c>
-      <c r="C82" s="14">
-        <f>C79</f>
-        <v/>
-      </c>
-      <c r="D82" s="14">
-        <f>D79</f>
-        <v/>
-      </c>
-      <c r="E82" s="14">
-        <f>E79</f>
-        <v/>
-      </c>
-      <c r="F82" s="14">
-        <f>F79</f>
-        <v/>
-      </c>
-      <c r="G82" s="14">
-        <f>G79</f>
-        <v/>
-      </c>
-      <c r="H82" s="14">
-        <f>H79</f>
-        <v/>
-      </c>
-      <c r="I82" s="14">
-        <f>I79</f>
-        <v/>
-      </c>
-      <c r="J82" s="14">
-        <f>J79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="15" t="inlineStr">
+      <c r="B83" s="14">
+        <f>B80</f>
+        <v/>
+      </c>
+      <c r="C83" s="14">
+        <f>C80</f>
+        <v/>
+      </c>
+      <c r="D83" s="14">
+        <f>D80</f>
+        <v/>
+      </c>
+      <c r="E83" s="14">
+        <f>E80</f>
+        <v/>
+      </c>
+      <c r="F83" s="14">
+        <f>F80</f>
+        <v/>
+      </c>
+      <c r="G83" s="14">
+        <f>G80</f>
+        <v/>
+      </c>
+      <c r="H83" s="14">
+        <f>H80</f>
+        <v/>
+      </c>
+      <c r="I83" s="14">
+        <f>I80</f>
+        <v/>
+      </c>
+      <c r="J83" s="14">
+        <f>J80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="15" t="inlineStr">
         <is>
           <t>SPV ECONOMICS  (Bucket 1 above baseline, 80/20; baseline = total current revenue, one lump)</t>
         </is>
       </c>
-      <c r="B84" s="16" t="n"/>
-      <c r="C84" s="16" t="n"/>
-      <c r="D84" s="16" t="n"/>
-      <c r="E84" s="16" t="n"/>
-      <c r="F84" s="16" t="n"/>
-      <c r="G84" s="16" t="n"/>
-      <c r="H84" s="16" t="n"/>
-      <c r="I84" s="16" t="n"/>
-      <c r="J84" s="16" t="n"/>
-    </row>
-    <row r="85" ht="26" customHeight="1">
-      <c r="A85" s="17" t="inlineStr"/>
-      <c r="B85" s="17" t="inlineStr">
+      <c r="B85" s="16" t="n"/>
+      <c r="C85" s="16" t="n"/>
+      <c r="D85" s="16" t="n"/>
+      <c r="E85" s="16" t="n"/>
+      <c r="F85" s="16" t="n"/>
+      <c r="G85" s="16" t="n"/>
+      <c r="H85" s="16" t="n"/>
+      <c r="I85" s="16" t="n"/>
+      <c r="J85" s="16" t="n"/>
+    </row>
+    <row r="86" ht="26" customHeight="1">
+      <c r="A86" s="17" t="inlineStr"/>
+      <c r="B86" s="17" t="inlineStr">
         <is>
           <t>Baseline (total curr.)</t>
         </is>
       </c>
-      <c r="C85" s="17" t="inlineStr">
+      <c r="C86" s="17" t="inlineStr">
         <is>
           <t>Bucket 1 Base w/MC</t>
         </is>
       </c>
-      <c r="D85" s="17" t="inlineStr">
+      <c r="D86" s="17" t="inlineStr">
         <is>
           <t>Bucket 1 Reach w/MC</t>
         </is>
       </c>
-      <c r="E85" s="17" t="inlineStr">
+      <c r="E86" s="17" t="inlineStr">
         <is>
           <t>SPV 80% Base</t>
         </is>
       </c>
-      <c r="F85" s="17" t="inlineStr">
+      <c r="F86" s="17" t="inlineStr">
         <is>
           <t>SPV 80% Reach</t>
         </is>
       </c>
-      <c r="G85" s="17" t="inlineStr">
+      <c r="G86" s="17" t="inlineStr">
         <is>
           <t>School keeps Base</t>
         </is>
       </c>
-      <c r="H85" s="17" t="inlineStr">
+      <c r="H86" s="17" t="inlineStr">
         <is>
           <t>School keeps Reach</t>
         </is>
       </c>
-      <c r="I85" s="17" t="inlineStr"/>
-      <c r="J85" s="17" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="18" t="inlineStr">
-        <is>
-          <t>St. Joseph's</t>
-        </is>
-      </c>
-      <c r="B86" s="19">
-        <f>B81</f>
-        <v/>
-      </c>
-      <c r="C86" s="19">
-        <f>C12+C19+C36+C51+C58+C64</f>
-        <v/>
-      </c>
-      <c r="D86" s="19">
-        <f>D12+D19+D36+D51+D58+D64</f>
-        <v/>
-      </c>
-      <c r="E86" s="20">
-        <f>0.8*(C86-B86)</f>
-        <v/>
-      </c>
-      <c r="F86" s="21">
-        <f>0.8*(D86-B86)</f>
-        <v/>
-      </c>
-      <c r="G86" s="19">
-        <f>B86+0.2*(C86-B86)</f>
-        <v/>
-      </c>
-      <c r="H86" s="19">
-        <f>B86+0.2*(D86-B86)</f>
-        <v/>
-      </c>
+      <c r="I86" s="17" t="inlineStr"/>
+      <c r="J86" s="17" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>Davidson</t>
+          <t>St. Joseph's</t>
         </is>
       </c>
       <c r="B87" s="19">
-        <f>E81</f>
+        <f>B82</f>
         <v/>
       </c>
       <c r="C87" s="19">
-        <f>F12+F19+F36+F51+F58+F64</f>
+        <f>C12+C19+C37+C52+C59+C65</f>
         <v/>
       </c>
       <c r="D87" s="19">
-        <f>G12+G19+G36+G51+G58+G64</f>
+        <f>D12+D19+D37+D52+D59+D65</f>
         <v/>
       </c>
       <c r="E87" s="20">
@@ -3022,19 +3021,19 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>Hawaii</t>
+          <t>Davidson</t>
         </is>
       </c>
       <c r="B88" s="19">
-        <f>H81</f>
+        <f>E82</f>
         <v/>
       </c>
       <c r="C88" s="19">
-        <f>I12+I19+I36+I51+I58+I64</f>
+        <f>F12+F19+F37+F52+F59+F65</f>
         <v/>
       </c>
       <c r="D88" s="19">
-        <f>J12+J19+J36+J51+J58+J64</f>
+        <f>G12+G19+G37+G52+G59+G65</f>
         <v/>
       </c>
       <c r="E88" s="20">
@@ -3054,87 +3053,122 @@
         <v/>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="22" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="18" t="inlineStr">
+        <is>
+          <t>Hawaii</t>
+        </is>
+      </c>
+      <c r="B89" s="19">
+        <f>H82</f>
+        <v/>
+      </c>
+      <c r="C89" s="19">
+        <f>I12+I19+I37+I52+I59+I65</f>
+        <v/>
+      </c>
+      <c r="D89" s="19">
+        <f>J12+J19+J37+J52+J59+J65</f>
+        <v/>
+      </c>
+      <c r="E89" s="20">
+        <f>0.8*(C89-B89)</f>
+        <v/>
+      </c>
+      <c r="F89" s="21">
+        <f>0.8*(D89-B89)</f>
+        <v/>
+      </c>
+      <c r="G89" s="19">
+        <f>B89+0.2*(C89-B89)</f>
+        <v/>
+      </c>
+      <c r="H89" s="19">
+        <f>B89+0.2*(D89-B89)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="22" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
-      <c r="B90" s="23" t="n"/>
-      <c r="C90" s="23" t="n"/>
-      <c r="D90" s="23" t="n"/>
-      <c r="E90" s="23" t="n"/>
-      <c r="F90" s="23" t="n"/>
-      <c r="G90" s="23" t="n"/>
-      <c r="H90" s="23" t="n"/>
-      <c r="I90" s="23" t="n"/>
-      <c r="J90" s="23" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="24" t="inlineStr">
-        <is>
-          <t>Reach = full-attachment estimate (celebrity + Netflix + top-10 roster + deep tournament run all landing). Base = Current + a conservative fraction of that uplift (55-65% on commercial lines).</t>
-        </is>
-      </c>
+      <c r="B91" s="23" t="n"/>
+      <c r="C91" s="23" t="n"/>
+      <c r="D91" s="23" t="n"/>
+      <c r="E91" s="23" t="n"/>
+      <c r="F91" s="23" t="n"/>
+      <c r="G91" s="23" t="n"/>
+      <c r="H91" s="23" t="n"/>
+      <c r="I91" s="23" t="n"/>
+      <c r="J91" s="23" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="24" t="inlineStr">
         <is>
-          <t>MECHANIC (simplified): baseline = the school's TOTAL current program revenue (one lump, the green PROGRAM REVENUE row). The school keeps the first [baseline] dollars; everything in Bucket 1 above the baseline splits 80/20 (SPV 80, school 20). Not itemized line-by-line.</t>
+          <t>Reach = full-attachment estimate (celebrity + Netflix + top-10 roster + deep tournament run all landing). Base = Current + a conservative fraction of that uplift (55-65% on commercial lines).</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="24" t="inlineStr">
         <is>
-          <t>Bucket 1 = the school's commercial revenue with MC (Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps). SPV 80% = 0.8 x (Bucket 1 w/MC - total baseline). School keeps baseline + 20% of the excess.</t>
+          <t>MECHANIC (simplified): baseline = the school's TOTAL current program revenue (one lump, the green PROGRAM REVENUE row). The school keeps the first [baseline] dollars; everything in Bucket 1 above the baseline splits 80/20 (SPV 80, school 20). Not itemized line-by-line.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="24" t="inlineStr">
         <is>
-          <t>Postseason gate: conf tournament &amp; NCAA tournament ticket revenue goes to the CONFERENCE / NCAA, not the school — line reduced to a small allotment margin only.</t>
+          <t>Bucket 1 = the school's commercial revenue with MC (Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps). SPV 80% = 0.8 x (Bucket 1 w/MC - total baseline). School keeps baseline + 20% of the excess.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="24" t="inlineStr">
         <is>
-          <t>Concessions &amp; parking DO grow: marquee home games are relocated to big arenas (St. Joe's -&gt; Xfinity Mobile Arena) where the school is the home promoter and keeps/splits the ancillaries.</t>
+          <t>Postseason gate: conf tournament &amp; NCAA tournament ticket revenue goes to the CONFERENCE / NCAA, not the school — line reduced to a small allotment margin only.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="24" t="inlineStr">
         <is>
-          <t>MMR constraint (Learfield/Playfly own school inventory): Bucket 1 sponsorship kept modest. National / Netflix-grade sponsor + patch = SPV IP (Bucket 2, off this sheet), not school MMR inventory.</t>
+          <t>Concessions &amp; parking DO grow: marquee home games are relocated to big arenas (St. Joe's -&gt; Xfinity Mobile Arena) where the school is the home promoter and keeps/splits the ancillaries.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="24" t="inlineStr">
         <is>
-          <t>Apparel shoe contract held FLAT — multi-year locked deal, no mid-term jump (renewal upside later). Licensing/merch/retail still grow (flexible).</t>
+          <t>MMR/Learfield: MC-originated signage/MMR-scope sponsorship is negotiated 85% to the program / 15% to Learfield, and the 85% is booked HERE in Bucket 1 — then runs through the 80/20 like all team revenue. Only purely on-screen / in-documentary sponsorship sits in Bucket 2.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="24" t="inlineStr">
         <is>
-          <t>NIL memo lines are NOT program revenue: (1) third-party athlete NIL income = athletes' own earnings (a recruiting benefit, not SPV rev/cost); (2) athlete marketing/activation = SPV-produced Bucket 2; (3) House rev-share pool = SPV-funded roster COST.</t>
+          <t>Apparel shoe contract held FLAT — multi-year locked deal, no mid-term jump (renewal upside later). Licensing/merch/retail still grow (flexible).</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="24" t="inlineStr">
         <is>
-          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, athlete-marketing/activation, international + format. Roughly recoups the $15M SPV cost.</t>
+          <t>NIL memo lines are NOT program revenue: (1) third-party athlete NIL income = athletes' own earnings (a recruiting benefit, not SPV rev/cost); (2) athlete marketing/activation = SPV-produced Bucket 2; (3) House rev-share pool = SPV-funded roster COST.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="24" t="inlineStr">
+        <is>
+          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, athlete-marketing/activation, international + format. Roughly recoups the $15M SPV cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="24" t="inlineStr">
         <is>
           <t>Marquee-game relocation assumed: St. Joe's -&gt; Xfinity Mobile Arena (19k); Davidson -&gt; Spectrum Center (19k); Hawaii carried by its 10,300 arena + Diamond Head Classic. All figures ESTIMATES in $000s.</t>
         </is>
@@ -3150,10 +3184,10 @@
     <mergeCell ref="A97:J97"/>
     <mergeCell ref="A100:J100"/>
     <mergeCell ref="A92:J92"/>
-    <mergeCell ref="A91:J91"/>
     <mergeCell ref="A95:J95"/>
     <mergeCell ref="A96:J96"/>
     <mergeCell ref="H2:J2"/>
+    <mergeCell ref="A101:J101"/>
     <mergeCell ref="A98:J98"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
@@ -3167,7 +3201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3271,110 +3305,114 @@
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>priced off Netflix eyeballs; SPV IP, not school MMR</t>
+          <t>on-screen/in-documentary sponsor; SPV IP, not school MMR</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   MC-originated sponsorship (signage/MMR-scope, ~85% SPV)</t>
+          <t xml:space="preserve">   Content engine / athlete marketing &amp; activation</t>
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>6000</v>
+        <v>1500</v>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>MC sources it, keeps ~85% via originator deal; Learfield ~15%</t>
+          <t>SPV-produced branded content; players' NIL contracted</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Content engine / athlete marketing &amp; activation</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="n">
-        <v>500</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D9" s="25" t="inlineStr">
-        <is>
-          <t>SPV-produced branded content; players' NIL contracted</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">   Bucket 2 total (SPV)</t>
         </is>
       </c>
-      <c r="B10" s="10">
-        <f>SUM(B4:B9)</f>
-        <v/>
-      </c>
-      <c r="C10" s="10">
-        <f>SUM(C4:C9)</f>
-        <v/>
-      </c>
+      <c r="B9" s="10">
+        <f>SUM(B4:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="10">
+        <f>SUM(C4:C8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>FULL SPV PICTURE — single season  (Bucket 1 share + Bucket 2 − $15M SPV cost)</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="16" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>FULL SPV PICTURE — single season  (Bucket 1 share + Bucket 2 − $15M SPV cost)</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="16" t="n"/>
-      <c r="E12" s="16" t="n"/>
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Bkt1 SPV Base</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>+ Bkt2 Base</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>− SPV cost</t>
+        </is>
+      </c>
+      <c r="E12" s="17">
+        <f> SPV net Base</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>School</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Bkt1 SPV Base</t>
-        </is>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
-        <is>
-          <t>+ Bkt2 Base</t>
-        </is>
-      </c>
-      <c r="D13" s="17" t="inlineStr">
-        <is>
-          <t>− SPV cost</t>
-        </is>
-      </c>
-      <c r="E13" s="17">
-        <f> SPV net Base</f>
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>St. Joseph's</t>
+        </is>
+      </c>
+      <c r="B13" s="19">
+        <f>'Three-School Projection'!E87</f>
+        <v/>
+      </c>
+      <c r="C13" s="19">
+        <f>B9</f>
+        <v/>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E13" s="21">
+        <f>B13+C13+D13</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>St. Joseph's</t>
+          <t>Davidson</t>
         </is>
       </c>
       <c r="B14" s="19">
-        <f>'Three-School Projection'!E86</f>
+        <f>'Three-School Projection'!E88</f>
         <v/>
       </c>
       <c r="C14" s="19">
-        <f>B10</f>
+        <f>B9</f>
         <v/>
       </c>
       <c r="D14" s="19" t="n">
@@ -3388,15 +3426,15 @@
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>Davidson</t>
+          <t>Hawaii</t>
         </is>
       </c>
       <c r="B15" s="19">
-        <f>'Three-School Projection'!E87</f>
+        <f>'Three-School Projection'!E89</f>
         <v/>
       </c>
       <c r="C15" s="19">
-        <f>B10</f>
+        <f>B9</f>
         <v/>
       </c>
       <c r="D15" s="19" t="n">
@@ -3407,66 +3445,66 @@
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Hawaii</t>
-        </is>
-      </c>
-      <c r="B16" s="19">
-        <f>'Three-School Projection'!E88</f>
-        <v/>
-      </c>
-      <c r="C16" s="19">
-        <f>B10</f>
-        <v/>
-      </c>
-      <c r="D16" s="19" t="n">
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Bkt1 SPV Reach</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>+ Bkt2 Reach</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>− SPV cost</t>
+        </is>
+      </c>
+      <c r="E17" s="17">
+        <f> SPV net Reach</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>St. Joseph's</t>
+        </is>
+      </c>
+      <c r="B18" s="19">
+        <f>'Three-School Projection'!F87</f>
+        <v/>
+      </c>
+      <c r="C18" s="19">
+        <f>C9</f>
+        <v/>
+      </c>
+      <c r="D18" s="19" t="n">
         <v>-15000</v>
       </c>
-      <c r="E16" s="21">
-        <f>B16+C16+D16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>School</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>Bkt1 SPV Reach</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>+ Bkt2 Reach</t>
-        </is>
-      </c>
-      <c r="D18" s="17" t="inlineStr">
-        <is>
-          <t>− SPV cost</t>
-        </is>
-      </c>
-      <c r="E18" s="17">
-        <f> SPV net Reach</f>
+      <c r="E18" s="21">
+        <f>B18+C18+D18</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t>St. Joseph's</t>
+          <t>Davidson</t>
         </is>
       </c>
       <c r="B19" s="19">
-        <f>'Three-School Projection'!F86</f>
+        <f>'Three-School Projection'!F88</f>
         <v/>
       </c>
       <c r="C19" s="19">
-        <f>C10</f>
+        <f>C9</f>
         <v/>
       </c>
       <c r="D19" s="19" t="n">
@@ -3480,15 +3518,15 @@
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
         <is>
-          <t>Davidson</t>
+          <t>Hawaii</t>
         </is>
       </c>
       <c r="B20" s="19">
-        <f>'Three-School Projection'!F87</f>
+        <f>'Three-School Projection'!F89</f>
         <v/>
       </c>
       <c r="C20" s="19">
-        <f>C10</f>
+        <f>C9</f>
         <v/>
       </c>
       <c r="D20" s="19" t="n">
@@ -3499,63 +3537,41 @@
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Hawaii</t>
-        </is>
-      </c>
-      <c r="B21" s="19">
-        <f>'Three-School Projection'!F88</f>
-        <v/>
-      </c>
-      <c r="C21" s="19">
-        <f>C10</f>
-        <v/>
-      </c>
-      <c r="D21" s="19" t="n">
-        <v>-15000</v>
-      </c>
-      <c r="E21" s="21">
-        <f>B21+C21+D21</f>
-        <v/>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>Bucket 2 is 100% SPV and never touches the school sheet or the 80/20 split.</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>Bucket 2 is 100% SPV and never touches the school sheet or the 80/20 split.</t>
+          <t>Series &amp; live-game costs are already netted in their lines (EverWonder finances production, recoups cost+10%). The $15M SPV cost = roster/NIL + ops.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>Series &amp; live-game costs are already netted in their lines (EverWonder finances production, recoups cost+10%). The $15M SPV cost = roster/NIL + ops.</t>
+          <t>Bucket 2 = purely on-screen / in-documentary revenue. MC-originated MMR/signage sponsorship is NOT here — it's booked in Bucket 1 (school sheet) at 85% kept / 15% Learfield, then runs through the 80/20.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>MC-originated sponsorship: rather than routing MC-sourced signage/MMR-scope deals through Learfield's fixed guarantee (where the upside gets trapped), MC originates and keeps ~85%. Safer and higher than the 80/20 team-revenue path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="24" t="inlineStr">
-        <is>
           <t>Per-school variance is minor (national platform) — Davidson skews high via the Curry anchor. Reach is the optimistic ceiling; underwrite on Base.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A22:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove NIL/rev-share section and collective-donor line — none are team revenue
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -99,12 +99,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00808080"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00808080"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -147,8 +147,6 @@
     <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -157,9 +155,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -528,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1790,789 +1788,789 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Collective / NIL donor contributions</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="C44" s="8" t="n">
-        <v>700</v>
-      </c>
-      <c r="D44" s="7" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E44" s="7" t="n">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Subtotal — Philanthropy &amp; donor</t>
+        </is>
+      </c>
+      <c r="B44" s="10">
+        <f>SUM(B40:B43)</f>
+        <v/>
+      </c>
+      <c r="C44" s="10">
+        <f>SUM(C40:C43)</f>
+        <v/>
+      </c>
+      <c r="D44" s="10">
+        <f>SUM(D40:D43)</f>
+        <v/>
+      </c>
+      <c r="E44" s="10">
+        <f>SUM(E40:E43)</f>
+        <v/>
+      </c>
+      <c r="F44" s="10">
+        <f>SUM(F40:F43)</f>
+        <v/>
+      </c>
+      <c r="G44" s="10">
+        <f>SUM(G40:G43)</f>
+        <v/>
+      </c>
+      <c r="H44" s="10">
+        <f>SUM(H40:H43)</f>
+        <v/>
+      </c>
+      <c r="I44" s="10">
+        <f>SUM(I40:I43)</f>
+        <v/>
+      </c>
+      <c r="J44" s="10">
+        <f>SUM(J40:J43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Apparel &amp; licensing</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="n"/>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
+      <c r="I46" s="6" t="n"/>
+      <c r="J46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Shoe/apparel contract (cash + product)</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="F47" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="H47" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="F44" s="8" t="n">
-        <v>890</v>
-      </c>
-      <c r="G44" s="7" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H44" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="I44" s="8" t="n">
-        <v>590</v>
-      </c>
-      <c r="J44" s="7" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Subtotal — Philanthropy &amp; donor</t>
-        </is>
-      </c>
-      <c r="B45" s="10">
-        <f>SUM(B40:B44)</f>
-        <v/>
-      </c>
-      <c r="C45" s="10">
-        <f>SUM(C40:C44)</f>
-        <v/>
-      </c>
-      <c r="D45" s="10">
-        <f>SUM(D40:D44)</f>
-        <v/>
-      </c>
-      <c r="E45" s="10">
-        <f>SUM(E40:E44)</f>
-        <v/>
-      </c>
-      <c r="F45" s="10">
-        <f>SUM(F40:F44)</f>
-        <v/>
-      </c>
-      <c r="G45" s="10">
-        <f>SUM(G40:G44)</f>
-        <v/>
-      </c>
-      <c r="H45" s="10">
-        <f>SUM(H40:H44)</f>
-        <v/>
-      </c>
-      <c r="I45" s="10">
-        <f>SUM(I40:I44)</f>
-        <v/>
-      </c>
-      <c r="J45" s="10">
-        <f>SUM(J40:J44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>Apparel &amp; licensing</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
-      <c r="D47" s="6" t="n"/>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="6" t="n"/>
-      <c r="H47" s="6" t="n"/>
-      <c r="I47" s="6" t="n"/>
-      <c r="J47" s="6" t="n"/>
+      <c r="I47" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="J47" s="7" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Shoe/apparel contract (cash + product)</t>
+          <t xml:space="preserve">   Trademark / logo licensing royalties</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="C48" s="8" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="D48" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="E48" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F48" s="8" t="n">
+        <v>370</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="H48" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I48" s="8" t="n">
+        <v>180</v>
+      </c>
+      <c r="J48" s="7" t="n">
         <v>300</v>
-      </c>
-      <c r="F48" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G48" s="7" t="n">
-        <v>300</v>
-      </c>
-      <c r="H48" s="7" t="n">
-        <v>150</v>
-      </c>
-      <c r="I48" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="J48" s="7" t="n">
-        <v>150</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Trademark / logo licensing royalties</t>
+          <t xml:space="preserve">   Team retail merchandise sales</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C49" s="8" t="n">
-        <v>240</v>
+        <v>490</v>
       </c>
       <c r="D49" s="7" t="n">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>370</v>
+        <v>620</v>
       </c>
       <c r="G49" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H49" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="I49" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="J49" s="7" t="n">
         <v>600</v>
-      </c>
-      <c r="H49" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="I49" s="8" t="n">
-        <v>180</v>
-      </c>
-      <c r="J49" s="7" t="n">
-        <v>300</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Team retail merchandise sales</t>
+          <t xml:space="preserve">   Video-game / EA royalties</t>
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C50" s="8" t="n">
-        <v>490</v>
+        <v>60</v>
       </c>
       <c r="D50" s="7" t="n">
-        <v>800</v>
+        <v>100</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>620</v>
+        <v>90</v>
       </c>
       <c r="G50" s="7" t="n">
-        <v>1000</v>
+        <v>150</v>
       </c>
       <c r="H50" s="7" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I50" s="8" t="n">
-        <v>380</v>
+        <v>50</v>
       </c>
       <c r="J50" s="7" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Subtotal — Apparel &amp; licensing</t>
+        </is>
+      </c>
+      <c r="B51" s="10">
+        <f>SUM(B47:B50)</f>
+        <v/>
+      </c>
+      <c r="C51" s="10">
+        <f>SUM(C47:C50)</f>
+        <v/>
+      </c>
+      <c r="D51" s="10">
+        <f>SUM(D47:D50)</f>
+        <v/>
+      </c>
+      <c r="E51" s="10">
+        <f>SUM(E47:E50)</f>
+        <v/>
+      </c>
+      <c r="F51" s="10">
+        <f>SUM(F47:F50)</f>
+        <v/>
+      </c>
+      <c r="G51" s="10">
+        <f>SUM(G47:G50)</f>
+        <v/>
+      </c>
+      <c r="H51" s="10">
+        <f>SUM(H47:H50)</f>
+        <v/>
+      </c>
+      <c r="I51" s="10">
+        <f>SUM(I47:I50)</f>
+        <v/>
+      </c>
+      <c r="J51" s="10">
+        <f>SUM(J47:J50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Guarantees &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="6" t="n"/>
+      <c r="I53" s="6" t="n"/>
+      <c r="J53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Guarantee ('buy') game income</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="C54" s="8" t="n">
+        <v>410</v>
+      </c>
+      <c r="D54" s="7" t="n">
         <v>600</v>
       </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Video-game / EA royalties</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="C51" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="D51" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E51" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F51" s="8" t="n">
+      <c r="E54" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="G51" s="7" t="n">
-        <v>150</v>
-      </c>
-      <c r="H51" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="I51" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="J51" s="7" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Subtotal — Apparel &amp; licensing</t>
-        </is>
-      </c>
-      <c r="B52" s="10">
-        <f>SUM(B48:B51)</f>
-        <v/>
-      </c>
-      <c r="C52" s="10">
-        <f>SUM(C48:C51)</f>
-        <v/>
-      </c>
-      <c r="D52" s="10">
-        <f>SUM(D48:D51)</f>
-        <v/>
-      </c>
-      <c r="E52" s="10">
-        <f>SUM(E48:E51)</f>
-        <v/>
-      </c>
-      <c r="F52" s="10">
-        <f>SUM(F48:F51)</f>
-        <v/>
-      </c>
-      <c r="G52" s="10">
-        <f>SUM(G48:G51)</f>
-        <v/>
-      </c>
-      <c r="H52" s="10">
-        <f>SUM(H48:H51)</f>
-        <v/>
-      </c>
-      <c r="I52" s="10">
-        <f>SUM(I48:I51)</f>
-        <v/>
-      </c>
-      <c r="J52" s="10">
-        <f>SUM(J48:J51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Guarantees &amp; scheduling</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="6" t="n"/>
-      <c r="D54" s="6" t="n"/>
-      <c r="E54" s="6" t="n"/>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="6" t="n"/>
-      <c r="H54" s="6" t="n"/>
-      <c r="I54" s="6" t="n"/>
-      <c r="J54" s="6" t="n"/>
+      <c r="F54" s="8" t="n">
+        <v>410</v>
+      </c>
+      <c r="G54" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="H54" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="I54" s="8" t="n">
+        <v>360</v>
+      </c>
+      <c r="J54" s="7" t="n">
+        <v>500</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Guarantee ('buy') game income</t>
+          <t xml:space="preserve">   Neutral-site / MTE appearance fees</t>
         </is>
       </c>
       <c r="B55" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C55" s="8" t="n">
+        <v>510</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="F55" s="8" t="n">
+        <v>570</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>900</v>
+      </c>
+      <c r="H55" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="C55" s="8" t="n">
-        <v>410</v>
-      </c>
-      <c r="D55" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="E55" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="F55" s="8" t="n">
-        <v>410</v>
-      </c>
-      <c r="G55" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="H55" s="7" t="n">
-        <v>120</v>
-      </c>
       <c r="I55" s="8" t="n">
-        <v>360</v>
+        <v>470</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Neutral-site / MTE appearance fees</t>
+          <t xml:space="preserve">   Early-season / holiday tournament payouts</t>
         </is>
       </c>
       <c r="B56" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C56" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="E56" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="C56" s="8" t="n">
-        <v>510</v>
-      </c>
-      <c r="D56" s="7" t="n">
-        <v>800</v>
-      </c>
-      <c r="E56" s="7" t="n">
+      <c r="F56" s="8" t="n">
+        <v>320</v>
+      </c>
+      <c r="G56" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="H56" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="F56" s="8" t="n">
-        <v>570</v>
-      </c>
-      <c r="G56" s="7" t="n">
-        <v>900</v>
-      </c>
-      <c r="H56" s="7" t="n">
-        <v>90</v>
-      </c>
       <c r="I56" s="8" t="n">
-        <v>470</v>
+        <v>260</v>
       </c>
       <c r="J56" s="7" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Early-season / holiday tournament payouts</t>
+          <t xml:space="preserve">   Exhibition / charity game revenue</t>
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C57" s="8" t="n">
-        <v>260</v>
+        <v>70</v>
       </c>
       <c r="D57" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F57" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="G57" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H57" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I57" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="J57" s="7" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Subtotal — Guarantees &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="B58" s="10">
+        <f>SUM(B54:B57)</f>
+        <v/>
+      </c>
+      <c r="C58" s="10">
+        <f>SUM(C54:C57)</f>
+        <v/>
+      </c>
+      <c r="D58" s="10">
+        <f>SUM(D54:D57)</f>
+        <v/>
+      </c>
+      <c r="E58" s="10">
+        <f>SUM(E54:E57)</f>
+        <v/>
+      </c>
+      <c r="F58" s="10">
+        <f>SUM(F54:F57)</f>
+        <v/>
+      </c>
+      <c r="G58" s="10">
+        <f>SUM(G54:G57)</f>
+        <v/>
+      </c>
+      <c r="H58" s="10">
+        <f>SUM(H54:H57)</f>
+        <v/>
+      </c>
+      <c r="I58" s="10">
+        <f>SUM(I54:I57)</f>
+        <v/>
+      </c>
+      <c r="J58" s="10">
+        <f>SUM(J54:J57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Camps, clinics &amp; operations</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="n"/>
+      <c r="C60" s="6" t="n"/>
+      <c r="D60" s="6" t="n"/>
+      <c r="E60" s="6" t="n"/>
+      <c r="F60" s="6" t="n"/>
+      <c r="G60" s="6" t="n"/>
+      <c r="H60" s="6" t="n"/>
+      <c r="I60" s="6" t="n"/>
+      <c r="J60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Basketball camps &amp; clinics revenue</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="C61" s="8" t="n">
+        <v>270</v>
+      </c>
+      <c r="D61" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="E57" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="F57" s="8" t="n">
-        <v>320</v>
-      </c>
-      <c r="G57" s="7" t="n">
+      <c r="E61" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F61" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="G61" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="H57" s="7" t="n">
+      <c r="H61" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="I57" s="8" t="n">
-        <v>260</v>
-      </c>
-      <c r="J57" s="7" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Exhibition / charity game revenue</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="C58" s="8" t="n">
-        <v>70</v>
-      </c>
-      <c r="D58" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E58" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F58" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="G58" s="7" t="n">
-        <v>120</v>
-      </c>
-      <c r="H58" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="I58" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="J58" s="7" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Subtotal — Guarantees &amp; scheduling</t>
-        </is>
-      </c>
-      <c r="B59" s="10">
-        <f>SUM(B55:B58)</f>
-        <v/>
-      </c>
-      <c r="C59" s="10">
-        <f>SUM(C55:C58)</f>
-        <v/>
-      </c>
-      <c r="D59" s="10">
-        <f>SUM(D55:D58)</f>
-        <v/>
-      </c>
-      <c r="E59" s="10">
-        <f>SUM(E55:E58)</f>
-        <v/>
-      </c>
-      <c r="F59" s="10">
-        <f>SUM(F55:F58)</f>
-        <v/>
-      </c>
-      <c r="G59" s="10">
-        <f>SUM(G55:G58)</f>
-        <v/>
-      </c>
-      <c r="H59" s="10">
-        <f>SUM(H55:H58)</f>
-        <v/>
-      </c>
-      <c r="I59" s="10">
-        <f>SUM(I55:I58)</f>
-        <v/>
-      </c>
-      <c r="J59" s="10">
-        <f>SUM(J55:J58)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>Camps, clinics &amp; operations</t>
-        </is>
-      </c>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="6" t="n"/>
-      <c r="D61" s="6" t="n"/>
-      <c r="E61" s="6" t="n"/>
-      <c r="F61" s="6" t="n"/>
-      <c r="G61" s="6" t="n"/>
-      <c r="H61" s="6" t="n"/>
-      <c r="I61" s="6" t="n"/>
-      <c r="J61" s="6" t="n"/>
+      <c r="I61" s="8" t="n">
+        <v>240</v>
+      </c>
+      <c r="J61" s="7" t="n">
+        <v>350</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Basketball camps &amp; clinics revenue</t>
+          <t xml:space="preserve">   Coach's camps</t>
         </is>
       </c>
       <c r="B62" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C62" s="8" t="n">
-        <v>270</v>
+        <v>140</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="E62" s="7" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>350</v>
+        <v>170</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H62" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I62" s="8" t="n">
-        <v>240</v>
+        <v>100</v>
       </c>
       <c r="J62" s="7" t="n">
-        <v>350</v>
+        <v>150</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Coach's camps</t>
+          <t xml:space="preserve">   Facility rentals (MBB-allocated)</t>
         </is>
       </c>
       <c r="B63" s="7" t="n">
         <v>20</v>
       </c>
       <c r="C63" s="8" t="n">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="D63" s="7" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="E63" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F63" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>180</v>
+      </c>
+      <c r="H63" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="F63" s="8" t="n">
+      <c r="I63" s="8" t="n">
         <v>170</v>
       </c>
-      <c r="G63" s="7" t="n">
+      <c r="J63" s="7" t="n">
         <v>250</v>
       </c>
-      <c r="H63" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="I63" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="J63" s="7" t="n">
-        <v>150</v>
-      </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Facility rentals (MBB-allocated)</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="C64" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="D64" s="7" t="n">
-        <v>150</v>
-      </c>
-      <c r="E64" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="F64" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="G64" s="7" t="n">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Subtotal — Camps, clinics &amp; operations</t>
+        </is>
+      </c>
+      <c r="B64" s="10">
+        <f>SUM(B61:B63)</f>
+        <v/>
+      </c>
+      <c r="C64" s="10">
+        <f>SUM(C61:C63)</f>
+        <v/>
+      </c>
+      <c r="D64" s="10">
+        <f>SUM(D61:D63)</f>
+        <v/>
+      </c>
+      <c r="E64" s="10">
+        <f>SUM(E61:E63)</f>
+        <v/>
+      </c>
+      <c r="F64" s="10">
+        <f>SUM(F61:F63)</f>
+        <v/>
+      </c>
+      <c r="G64" s="10">
+        <f>SUM(G61:G63)</f>
+        <v/>
+      </c>
+      <c r="H64" s="10">
+        <f>SUM(H61:H63)</f>
+        <v/>
+      </c>
+      <c r="I64" s="10">
+        <f>SUM(I61:I63)</f>
+        <v/>
+      </c>
+      <c r="J64" s="10">
+        <f>SUM(J61:J63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Institutional &amp; other support</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="6" t="n"/>
+      <c r="F66" s="6" t="n"/>
+      <c r="G66" s="6" t="n"/>
+      <c r="H66" s="6" t="n"/>
+      <c r="I66" s="6" t="n"/>
+      <c r="J66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Direct institutional / university support</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="C67" s="8" t="n">
+        <v>320</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="E67" s="7" t="n">
         <v>180</v>
       </c>
-      <c r="H64" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="I64" s="8" t="n">
-        <v>170</v>
-      </c>
-      <c r="J64" s="7" t="n">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Subtotal — Camps, clinics &amp; operations</t>
-        </is>
-      </c>
-      <c r="B65" s="10">
-        <f>SUM(B62:B64)</f>
-        <v/>
-      </c>
-      <c r="C65" s="10">
-        <f>SUM(C62:C64)</f>
-        <v/>
-      </c>
-      <c r="D65" s="10">
-        <f>SUM(D62:D64)</f>
-        <v/>
-      </c>
-      <c r="E65" s="10">
-        <f>SUM(E62:E64)</f>
-        <v/>
-      </c>
-      <c r="F65" s="10">
-        <f>SUM(F62:F64)</f>
-        <v/>
-      </c>
-      <c r="G65" s="10">
-        <f>SUM(G62:G64)</f>
-        <v/>
-      </c>
-      <c r="H65" s="10">
-        <f>SUM(H62:H64)</f>
-        <v/>
-      </c>
-      <c r="I65" s="10">
-        <f>SUM(I62:I64)</f>
-        <v/>
-      </c>
-      <c r="J65" s="10">
-        <f>SUM(J62:J64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>Institutional &amp; other support</t>
-        </is>
-      </c>
-      <c r="B67" s="6" t="n"/>
-      <c r="C67" s="6" t="n"/>
-      <c r="D67" s="6" t="n"/>
-      <c r="E67" s="6" t="n"/>
-      <c r="F67" s="6" t="n"/>
-      <c r="G67" s="6" t="n"/>
-      <c r="H67" s="6" t="n"/>
-      <c r="I67" s="6" t="n"/>
-      <c r="J67" s="6" t="n"/>
+      <c r="F67" s="8" t="n">
+        <v>240</v>
+      </c>
+      <c r="G67" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="H67" s="7" t="n">
+        <v>360</v>
+      </c>
+      <c r="I67" s="8" t="n">
+        <v>530</v>
+      </c>
+      <c r="J67" s="7" t="n">
+        <v>700</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Direct institutional / university support</t>
+          <t xml:space="preserve">   Student-fee allocation</t>
         </is>
       </c>
       <c r="B68" s="7" t="n">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="C68" s="8" t="n">
-        <v>320</v>
+        <v>80</v>
       </c>
       <c r="D68" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E68" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F68" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="H68" s="7" t="n">
+        <v>180</v>
+      </c>
+      <c r="I68" s="8" t="n">
+        <v>290</v>
+      </c>
+      <c r="J68" s="7" t="n">
         <v>400</v>
-      </c>
-      <c r="E68" s="7" t="n">
-        <v>180</v>
-      </c>
-      <c r="F68" s="8" t="n">
-        <v>240</v>
-      </c>
-      <c r="G68" s="7" t="n">
-        <v>300</v>
-      </c>
-      <c r="H68" s="7" t="n">
-        <v>360</v>
-      </c>
-      <c r="I68" s="8" t="n">
-        <v>530</v>
-      </c>
-      <c r="J68" s="7" t="n">
-        <v>700</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Student-fee allocation</t>
+          <t xml:space="preserve">   Direct state / government support</t>
         </is>
       </c>
       <c r="B69" s="7" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="C69" s="8" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="D69" s="7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="I69" s="8" t="n">
-        <v>290</v>
+        <v>420</v>
       </c>
       <c r="J69" s="7" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Direct state / government support</t>
+          <t xml:space="preserve">   Athletics endowment / investment income</t>
         </is>
       </c>
       <c r="B70" s="7" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C70" s="8" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="H70" s="7" t="n">
-        <v>240</v>
+        <v>20</v>
       </c>
       <c r="I70" s="8" t="n">
-        <v>420</v>
+        <v>50</v>
       </c>
       <c r="J70" s="7" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Athletics endowment / investment income</t>
+          <t xml:space="preserve">   Third-party in-kind &amp; third-party-paid comp</t>
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C71" s="8" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D71" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E71" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F71" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="G71" s="7" t="n">
         <v>150</v>
-      </c>
-      <c r="E71" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="F71" s="8" t="n">
-        <v>240</v>
-      </c>
-      <c r="G71" s="7" t="n">
-        <v>400</v>
       </c>
       <c r="H71" s="7" t="n">
         <v>20</v>
       </c>
       <c r="I71" s="8" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="J71" s="7" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Third-party in-kind &amp; third-party-paid comp</t>
+          <t xml:space="preserve">   Other / misc operating revenue</t>
         </is>
       </c>
       <c r="B72" s="7" t="n">
@@ -2588,587 +2586,349 @@
         <v>20</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="H72" s="7" t="n">
         <v>20</v>
       </c>
       <c r="I72" s="8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="J72" s="7" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Other / misc operating revenue</t>
-        </is>
-      </c>
-      <c r="B73" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="C73" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="D73" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E73" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="F73" s="8" t="n">
-        <v>70</v>
-      </c>
-      <c r="G73" s="7" t="n">
-        <v>120</v>
-      </c>
-      <c r="H73" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="I73" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="J73" s="7" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="9" t="inlineStr">
+      <c r="A73" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal — Institutional &amp; other support</t>
         </is>
       </c>
-      <c r="B74" s="10">
-        <f>SUM(B68:B73)</f>
-        <v/>
-      </c>
-      <c r="C74" s="10">
-        <f>SUM(C68:C73)</f>
-        <v/>
-      </c>
-      <c r="D74" s="10">
-        <f>SUM(D68:D73)</f>
-        <v/>
-      </c>
-      <c r="E74" s="10">
-        <f>SUM(E68:E73)</f>
-        <v/>
-      </c>
-      <c r="F74" s="10">
-        <f>SUM(F68:F73)</f>
-        <v/>
-      </c>
-      <c r="G74" s="10">
-        <f>SUM(G68:G73)</f>
-        <v/>
-      </c>
-      <c r="H74" s="10">
-        <f>SUM(H68:H73)</f>
-        <v/>
-      </c>
-      <c r="I74" s="10">
-        <f>SUM(I68:I73)</f>
-        <v/>
-      </c>
-      <c r="J74" s="10">
-        <f>SUM(J68:J73)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="5" t="inlineStr">
-        <is>
-          <t>NIL / rev-share era  (memo — NOT program revenue; see per-line notes)</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="n"/>
-      <c r="C76" s="6" t="n"/>
-      <c r="D76" s="6" t="n"/>
-      <c r="E76" s="6" t="n"/>
-      <c r="F76" s="6" t="n"/>
-      <c r="G76" s="6" t="n"/>
-      <c r="H76" s="6" t="n"/>
-      <c r="I76" s="6" t="n"/>
-      <c r="J76" s="6" t="n"/>
+      <c r="B73" s="10">
+        <f>SUM(B67:B72)</f>
+        <v/>
+      </c>
+      <c r="C73" s="10">
+        <f>SUM(C67:C72)</f>
+        <v/>
+      </c>
+      <c r="D73" s="10">
+        <f>SUM(D67:D72)</f>
+        <v/>
+      </c>
+      <c r="E73" s="10">
+        <f>SUM(E67:E72)</f>
+        <v/>
+      </c>
+      <c r="F73" s="10">
+        <f>SUM(F67:F72)</f>
+        <v/>
+      </c>
+      <c r="G73" s="10">
+        <f>SUM(G67:G72)</f>
+        <v/>
+      </c>
+      <c r="H73" s="10">
+        <f>SUM(H67:H72)</f>
+        <v/>
+      </c>
+      <c r="I73" s="10">
+        <f>SUM(I67:I72)</f>
+        <v/>
+      </c>
+      <c r="J73" s="10">
+        <f>SUM(J67:J72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>PROGRAM REVENUE  (all categories)  = the total baseline</t>
+        </is>
+      </c>
+      <c r="B75" s="12">
+        <f>B12+B19+B26+B37+B44+B51+B58+B64+B73</f>
+        <v/>
+      </c>
+      <c r="C75" s="12">
+        <f>C12+C19+C26+C37+C44+C51+C58+C64+C73</f>
+        <v/>
+      </c>
+      <c r="D75" s="12">
+        <f>D12+D19+D26+D37+D44+D51+D58+D64+D73</f>
+        <v/>
+      </c>
+      <c r="E75" s="12">
+        <f>E12+E19+E26+E37+E44+E51+E58+E64+E73</f>
+        <v/>
+      </c>
+      <c r="F75" s="12">
+        <f>F12+F19+F26+F37+F44+F51+F58+F64+F73</f>
+        <v/>
+      </c>
+      <c r="G75" s="12">
+        <f>G12+G19+G26+G37+G44+G51+G58+G64+G73</f>
+        <v/>
+      </c>
+      <c r="H75" s="12">
+        <f>H12+H19+H26+H37+H44+H51+H58+H64+H73</f>
+        <v/>
+      </c>
+      <c r="I75" s="12">
+        <f>I12+I19+I26+I37+I44+I51+I58+I64+I73</f>
+        <v/>
+      </c>
+      <c r="J75" s="12">
+        <f>J12+J19+J26+J37+J44+J51+J58+J64+J73</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Third-party athlete NIL income (memo — athletes' own $, not SPV rev/cost)</t>
-        </is>
-      </c>
-      <c r="B77" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="C77" s="8" t="n">
-        <v>990</v>
-      </c>
-      <c r="D77" s="7" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E77" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="F77" s="8" t="n">
-        <v>1310</v>
-      </c>
-      <c r="G77" s="7" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H77" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="I77" s="8" t="n">
-        <v>660</v>
-      </c>
-      <c r="J77" s="7" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Athlete marketing / activation (SPV-produced = Bucket 2)</t>
-        </is>
-      </c>
-      <c r="B78" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="C78" s="8" t="n">
-        <v>530</v>
-      </c>
-      <c r="D78" s="7" t="n">
-        <v>800</v>
-      </c>
-      <c r="E78" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="F78" s="8" t="n">
-        <v>660</v>
-      </c>
-      <c r="G78" s="7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H78" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="I78" s="8" t="n">
-        <v>390</v>
-      </c>
-      <c r="J78" s="7" t="n">
-        <v>600</v>
-      </c>
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>SPV ECONOMICS  (Bucket 1 above baseline, 80/20; baseline = total current revenue, one lump)</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="n"/>
+      <c r="C77" s="14" t="n"/>
+      <c r="D77" s="14" t="n"/>
+      <c r="E77" s="14" t="n"/>
+      <c r="F77" s="14" t="n"/>
+      <c r="G77" s="14" t="n"/>
+      <c r="H77" s="14" t="n"/>
+      <c r="I77" s="14" t="n"/>
+      <c r="J77" s="14" t="n"/>
+    </row>
+    <row r="78" ht="26" customHeight="1">
+      <c r="A78" s="15" t="inlineStr"/>
+      <c r="B78" s="15" t="inlineStr">
+        <is>
+          <t>Baseline (total curr.)</t>
+        </is>
+      </c>
+      <c r="C78" s="15" t="inlineStr">
+        <is>
+          <t>Bucket 1 Base w/MC</t>
+        </is>
+      </c>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>Bucket 1 Reach w/MC</t>
+        </is>
+      </c>
+      <c r="E78" s="15" t="inlineStr">
+        <is>
+          <t>SPV 80% Base</t>
+        </is>
+      </c>
+      <c r="F78" s="15" t="inlineStr">
+        <is>
+          <t>SPV 80% Reach</t>
+        </is>
+      </c>
+      <c r="G78" s="15" t="inlineStr">
+        <is>
+          <t>School keeps Base</t>
+        </is>
+      </c>
+      <c r="H78" s="15" t="inlineStr">
+        <is>
+          <t>School keeps Reach</t>
+        </is>
+      </c>
+      <c r="I78" s="15" t="inlineStr"/>
+      <c r="J78" s="15" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   House-settlement rev-share pool (SPV-funded roster COST)</t>
-        </is>
-      </c>
-      <c r="B79" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C79" s="8" t="n">
-        <v>1620</v>
-      </c>
-      <c r="D79" s="7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E79" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="8" t="n">
-        <v>1620</v>
-      </c>
-      <c r="G79" s="7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H79" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I79" s="8" t="n">
-        <v>1620</v>
-      </c>
-      <c r="J79" s="7" t="n">
-        <v>2500</v>
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>St. Joseph's</t>
+        </is>
+      </c>
+      <c r="B79" s="17">
+        <f>B75</f>
+        <v/>
+      </c>
+      <c r="C79" s="17">
+        <f>C12+C19+C37+C51+C58+C64</f>
+        <v/>
+      </c>
+      <c r="D79" s="17">
+        <f>D12+D19+D37+D51+D58+D64</f>
+        <v/>
+      </c>
+      <c r="E79" s="18">
+        <f>0.8*(C79-B79)</f>
+        <v/>
+      </c>
+      <c r="F79" s="19">
+        <f>0.8*(D79-B79)</f>
+        <v/>
+      </c>
+      <c r="G79" s="17">
+        <f>B79+0.2*(C79-B79)</f>
+        <v/>
+      </c>
+      <c r="H79" s="17">
+        <f>B79+0.2*(D79-B79)</f>
+        <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Subtotal — NIL / rev-share era</t>
-        </is>
-      </c>
-      <c r="B80" s="10">
-        <f>SUM(B77:B79)</f>
-        <v/>
-      </c>
-      <c r="C80" s="10">
-        <f>SUM(C77:C79)</f>
-        <v/>
-      </c>
-      <c r="D80" s="10">
-        <f>SUM(D77:D79)</f>
-        <v/>
-      </c>
-      <c r="E80" s="10">
-        <f>SUM(E77:E79)</f>
-        <v/>
-      </c>
-      <c r="F80" s="10">
-        <f>SUM(F77:F79)</f>
-        <v/>
-      </c>
-      <c r="G80" s="10">
-        <f>SUM(G77:G79)</f>
-        <v/>
-      </c>
-      <c r="H80" s="10">
-        <f>SUM(H77:H79)</f>
-        <v/>
-      </c>
-      <c r="I80" s="10">
-        <f>SUM(I77:I79)</f>
-        <v/>
-      </c>
-      <c r="J80" s="10">
-        <f>SUM(J77:J79)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAM REVENUE  (categories 1–9, excl. NIL)  = the total baseline</t>
-        </is>
-      </c>
-      <c r="B82" s="12">
-        <f>B12+B19+B26+B37+B45+B52+B59+B65+B74</f>
-        <v/>
-      </c>
-      <c r="C82" s="12">
-        <f>C12+C19+C26+C37+C45+C52+C59+C65+C74</f>
-        <v/>
-      </c>
-      <c r="D82" s="12">
-        <f>D12+D19+D26+D37+D45+D52+D59+D65+D74</f>
-        <v/>
-      </c>
-      <c r="E82" s="12">
-        <f>E12+E19+E26+E37+E45+E52+E59+E65+E74</f>
-        <v/>
-      </c>
-      <c r="F82" s="12">
-        <f>F12+F19+F26+F37+F45+F52+F59+F65+F74</f>
-        <v/>
-      </c>
-      <c r="G82" s="12">
-        <f>G12+G19+G26+G37+G45+G52+G59+G65+G74</f>
-        <v/>
-      </c>
-      <c r="H82" s="12">
-        <f>H12+H19+H26+H37+H45+H52+H59+H65+H74</f>
-        <v/>
-      </c>
-      <c r="I82" s="12">
-        <f>I12+I19+I26+I37+I45+I52+I59+I65+I74</f>
-        <v/>
-      </c>
-      <c r="J82" s="12">
-        <f>J12+J19+J26+J37+J45+J52+J59+J65+J74</f>
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>Davidson</t>
+        </is>
+      </c>
+      <c r="B80" s="17">
+        <f>E75</f>
+        <v/>
+      </c>
+      <c r="C80" s="17">
+        <f>F12+F19+F37+F51+F58+F64</f>
+        <v/>
+      </c>
+      <c r="D80" s="17">
+        <f>G12+G19+G37+G51+G58+G64</f>
+        <v/>
+      </c>
+      <c r="E80" s="18">
+        <f>0.8*(C80-B80)</f>
+        <v/>
+      </c>
+      <c r="F80" s="19">
+        <f>0.8*(D80-B80)</f>
+        <v/>
+      </c>
+      <c r="G80" s="17">
+        <f>B80+0.2*(C80-B80)</f>
+        <v/>
+      </c>
+      <c r="H80" s="17">
+        <f>B80+0.2*(D80-B80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>Hawaii</t>
+        </is>
+      </c>
+      <c r="B81" s="17">
+        <f>H75</f>
+        <v/>
+      </c>
+      <c r="C81" s="17">
+        <f>I12+I19+I37+I51+I58+I64</f>
+        <v/>
+      </c>
+      <c r="D81" s="17">
+        <f>J12+J19+J37+J51+J58+J64</f>
+        <v/>
+      </c>
+      <c r="E81" s="18">
+        <f>0.8*(C81-B81)</f>
+        <v/>
+      </c>
+      <c r="F81" s="19">
+        <f>0.8*(D81-B81)</f>
+        <v/>
+      </c>
+      <c r="G81" s="17">
+        <f>B81+0.2*(C81-B81)</f>
+        <v/>
+      </c>
+      <c r="H81" s="17">
+        <f>B81+0.2*(D81-B81)</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="13" t="inlineStr">
-        <is>
-          <t>NIL / rev-share funding  (memo — SPV-funded cost)</t>
-        </is>
-      </c>
-      <c r="B83" s="14">
-        <f>B80</f>
-        <v/>
-      </c>
-      <c r="C83" s="14">
-        <f>C80</f>
-        <v/>
-      </c>
-      <c r="D83" s="14">
-        <f>D80</f>
-        <v/>
-      </c>
-      <c r="E83" s="14">
-        <f>E80</f>
-        <v/>
-      </c>
-      <c r="F83" s="14">
-        <f>F80</f>
-        <v/>
-      </c>
-      <c r="G83" s="14">
-        <f>G80</f>
-        <v/>
-      </c>
-      <c r="H83" s="14">
-        <f>H80</f>
-        <v/>
-      </c>
-      <c r="I83" s="14">
-        <f>I80</f>
-        <v/>
-      </c>
-      <c r="J83" s="14">
-        <f>J80</f>
-        <v/>
+      <c r="A83" s="20" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+      <c r="B83" s="21" t="n"/>
+      <c r="C83" s="21" t="n"/>
+      <c r="D83" s="21" t="n"/>
+      <c r="E83" s="21" t="n"/>
+      <c r="F83" s="21" t="n"/>
+      <c r="G83" s="21" t="n"/>
+      <c r="H83" s="21" t="n"/>
+      <c r="I83" s="21" t="n"/>
+      <c r="J83" s="21" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="22" t="inlineStr">
+        <is>
+          <t>Reach = full-attachment estimate (celebrity + Netflix + top-10 roster + deep tournament run all landing). Base = Current + a conservative fraction of that uplift (55-65% on commercial lines).</t>
+        </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="15" t="inlineStr">
-        <is>
-          <t>SPV ECONOMICS  (Bucket 1 above baseline, 80/20; baseline = total current revenue, one lump)</t>
-        </is>
-      </c>
-      <c r="B85" s="16" t="n"/>
-      <c r="C85" s="16" t="n"/>
-      <c r="D85" s="16" t="n"/>
-      <c r="E85" s="16" t="n"/>
-      <c r="F85" s="16" t="n"/>
-      <c r="G85" s="16" t="n"/>
-      <c r="H85" s="16" t="n"/>
-      <c r="I85" s="16" t="n"/>
-      <c r="J85" s="16" t="n"/>
-    </row>
-    <row r="86" ht="26" customHeight="1">
-      <c r="A86" s="17" t="inlineStr"/>
-      <c r="B86" s="17" t="inlineStr">
-        <is>
-          <t>Baseline (total curr.)</t>
-        </is>
-      </c>
-      <c r="C86" s="17" t="inlineStr">
-        <is>
-          <t>Bucket 1 Base w/MC</t>
-        </is>
-      </c>
-      <c r="D86" s="17" t="inlineStr">
-        <is>
-          <t>Bucket 1 Reach w/MC</t>
-        </is>
-      </c>
-      <c r="E86" s="17" t="inlineStr">
-        <is>
-          <t>SPV 80% Base</t>
-        </is>
-      </c>
-      <c r="F86" s="17" t="inlineStr">
-        <is>
-          <t>SPV 80% Reach</t>
-        </is>
-      </c>
-      <c r="G86" s="17" t="inlineStr">
-        <is>
-          <t>School keeps Base</t>
-        </is>
-      </c>
-      <c r="H86" s="17" t="inlineStr">
-        <is>
-          <t>School keeps Reach</t>
-        </is>
-      </c>
-      <c r="I86" s="17" t="inlineStr"/>
-      <c r="J86" s="17" t="inlineStr"/>
+      <c r="A85" s="22" t="inlineStr">
+        <is>
+          <t>MECHANIC (simplified): baseline = the school's TOTAL current program revenue (one lump, the green PROGRAM REVENUE row). The school keeps the first [baseline] dollars; everything in Bucket 1 above the baseline splits 80/20 (SPV 80, school 20). Not itemized line-by-line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="22" t="inlineStr">
+        <is>
+          <t>Bucket 1 = the school's commercial revenue with MC (Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps). SPV 80% = 0.8 x (Bucket 1 w/MC - total baseline). School keeps baseline + 20% of the excess.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="18" t="inlineStr">
-        <is>
-          <t>St. Joseph's</t>
-        </is>
-      </c>
-      <c r="B87" s="19">
-        <f>B82</f>
-        <v/>
-      </c>
-      <c r="C87" s="19">
-        <f>C12+C19+C37+C52+C59+C65</f>
-        <v/>
-      </c>
-      <c r="D87" s="19">
-        <f>D12+D19+D37+D52+D59+D65</f>
-        <v/>
-      </c>
-      <c r="E87" s="20">
-        <f>0.8*(C87-B87)</f>
-        <v/>
-      </c>
-      <c r="F87" s="21">
-        <f>0.8*(D87-B87)</f>
-        <v/>
-      </c>
-      <c r="G87" s="19">
-        <f>B87+0.2*(C87-B87)</f>
-        <v/>
-      </c>
-      <c r="H87" s="19">
-        <f>B87+0.2*(D87-B87)</f>
-        <v/>
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>Postseason gate: conf tournament &amp; NCAA tournament ticket revenue goes to the CONFERENCE / NCAA, not the school — line reduced to a small allotment margin only.</t>
+        </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="18" t="inlineStr">
-        <is>
-          <t>Davidson</t>
-        </is>
-      </c>
-      <c r="B88" s="19">
-        <f>E82</f>
-        <v/>
-      </c>
-      <c r="C88" s="19">
-        <f>F12+F19+F37+F52+F59+F65</f>
-        <v/>
-      </c>
-      <c r="D88" s="19">
-        <f>G12+G19+G37+G52+G59+G65</f>
-        <v/>
-      </c>
-      <c r="E88" s="20">
-        <f>0.8*(C88-B88)</f>
-        <v/>
-      </c>
-      <c r="F88" s="21">
-        <f>0.8*(D88-B88)</f>
-        <v/>
-      </c>
-      <c r="G88" s="19">
-        <f>B88+0.2*(C88-B88)</f>
-        <v/>
-      </c>
-      <c r="H88" s="19">
-        <f>B88+0.2*(D88-B88)</f>
-        <v/>
+      <c r="A88" s="22" t="inlineStr">
+        <is>
+          <t>Concessions &amp; parking DO grow: marquee home games are relocated to big arenas (St. Joe's -&gt; Xfinity Mobile Arena) where the school is the home promoter and keeps/splits the ancillaries.</t>
+        </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="18" t="inlineStr">
-        <is>
-          <t>Hawaii</t>
-        </is>
-      </c>
-      <c r="B89" s="19">
-        <f>H82</f>
-        <v/>
-      </c>
-      <c r="C89" s="19">
-        <f>I12+I19+I37+I52+I59+I65</f>
-        <v/>
-      </c>
-      <c r="D89" s="19">
-        <f>J12+J19+J37+J52+J59+J65</f>
-        <v/>
-      </c>
-      <c r="E89" s="20">
-        <f>0.8*(C89-B89)</f>
-        <v/>
-      </c>
-      <c r="F89" s="21">
-        <f>0.8*(D89-B89)</f>
-        <v/>
-      </c>
-      <c r="G89" s="19">
-        <f>B89+0.2*(C89-B89)</f>
-        <v/>
-      </c>
-      <c r="H89" s="19">
-        <f>B89+0.2*(D89-B89)</f>
-        <v/>
+      <c r="A89" s="22" t="inlineStr">
+        <is>
+          <t>MMR/Learfield: MC-originated signage/MMR-scope sponsorship is negotiated 85% to the program / 15% to Learfield, and the 85% is booked HERE in Bucket 1 — then runs through the 80/20 like all team revenue. Only purely on-screen / in-documentary sponsorship sits in Bucket 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="22" t="inlineStr">
+        <is>
+          <t>Apparel shoe contract held FLAT — multi-year locked deal, no mid-term jump (renewal upside later). Licensing/merch/retail still grow (flexible).</t>
+        </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="22" t="inlineStr">
         <is>
-          <t>NOTES</t>
-        </is>
-      </c>
-      <c r="B91" s="23" t="n"/>
-      <c r="C91" s="23" t="n"/>
-      <c r="D91" s="23" t="n"/>
-      <c r="E91" s="23" t="n"/>
-      <c r="F91" s="23" t="n"/>
-      <c r="G91" s="23" t="n"/>
-      <c r="H91" s="23" t="n"/>
-      <c r="I91" s="23" t="n"/>
-      <c r="J91" s="23" t="n"/>
+          <t>Excluded from this sheet (none are team revenue): third-party athlete NIL income = athletes' own earnings (a recruiting benefit); athlete marketing/activation = Bucket 2 content; House rev-share pool + booster collective = SPV-funded roster COST (part of the $15M).</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="24" t="inlineStr">
-        <is>
-          <t>Reach = full-attachment estimate (celebrity + Netflix + top-10 roster + deep tournament run all landing). Base = Current + a conservative fraction of that uplift (55-65% on commercial lines).</t>
+      <c r="A92" s="22" t="inlineStr">
+        <is>
+          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, athlete-marketing/activation, international + format. Roughly recoups the $15M SPV cost.</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="24" t="inlineStr">
-        <is>
-          <t>MECHANIC (simplified): baseline = the school's TOTAL current program revenue (one lump, the green PROGRAM REVENUE row). The school keeps the first [baseline] dollars; everything in Bucket 1 above the baseline splits 80/20 (SPV 80, school 20). Not itemized line-by-line.</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="24" t="inlineStr">
-        <is>
-          <t>Bucket 1 = the school's commercial revenue with MC (Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps). SPV 80% = 0.8 x (Bucket 1 w/MC - total baseline). School keeps baseline + 20% of the excess.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="24" t="inlineStr">
-        <is>
-          <t>Postseason gate: conf tournament &amp; NCAA tournament ticket revenue goes to the CONFERENCE / NCAA, not the school — line reduced to a small allotment margin only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="24" t="inlineStr">
-        <is>
-          <t>Concessions &amp; parking DO grow: marquee home games are relocated to big arenas (St. Joe's -&gt; Xfinity Mobile Arena) where the school is the home promoter and keeps/splits the ancillaries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="24" t="inlineStr">
-        <is>
-          <t>MMR/Learfield: MC-originated signage/MMR-scope sponsorship is negotiated 85% to the program / 15% to Learfield, and the 85% is booked HERE in Bucket 1 — then runs through the 80/20 like all team revenue. Only purely on-screen / in-documentary sponsorship sits in Bucket 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="24" t="inlineStr">
-        <is>
-          <t>Apparel shoe contract held FLAT — multi-year locked deal, no mid-term jump (renewal upside later). Licensing/merch/retail still grow (flexible).</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="24" t="inlineStr">
-        <is>
-          <t>NIL memo lines are NOT program revenue: (1) third-party athlete NIL income = athletes' own earnings (a recruiting benefit, not SPV rev/cost); (2) athlete marketing/activation = SPV-produced Bucket 2; (3) House rev-share pool = SPV-funded roster COST.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="24" t="inlineStr">
-        <is>
-          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, athlete-marketing/activation, international + format. Roughly recoups the $15M SPV cost.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="24" t="inlineStr">
+      <c r="A93" s="22" t="inlineStr">
         <is>
           <t>Marquee-game relocation assumed: St. Joe's -&gt; Xfinity Mobile Arena (19k); Davidson -&gt; Spectrum Center (19k); Hawaii carried by its 10,300 arena + Diamond Head Classic. All figures ESTIMATES in $000s.</t>
         </is>
@@ -3176,19 +2936,19 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A99:J99"/>
+    <mergeCell ref="A85:J85"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A84:J84"/>
     <mergeCell ref="A93:J93"/>
-    <mergeCell ref="A94:J94"/>
-    <mergeCell ref="A97:J97"/>
-    <mergeCell ref="A100:J100"/>
+    <mergeCell ref="A89:J89"/>
+    <mergeCell ref="A88:J88"/>
     <mergeCell ref="A92:J92"/>
-    <mergeCell ref="A95:J95"/>
-    <mergeCell ref="A96:J96"/>
+    <mergeCell ref="A91:J91"/>
+    <mergeCell ref="A87:J87"/>
     <mergeCell ref="H2:J2"/>
-    <mergeCell ref="A101:J101"/>
-    <mergeCell ref="A98:J98"/>
+    <mergeCell ref="A86:J86"/>
+    <mergeCell ref="A90:J90"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3243,13 +3003,13 @@
           <t xml:space="preserve">   Streaming series (10 hrs @ $1.0M sold / $0.6M cost)</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n">
+      <c r="B4" s="17" t="n">
         <v>3200</v>
       </c>
-      <c r="C4" s="19" t="n">
+      <c r="C4" s="17" t="n">
         <v>5000</v>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="23" t="inlineStr">
         <is>
           <t>$400k/hr margin before intl/format</t>
         </is>
@@ -3261,13 +3021,13 @@
           <t xml:space="preserve">   International + format windows</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="17" t="n">
         <v>1500</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="17" t="n">
         <v>5000</v>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="23" t="inlineStr">
         <is>
           <t>durable franchise asset; grows w/ library</t>
         </is>
@@ -3279,13 +3039,13 @@
           <t xml:space="preserve">   Live games (3 @ &gt;$1.0M rev / $0.3M cost each)</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="17" t="n">
         <v>2100</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="17" t="n">
         <v>4000</v>
       </c>
-      <c r="D6" s="25" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>school-owned neutral/non-conf games</t>
         </is>
@@ -3297,13 +3057,13 @@
           <t xml:space="preserve">   National presenting sponsor + premium patch</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="17" t="n">
         <v>3000</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="17" t="n">
         <v>8000</v>
       </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="D7" s="23" t="inlineStr">
         <is>
           <t>on-screen/in-documentary sponsor; SPV IP, not school MMR</t>
         </is>
@@ -3315,20 +3075,20 @@
           <t xml:space="preserve">   Content engine / athlete marketing &amp; activation</t>
         </is>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="17" t="n">
         <v>500</v>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C8" s="17" t="n">
         <v>1500</v>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>SPV-produced branded content; players' NIL contracted</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">   Bucket 2 total (SPV)</t>
         </is>
@@ -3343,223 +3103,223 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>FULL SPV PICTURE — single season  (Bucket 1 share + Bucket 2 − $15M SPV cost)</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n"/>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="16" t="n"/>
+      <c r="B11" s="14" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>School</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Bkt1 SPV Base</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>+ Bkt2 Base</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>− SPV cost</t>
         </is>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="15">
         <f> SPV net Base</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>St. Joseph's</t>
         </is>
       </c>
-      <c r="B13" s="19">
-        <f>'Three-School Projection'!E87</f>
-        <v/>
-      </c>
-      <c r="C13" s="19">
+      <c r="B13" s="17">
+        <f>'Three-School Projection'!E79</f>
+        <v/>
+      </c>
+      <c r="C13" s="17">
         <f>B9</f>
         <v/>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="17" t="n">
         <v>-15000</v>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="19">
         <f>B13+C13+D13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Davidson</t>
         </is>
       </c>
-      <c r="B14" s="19">
-        <f>'Three-School Projection'!E88</f>
-        <v/>
-      </c>
-      <c r="C14" s="19">
+      <c r="B14" s="17">
+        <f>'Three-School Projection'!E80</f>
+        <v/>
+      </c>
+      <c r="C14" s="17">
         <f>B9</f>
         <v/>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="17" t="n">
         <v>-15000</v>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="19">
         <f>B14+C14+D14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Hawaii</t>
         </is>
       </c>
-      <c r="B15" s="19">
-        <f>'Three-School Projection'!E89</f>
-        <v/>
-      </c>
-      <c r="C15" s="19">
+      <c r="B15" s="17">
+        <f>'Three-School Projection'!E81</f>
+        <v/>
+      </c>
+      <c r="C15" s="17">
         <f>B9</f>
         <v/>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="17" t="n">
         <v>-15000</v>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="19">
         <f>B15+C15+D15</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>School</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>Bkt1 SPV Reach</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>+ Bkt2 Reach</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>− SPV cost</t>
         </is>
       </c>
-      <c r="E17" s="17">
+      <c r="E17" s="15">
         <f> SPV net Reach</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>St. Joseph's</t>
         </is>
       </c>
-      <c r="B18" s="19">
-        <f>'Three-School Projection'!F87</f>
-        <v/>
-      </c>
-      <c r="C18" s="19">
+      <c r="B18" s="17">
+        <f>'Three-School Projection'!F79</f>
+        <v/>
+      </c>
+      <c r="C18" s="17">
         <f>C9</f>
         <v/>
       </c>
-      <c r="D18" s="19" t="n">
+      <c r="D18" s="17" t="n">
         <v>-15000</v>
       </c>
-      <c r="E18" s="21">
+      <c r="E18" s="19">
         <f>B18+C18+D18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Davidson</t>
         </is>
       </c>
-      <c r="B19" s="19">
-        <f>'Three-School Projection'!F88</f>
-        <v/>
-      </c>
-      <c r="C19" s="19">
+      <c r="B19" s="17">
+        <f>'Three-School Projection'!F80</f>
+        <v/>
+      </c>
+      <c r="C19" s="17">
         <f>C9</f>
         <v/>
       </c>
-      <c r="D19" s="19" t="n">
+      <c r="D19" s="17" t="n">
         <v>-15000</v>
       </c>
-      <c r="E19" s="21">
+      <c r="E19" s="19">
         <f>B19+C19+D19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Hawaii</t>
         </is>
       </c>
-      <c r="B20" s="19">
-        <f>'Three-School Projection'!F89</f>
-        <v/>
-      </c>
-      <c r="C20" s="19">
+      <c r="B20" s="17">
+        <f>'Three-School Projection'!F81</f>
+        <v/>
+      </c>
+      <c r="C20" s="17">
         <f>C9</f>
         <v/>
       </c>
-      <c r="D20" s="19" t="n">
+      <c r="D20" s="17" t="n">
         <v>-15000</v>
       </c>
-      <c r="E20" s="21">
+      <c r="E20" s="19">
         <f>B20+C20+D20</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>Bucket 2 is 100% SPV and never touches the school sheet or the 80/20 split.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>Series &amp; live-game costs are already netted in their lines (EverWonder finances production, recoups cost+10%). The $15M SPV cost = roster/NIL + ops.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>Bucket 2 = purely on-screen / in-documentary revenue. MC-originated MMR/signage sponsorship is NOT here — it's booked in Bucket 1 (school sheet) at 85% kept / 15% Learfield, then runs through the 80/20.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>Per-school variance is minor (national platform) — Davidson skews high via the Curry anchor. Reach is the optimistic ceiling; underwrite on Base.</t>
         </is>

</xml_diff>

<commit_message>
Clarify activation is already in MMR/Bucket 2; relabel content-engine line to avoid double-count
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -2916,7 +2916,7 @@
     <row r="91">
       <c r="A91" s="22" t="inlineStr">
         <is>
-          <t>Excluded from this sheet (none are team revenue): third-party athlete NIL income = athletes' own earnings (a recruiting benefit); athlete marketing/activation = Bucket 2 content; House rev-share pool + booster collective = SPV-funded roster COST (part of the $15M).</t>
+          <t>Excluded from this sheet (none are a separate team-revenue stream): third-party athlete NIL income = athletes' own earnings (a recruiting benefit); 'activation' revenue is already inside MMR/sponsorship (in-arena) and Bucket 2 (on-screen); the athlete's NIL cut is a COST; House rev-share pool + booster collective = SPV-funded roster COST (part of the $15M).</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Content engine / athlete marketing &amp; activation</t>
+          <t xml:space="preserve">   Content engine (social/digital ads + branded integrations)</t>
         </is>
       </c>
       <c r="B8" s="17" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>SPV-produced branded content; players' NIL contracted</t>
+          <t>SPV content monetization only; in-arena activation is in Bkt1 MMR; athlete NIL is a cost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Per-bucket SPV split: commercial 80/20, donor 50/50, NCAA units 50/50; conference base = 100% school
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -56,12 +56,12 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00404040"/>
+      <color rgb="00595959"/>
       <sz val="9"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="00404040"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -156,9 +156,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2690,7 +2690,7 @@
     <row r="77">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>SPV ECONOMICS  (Bucket 1 above baseline, 80/20; baseline = total current revenue, one lump)</t>
+          <t>SPV ECONOMICS — per-bucket split of the increase over baseline (school keeps 100% of baseline)</t>
         </is>
       </c>
       <c r="B77" s="14" t="n"/>
@@ -2707,40 +2707,44 @@
       <c r="A78" s="15" t="inlineStr"/>
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>Baseline (total curr.)</t>
+          <t>Comm 80% Base</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Bucket 1 Base w/MC</t>
+          <t>Donor 50% Base</t>
         </is>
       </c>
       <c r="D78" s="15" t="inlineStr">
         <is>
-          <t>Bucket 1 Reach w/MC</t>
+          <t>Units 50% Base</t>
         </is>
       </c>
       <c r="E78" s="15" t="inlineStr">
         <is>
-          <t>SPV 80% Base</t>
+          <t>SPV Base</t>
         </is>
       </c>
       <c r="F78" s="15" t="inlineStr">
         <is>
-          <t>SPV 80% Reach</t>
+          <t>Comm 80% Reach</t>
         </is>
       </c>
       <c r="G78" s="15" t="inlineStr">
         <is>
-          <t>School keeps Base</t>
+          <t>Donor 50% Reach</t>
         </is>
       </c>
       <c r="H78" s="15" t="inlineStr">
         <is>
-          <t>School keeps Reach</t>
-        </is>
-      </c>
-      <c r="I78" s="15" t="inlineStr"/>
+          <t>Units 50% Reach</t>
+        </is>
+      </c>
+      <c r="I78" s="15" t="inlineStr">
+        <is>
+          <t>SPV Reach</t>
+        </is>
+      </c>
       <c r="J78" s="15" t="inlineStr"/>
     </row>
     <row r="79">
@@ -2750,31 +2754,35 @@
         </is>
       </c>
       <c r="B79" s="17">
-        <f>B75</f>
+        <f>0.8*((C12+C19+C37+C51+C58+C64)-(B12+B19+B37+B51+B58+B64))</f>
         <v/>
       </c>
       <c r="C79" s="17">
-        <f>C12+C19+C37+C51+C58+C64</f>
+        <f>0.5*(C44-B44)</f>
         <v/>
       </c>
       <c r="D79" s="17">
-        <f>D12+D19+D37+D51+D58+D64</f>
+        <f>0.5*(C24-B24)</f>
         <v/>
       </c>
       <c r="E79" s="18">
-        <f>0.8*(C79-B79)</f>
-        <v/>
-      </c>
-      <c r="F79" s="19">
-        <f>0.8*(D79-B79)</f>
+        <f>B79+C79+D79</f>
+        <v/>
+      </c>
+      <c r="F79" s="17">
+        <f>0.8*((D12+D19+D37+D51+D58+D64)-(B12+B19+B37+B51+B58+B64))</f>
         <v/>
       </c>
       <c r="G79" s="17">
-        <f>B79+0.2*(C79-B79)</f>
+        <f>0.5*(D44-B44)</f>
         <v/>
       </c>
       <c r="H79" s="17">
-        <f>B79+0.2*(D79-B79)</f>
+        <f>0.5*(D24-B24)</f>
+        <v/>
+      </c>
+      <c r="I79" s="19">
+        <f>F79+G79+H79</f>
         <v/>
       </c>
     </row>
@@ -2785,31 +2793,35 @@
         </is>
       </c>
       <c r="B80" s="17">
-        <f>E75</f>
+        <f>0.8*((F12+F19+F37+F51+F58+F64)-(E12+E19+E37+E51+E58+E64))</f>
         <v/>
       </c>
       <c r="C80" s="17">
-        <f>F12+F19+F37+F51+F58+F64</f>
+        <f>0.5*(F44-E44)</f>
         <v/>
       </c>
       <c r="D80" s="17">
-        <f>G12+G19+G37+G51+G58+G64</f>
+        <f>0.5*(F24-E24)</f>
         <v/>
       </c>
       <c r="E80" s="18">
-        <f>0.8*(C80-B80)</f>
-        <v/>
-      </c>
-      <c r="F80" s="19">
-        <f>0.8*(D80-B80)</f>
+        <f>B80+C80+D80</f>
+        <v/>
+      </c>
+      <c r="F80" s="17">
+        <f>0.8*((G12+G19+G37+G51+G58+G64)-(E12+E19+E37+E51+E58+E64))</f>
         <v/>
       </c>
       <c r="G80" s="17">
-        <f>B80+0.2*(C80-B80)</f>
+        <f>0.5*(G44-E44)</f>
         <v/>
       </c>
       <c r="H80" s="17">
-        <f>B80+0.2*(D80-B80)</f>
+        <f>0.5*(G24-E24)</f>
+        <v/>
+      </c>
+      <c r="I80" s="19">
+        <f>F80+G80+H80</f>
         <v/>
       </c>
     </row>
@@ -2820,115 +2832,126 @@
         </is>
       </c>
       <c r="B81" s="17">
-        <f>H75</f>
+        <f>0.8*((I12+I19+I37+I51+I58+I64)-(H12+H19+H37+H51+H58+H64))</f>
         <v/>
       </c>
       <c r="C81" s="17">
-        <f>I12+I19+I37+I51+I58+I64</f>
+        <f>0.5*(I44-H44)</f>
         <v/>
       </c>
       <c r="D81" s="17">
-        <f>J12+J19+J37+J51+J58+J64</f>
+        <f>0.5*(I24-H24)</f>
         <v/>
       </c>
       <c r="E81" s="18">
-        <f>0.8*(C81-B81)</f>
-        <v/>
-      </c>
-      <c r="F81" s="19">
-        <f>0.8*(D81-B81)</f>
+        <f>B81+C81+D81</f>
+        <v/>
+      </c>
+      <c r="F81" s="17">
+        <f>0.8*((J12+J19+J37+J51+J58+J64)-(H12+H19+H37+H51+H58+H64))</f>
         <v/>
       </c>
       <c r="G81" s="17">
-        <f>B81+0.2*(C81-B81)</f>
+        <f>0.5*(J44-H44)</f>
         <v/>
       </c>
       <c r="H81" s="17">
-        <f>B81+0.2*(D81-B81)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="20" t="inlineStr">
+        <f>0.5*(J24-H24)</f>
+        <v/>
+      </c>
+      <c r="I81" s="19">
+        <f>F81+G81+H81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Conference base/media distribution + institutional support = 100% school (fixed contract, no MC increment; not claimed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="21" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
-      <c r="B83" s="21" t="n"/>
-      <c r="C83" s="21" t="n"/>
-      <c r="D83" s="21" t="n"/>
-      <c r="E83" s="21" t="n"/>
-      <c r="F83" s="21" t="n"/>
-      <c r="G83" s="21" t="n"/>
-      <c r="H83" s="21" t="n"/>
-      <c r="I83" s="21" t="n"/>
-      <c r="J83" s="21" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="22" t="inlineStr">
+      <c r="B84" s="22" t="n"/>
+      <c r="C84" s="22" t="n"/>
+      <c r="D84" s="22" t="n"/>
+      <c r="E84" s="22" t="n"/>
+      <c r="F84" s="22" t="n"/>
+      <c r="G84" s="22" t="n"/>
+      <c r="H84" s="22" t="n"/>
+      <c r="I84" s="22" t="n"/>
+      <c r="J84" s="22" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="23" t="inlineStr">
         <is>
           <t>Reach = full-attachment estimate (celebrity + Netflix + top-10 roster + deep tournament run all landing). Base = Current + a conservative fraction of that uplift (55-65% on commercial lines).</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="22" t="inlineStr">
-        <is>
-          <t>MECHANIC (simplified): baseline = the school's TOTAL current program revenue (one lump, the green PROGRAM REVENUE row). The school keeps the first [baseline] dollars; everything in Bucket 1 above the baseline splits 80/20 (SPV 80, school 20). Not itemized line-by-line.</t>
-        </is>
-      </c>
-    </row>
     <row r="86">
-      <c r="A86" s="22" t="inlineStr">
-        <is>
-          <t>Bucket 1 = the school's commercial revenue with MC (Ticketing, Media, Sponsorship/MMR, Apparel/Licensing, Guarantees, Camps). SPV 80% = 0.8 x (Bucket 1 w/MC - total baseline). School keeps baseline + 20% of the excess.</t>
+      <c r="A86" s="23" t="inlineStr">
+        <is>
+          <t>MECHANIC: the school keeps 100% of its baseline (current column). The INCREASE over baseline is split per bucket: commercial 80/20, donor 50/50, NCAA units 50/50. Conference base/media + institutional support are NOT shared (fixed contracts, no MC-created increment, likely not assignable).</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="22" t="inlineStr">
+      <c r="A87" s="23" t="inlineStr">
+        <is>
+          <t>Commercial = Ticketing, Media, Sponsorship/MMR (incl. MC-originated), Apparel/Licensing, Guarantees, Camps. NCAA units are shared because the MC-manufactured tournament run earns them (pooled/lagged, so modest). Realignment upside on conference money = the separate Promotion SPV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="23" t="inlineStr">
         <is>
           <t>Postseason gate: conf tournament &amp; NCAA tournament ticket revenue goes to the CONFERENCE / NCAA, not the school — line reduced to a small allotment margin only.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="22" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="23" t="inlineStr">
         <is>
           <t>Concessions &amp; parking DO grow: marquee home games are relocated to big arenas (St. Joe's -&gt; Xfinity Mobile Arena) where the school is the home promoter and keeps/splits the ancillaries.</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="22" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="23" t="inlineStr">
         <is>
           <t>MMR/Learfield: MC-originated signage/MMR-scope sponsorship is negotiated 85% to the program / 15% to Learfield, and the 85% is booked HERE in Bucket 1 — then runs through the 80/20 like all team revenue. Only purely on-screen / in-documentary sponsorship sits in Bucket 2.</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="22" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="23" t="inlineStr">
         <is>
           <t>Apparel shoe contract held FLAT — multi-year locked deal, no mid-term jump (renewal upside later). Licensing/merch/retail still grow (flexible).</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="22" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="23" t="inlineStr">
         <is>
           <t>Excluded from this sheet (none are a separate team-revenue stream): third-party athlete NIL income = athletes' own earnings (a recruiting benefit); 'activation' revenue is already inside MMR/sponsorship (in-arena) and Bucket 2 (on-screen); the athlete's NIL cut is a COST; House rev-share pool + booster collective = SPV-funded roster COST (part of the $15M).</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="22" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="23" t="inlineStr">
         <is>
           <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, athlete-marketing/activation, international + format. Roughly recoups the $15M SPV cost.</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="22" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="23" t="inlineStr">
         <is>
           <t>Marquee-game relocation assumed: St. Joe's -&gt; Xfinity Mobile Arena (19k); Davidson -&gt; Spectrum Center (19k); Hawaii carried by its 10,300 arena + Diamond Head Classic. All figures ESTIMATES in $000s.</t>
         </is>
@@ -2939,8 +2962,8 @@
     <mergeCell ref="A85:J85"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="E2:G2"/>
-    <mergeCell ref="A84:J84"/>
     <mergeCell ref="A93:J93"/>
+    <mergeCell ref="A94:J94"/>
     <mergeCell ref="A89:J89"/>
     <mergeCell ref="A88:J88"/>
     <mergeCell ref="A92:J92"/>
@@ -3009,7 +3032,7 @@
       <c r="C4" s="17" t="n">
         <v>5000</v>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>$400k/hr margin before intl/format</t>
         </is>
@@ -3027,7 +3050,7 @@
       <c r="C5" s="17" t="n">
         <v>5000</v>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>durable franchise asset; grows w/ library</t>
         </is>
@@ -3045,7 +3068,7 @@
       <c r="C6" s="17" t="n">
         <v>4000</v>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>school-owned neutral/non-conf games</t>
         </is>
@@ -3063,7 +3086,7 @@
       <c r="C7" s="17" t="n">
         <v>8000</v>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>on-screen/in-documentary sponsor; SPV IP, not school MMR</t>
         </is>
@@ -3081,7 +3104,7 @@
       <c r="C8" s="17" t="n">
         <v>1500</v>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>SPV content monetization only; in-arena activation is in Bkt1 MMR; athlete NIL is a cost</t>
         </is>
@@ -3121,7 +3144,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Bkt1 SPV Base</t>
+          <t>SPV share Base</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
@@ -3213,7 +3236,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>Bkt1 SPV Reach</t>
+          <t>SPV share Reach</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
@@ -3238,7 +3261,7 @@
         </is>
       </c>
       <c r="B18" s="17">
-        <f>'Three-School Projection'!F79</f>
+        <f>'Three-School Projection'!I79</f>
         <v/>
       </c>
       <c r="C18" s="17">
@@ -3260,7 +3283,7 @@
         </is>
       </c>
       <c r="B19" s="17">
-        <f>'Three-School Projection'!F80</f>
+        <f>'Three-School Projection'!I80</f>
         <v/>
       </c>
       <c r="C19" s="17">
@@ -3282,7 +3305,7 @@
         </is>
       </c>
       <c r="B20" s="17">
-        <f>'Three-School Projection'!F81</f>
+        <f>'Three-School Projection'!I81</f>
         <v/>
       </c>
       <c r="C20" s="17">
@@ -3298,28 +3321,28 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>Bucket 2 is 100% SPV and never touches the school sheet or the 80/20 split.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>Series &amp; live-game costs are already netted in their lines (EverWonder finances production, recoups cost+10%). The $15M SPV cost = roster/NIL + ops.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>Bucket 2 = purely on-screen / in-documentary revenue. MC-originated MMR/signage sponsorship is NOT here — it's booked in Bucket 1 (school sheet) at 85% kept / 15% Learfield, then runs through the 80/20.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>Per-school variance is minor (national platform) — Davidson skews high via the Curry anchor. Reach is the optimistic ceiling; underwrite on Base.</t>
         </is>

</xml_diff>

<commit_message>
Uniform 80% on all above-baseline revenue (donor 50/50); school collects, remits secondarily
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -2690,7 +2690,7 @@
     <row r="77">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>SPV ECONOMICS — per-bucket split of the increase over baseline (school keeps 100% of baseline)</t>
+          <t>SPV ECONOMICS — school keeps 100% of baseline; SPV gets 80% of ALL revenue above baseline (donor 50/50)</t>
         </is>
       </c>
       <c r="B77" s="14" t="n"/>
@@ -2703,11 +2703,11 @@
       <c r="I77" s="14" t="n"/>
       <c r="J77" s="14" t="n"/>
     </row>
-    <row r="78" ht="26" customHeight="1">
+    <row r="78" ht="32" customHeight="1">
       <c r="A78" s="15" t="inlineStr"/>
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>Comm 80% Base</t>
+          <t>Above-baseline ex-donor 80% Base</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
@@ -2717,34 +2717,26 @@
       </c>
       <c r="D78" s="15" t="inlineStr">
         <is>
-          <t>Units 50% Base</t>
+          <t>SPV Base</t>
         </is>
       </c>
       <c r="E78" s="15" t="inlineStr">
         <is>
-          <t>SPV Base</t>
+          <t>Above-baseline ex-donor 80% Reach</t>
         </is>
       </c>
       <c r="F78" s="15" t="inlineStr">
         <is>
-          <t>Comm 80% Reach</t>
+          <t>Donor 50% Reach</t>
         </is>
       </c>
       <c r="G78" s="15" t="inlineStr">
         <is>
-          <t>Donor 50% Reach</t>
-        </is>
-      </c>
-      <c r="H78" s="15" t="inlineStr">
-        <is>
-          <t>Units 50% Reach</t>
-        </is>
-      </c>
-      <c r="I78" s="15" t="inlineStr">
-        <is>
           <t>SPV Reach</t>
         </is>
       </c>
+      <c r="H78" s="15" t="inlineStr"/>
+      <c r="I78" s="15" t="inlineStr"/>
       <c r="J78" s="15" t="inlineStr"/>
     </row>
     <row r="79">
@@ -2754,35 +2746,27 @@
         </is>
       </c>
       <c r="B79" s="17">
-        <f>0.8*((C12+C19+C37+C51+C58+C64)-(B12+B19+B37+B51+B58+B64))</f>
+        <f>0.8*((C12+C19+C37+C51+C58+C64+C26)-(B12+B19+B37+B51+B58+B64+B26))</f>
         <v/>
       </c>
       <c r="C79" s="17">
         <f>0.5*(C44-B44)</f>
         <v/>
       </c>
-      <c r="D79" s="17">
-        <f>0.5*(C24-B24)</f>
-        <v/>
-      </c>
-      <c r="E79" s="18">
-        <f>B79+C79+D79</f>
+      <c r="D79" s="18">
+        <f>B79+C79</f>
+        <v/>
+      </c>
+      <c r="E79" s="17">
+        <f>0.8*((D12+D19+D37+D51+D58+D64+D26)-(B12+B19+B37+B51+B58+B64+B26))</f>
         <v/>
       </c>
       <c r="F79" s="17">
-        <f>0.8*((D12+D19+D37+D51+D58+D64)-(B12+B19+B37+B51+B58+B64))</f>
-        <v/>
-      </c>
-      <c r="G79" s="17">
         <f>0.5*(D44-B44)</f>
         <v/>
       </c>
-      <c r="H79" s="17">
-        <f>0.5*(D24-B24)</f>
-        <v/>
-      </c>
-      <c r="I79" s="19">
-        <f>F79+G79+H79</f>
+      <c r="G79" s="19">
+        <f>E79+F79</f>
         <v/>
       </c>
     </row>
@@ -2793,35 +2777,27 @@
         </is>
       </c>
       <c r="B80" s="17">
-        <f>0.8*((F12+F19+F37+F51+F58+F64)-(E12+E19+E37+E51+E58+E64))</f>
+        <f>0.8*((F12+F19+F37+F51+F58+F64+F26)-(E12+E19+E37+E51+E58+E64+E26))</f>
         <v/>
       </c>
       <c r="C80" s="17">
         <f>0.5*(F44-E44)</f>
         <v/>
       </c>
-      <c r="D80" s="17">
-        <f>0.5*(F24-E24)</f>
-        <v/>
-      </c>
-      <c r="E80" s="18">
-        <f>B80+C80+D80</f>
+      <c r="D80" s="18">
+        <f>B80+C80</f>
+        <v/>
+      </c>
+      <c r="E80" s="17">
+        <f>0.8*((G12+G19+G37+G51+G58+G64+G26)-(E12+E19+E37+E51+E58+E64+E26))</f>
         <v/>
       </c>
       <c r="F80" s="17">
-        <f>0.8*((G12+G19+G37+G51+G58+G64)-(E12+E19+E37+E51+E58+E64))</f>
-        <v/>
-      </c>
-      <c r="G80" s="17">
         <f>0.5*(G44-E44)</f>
         <v/>
       </c>
-      <c r="H80" s="17">
-        <f>0.5*(G24-E24)</f>
-        <v/>
-      </c>
-      <c r="I80" s="19">
-        <f>F80+G80+H80</f>
+      <c r="G80" s="19">
+        <f>E80+F80</f>
         <v/>
       </c>
     </row>
@@ -2832,42 +2808,34 @@
         </is>
       </c>
       <c r="B81" s="17">
-        <f>0.8*((I12+I19+I37+I51+I58+I64)-(H12+H19+H37+H51+H58+H64))</f>
+        <f>0.8*((I12+I19+I37+I51+I58+I64+I26)-(H12+H19+H37+H51+H58+H64+H26))</f>
         <v/>
       </c>
       <c r="C81" s="17">
         <f>0.5*(I44-H44)</f>
         <v/>
       </c>
-      <c r="D81" s="17">
-        <f>0.5*(I24-H24)</f>
-        <v/>
-      </c>
-      <c r="E81" s="18">
-        <f>B81+C81+D81</f>
+      <c r="D81" s="18">
+        <f>B81+C81</f>
+        <v/>
+      </c>
+      <c r="E81" s="17">
+        <f>0.8*((J12+J19+J37+J51+J58+J64+J26)-(H12+H19+H37+H51+H58+H64+H26))</f>
         <v/>
       </c>
       <c r="F81" s="17">
-        <f>0.8*((J12+J19+J37+J51+J58+J64)-(H12+H19+H37+H51+H58+H64))</f>
-        <v/>
-      </c>
-      <c r="G81" s="17">
         <f>0.5*(J44-H44)</f>
         <v/>
       </c>
-      <c r="H81" s="17">
-        <f>0.5*(J24-H24)</f>
-        <v/>
-      </c>
-      <c r="I81" s="19">
-        <f>F81+G81+H81</f>
+      <c r="G81" s="19">
+        <f>E81+F81</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Conference base/media distribution + institutional support = 100% school (fixed contract, no MC increment; not claimed).</t>
+          <t xml:space="preserve">   Above-baseline pool = commercial + conference/NCAA (units). Institutional subsidy excluded (declining plug, not earned). School collects all revenue and remits the SPV's 80% secondarily — or the rights sit in an LLC.</t>
         </is>
       </c>
     </row>
@@ -2897,14 +2865,14 @@
     <row r="86">
       <c r="A86" s="23" t="inlineStr">
         <is>
-          <t>MECHANIC: the school keeps 100% of its baseline (current column). The INCREASE over baseline is split per bucket: commercial 80/20, donor 50/50, NCAA units 50/50. Conference base/media + institutional support are NOT shared (fixed contracts, no MC-created increment, likely not assignable).</t>
+          <t>MECHANIC: the school keeps 100% of its baseline (current column). The SPV gets 80% of ALL revenue above the baseline (commercial + conference/NCAA), and 50% of the donor uplift. Institutional subsidy is excluded (declining plug, not earned).</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="23" t="inlineStr">
         <is>
-          <t>Commercial = Ticketing, Media, Sponsorship/MMR (incl. MC-originated), Apparel/Licensing, Guarantees, Camps. NCAA units are shared because the MC-manufactured tournament run earns them (pooled/lagged, so modest). Realignment upside on conference money = the separate Promotion SPV.</t>
+          <t>Assignability is not an issue: the school collects every stream directly (conference, MMR, gate, etc.) and remits the SPV's 80% SECONDARILY — or the underlying rights are spun into an LLC. Conference base is in the pool but a flat contract, so it adds ~$0 during the term; the real conference upside is realignment (Promotion SPV).</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3137,7 @@
         </is>
       </c>
       <c r="B13" s="17">
-        <f>'Three-School Projection'!E79</f>
+        <f>'Three-School Projection'!D79</f>
         <v/>
       </c>
       <c r="C13" s="17">
@@ -3191,7 +3159,7 @@
         </is>
       </c>
       <c r="B14" s="17">
-        <f>'Three-School Projection'!E80</f>
+        <f>'Three-School Projection'!D80</f>
         <v/>
       </c>
       <c r="C14" s="17">
@@ -3213,7 +3181,7 @@
         </is>
       </c>
       <c r="B15" s="17">
-        <f>'Three-School Projection'!E81</f>
+        <f>'Three-School Projection'!D81</f>
         <v/>
       </c>
       <c r="C15" s="17">
@@ -3261,7 +3229,7 @@
         </is>
       </c>
       <c r="B18" s="17">
-        <f>'Three-School Projection'!I79</f>
+        <f>'Three-School Projection'!G79</f>
         <v/>
       </c>
       <c r="C18" s="17">
@@ -3283,7 +3251,7 @@
         </is>
       </c>
       <c r="B19" s="17">
-        <f>'Three-School Projection'!I80</f>
+        <f>'Three-School Projection'!G80</f>
         <v/>
       </c>
       <c r="C19" s="17">
@@ -3305,7 +3273,7 @@
         </is>
       </c>
       <c r="B20" s="17">
-        <f>'Three-School Projection'!I81</f>
+        <f>'Three-School Projection'!G81</f>
         <v/>
       </c>
       <c r="C20" s="17">

</xml_diff>

<commit_message>
Fix double-count: hold Learfield MMR guarantee flat; MC-driven MMR uplift lives only in MC-originated line
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J94"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1327,31 +1327,31 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>90</v>
+        <v>300</v>
       </c>
       <c r="C29" s="8" t="n">
-        <v>520</v>
+        <v>300</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>100</v>
+        <v>350</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>580</v>
+        <v>350</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>900</v>
+        <v>350</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>530</v>
+        <v>400</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
     </row>
     <row r="30">
@@ -2907,26 +2907,33 @@
     <row r="92">
       <c r="A92" s="23" t="inlineStr">
         <is>
-          <t>Excluded from this sheet (none are a separate team-revenue stream): third-party athlete NIL income = athletes' own earnings (a recruiting benefit); 'activation' revenue is already inside MMR/sponsorship (in-arena) and Bucket 2 (on-screen); the athlete's NIL cut is a COST; House rev-share pool + booster collective = SPV-funded roster COST (part of the $15M).</t>
+          <t>Learfield MMR guarantee held FLAT (fixed contract mid-term) to avoid double-counting: ALL MC-driven MMR/signage uplift is booked once, in the MC-originated line (85% kept). The 'corporate/category (school)' line is the school's own existing sponsors, distinct from MC-originated national brands.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="23" t="inlineStr">
         <is>
-          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, athlete-marketing/activation, international + format. Roughly recoups the $15M SPV cost.</t>
+          <t>Excluded from this sheet (none are a separate team-revenue stream): third-party athlete NIL income = athletes' own earnings (a recruiting benefit); 'activation' revenue is already inside MMR/sponsorship (in-arena) and Bucket 2 (on-screen); the athlete's NIL cut is a COST; House rev-share pool + booster collective = SPV-funded roster COST (part of the $15M).</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="23" t="inlineStr">
         <is>
+          <t>Bucket 2 (NOT on this sheet, 100% SPV, ~$15M): Netflix series (10 hrs @ $1.0M rev / $0.6M cost), 3 live games (&gt;$1M rev / $0.3M cost each), national presenting sponsor + patch, athlete-marketing/activation, international + format. Roughly recoups the $15M SPV cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="23" t="inlineStr">
+        <is>
           <t>Marquee-game relocation assumed: St. Joe's -&gt; Xfinity Mobile Arena (19k); Davidson -&gt; Spectrum Center (19k); Hawaii carried by its 10,300 arena + Diamond Head Classic. All figures ESTIMATES in $000s.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A85:J85"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="E2:G2"/>
@@ -2937,6 +2944,7 @@
     <mergeCell ref="A92:J92"/>
     <mergeCell ref="A91:J91"/>
     <mergeCell ref="A87:J87"/>
+    <mergeCell ref="A95:J95"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="A86:J86"/>
     <mergeCell ref="A90:J90"/>

</xml_diff>

<commit_message>
Add revenue-vectors doc + Ancillary Vectors tab (#1-4 base/reach) to the model
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
+++ b/cinderella/Outputs/2026-07-15-three-school-revenue-projection.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Three-School Projection" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bucket 2 (SPV)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ancillary Vectors" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;–&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,8 +65,18 @@
       <color rgb="00404040"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +118,11 @@
         <fgColor rgb="00808080"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -125,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -161,6 +177,18 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3334,4 +3362,291 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Vectors (optional) — 'relevance royalty', mostly win-independent   ($000s, per school-season)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Win-indep?</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Book at</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1  Enrollment / tuition-lift fee</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="n">
+        <v>250</v>
+      </c>
+      <c r="C4" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>Parent/MC</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>Flat marketing fee → base; +% of net-tuition lift → reach. Needs provost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2  D2C merch + experiences (net)</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>Partly</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>SPV</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>Own the margin; franchise-branded + player NIL SKUs compound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3  Tourism / econ-dev + film credit</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>750</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Parent/MC</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>Film credit 20-30% of local spend = fastest clean $; + CVB/state integration fee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4  Owned MTE event (net)</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Partly</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>SPV</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>Own gate/title/media; de-risks the live-game line; doubles as content + recruiting hub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>TOTAL ancillary vectors</t>
+        </is>
+      </c>
+      <c r="B8" s="19">
+        <f>SUM(B4:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="19">
+        <f>SUM(C4:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="29" t="n"/>
+      <c r="F8" s="29" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>EFFECT — layered on the existing venture revenue (StJoe reference)</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="31" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Bucket 1 SPV share (from main tab)</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>≈ 9,800</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>≈ 16,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Bucket 2 (100% SPV, from Bucket 2 tab)</t>
+        </is>
+      </c>
+      <c r="B12" s="32" t="inlineStr">
+        <is>
+          <t>≈ 10,300</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>≈ 23,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   + Ancillary vectors (this tab)</t>
+        </is>
+      </c>
+      <c r="B13" s="17">
+        <f>B8</f>
+        <v/>
+      </c>
+      <c r="C13" s="17">
+        <f>C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Ancillary adds ~$2.5M (base) / ~$15M (reach) per school-season — roughly a Bucket-2-sized layer, but mostly win-independent (the hedge).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>These are OPTIONAL upside layers, not in the base SPV economics on the other tabs. Base figures are the reliable floor; reach is the aspirational ceiling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>Booking: merch + MTE sit at the SPV (team-adjacent, split by equity → parent gets its 40%). Enrollment + tourism sit at the parent/MC (institutional deals, MC keeps ~all).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>#5 (university fundraising) and #6 (realignment) intentionally excluded here — messier (gift-optics / political). See the vault doc for their ranges &amp; structures.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>